<commit_message>
Update MLB weather 2026-07-14 01:48 PM PT
</commit_message>
<xml_diff>
--- a/mlb_weather_professional_v4_2026_07_14.xlsx
+++ b/mlb_weather_professional_v4_2026_07_14.xlsx
@@ -230,7 +230,7 @@
     <t>LOW</t>
   </si>
   <si>
-    <t>2026-07-14 01:47:55 PM PDT</t>
+    <t>2026-07-14 01:48:03 PM PDT</t>
   </si>
   <si>
     <t>Period</t>
@@ -473,7 +473,7 @@
     <t>11:00 PM EDT</t>
   </si>
   <si>
-    <t>2026-07-14 20:47:55 UTC</t>
+    <t>2026-07-14 20:48:03 UTC</t>
   </si>
   <si>
     <t>2026-07-14T20:08:45+00:00</t>
@@ -1305,7 +1305,7 @@
         <v>69</v>
       </c>
       <c r="AY2">
-        <v>39.2</v>
+        <v>39.3</v>
       </c>
       <c r="AZ2">
         <v>5</v>
@@ -1693,7 +1693,7 @@
         <v>151</v>
       </c>
       <c r="J2">
-        <v>39.2</v>
+        <v>39.3</v>
       </c>
       <c r="K2">
         <v>3.2</v>
@@ -1735,7 +1735,7 @@
         <v>1</v>
       </c>
       <c r="X2">
-        <v>0.5865</v>
+        <v>0.5867</v>
       </c>
       <c r="Y2">
         <v>-0.02</v>
@@ -1941,7 +1941,7 @@
         <v>151</v>
       </c>
       <c r="J3">
-        <v>39.2</v>
+        <v>39.3</v>
       </c>
       <c r="K3">
         <v>4.2</v>
@@ -1983,7 +1983,7 @@
         <v>1</v>
       </c>
       <c r="X3">
-        <v>0.4965</v>
+        <v>0.4967</v>
       </c>
       <c r="Y3">
         <v>-0.02</v>
@@ -2189,7 +2189,7 @@
         <v>151</v>
       </c>
       <c r="J4">
-        <v>39.2</v>
+        <v>39.3</v>
       </c>
       <c r="K4">
         <v>5.2</v>
@@ -2231,7 +2231,7 @@
         <v>1</v>
       </c>
       <c r="X4">
-        <v>0.4203</v>
+        <v>0.4204</v>
       </c>
       <c r="Y4">
         <v>-0.02</v>
@@ -2437,7 +2437,7 @@
         <v>151</v>
       </c>
       <c r="J5">
-        <v>39.2</v>
+        <v>39.3</v>
       </c>
       <c r="K5">
         <v>6.2</v>
@@ -2479,7 +2479,7 @@
         <v>1</v>
       </c>
       <c r="X5">
-        <v>0.3557</v>
+        <v>0.3559</v>
       </c>
       <c r="Y5">
         <v>-0.01</v>

</xml_diff>

<commit_message>
Update MLB weather 2026-07-14 02:15 PM PT
</commit_message>
<xml_diff>
--- a/mlb_weather_professional_v4_2026_07_14.xlsx
+++ b/mlb_weather_professional_v4_2026_07_14.xlsx
@@ -230,7 +230,7 @@
     <t>LOW</t>
   </si>
   <si>
-    <t>2026-07-14 01:48:28 PM PDT</t>
+    <t>2026-07-14 02:15:43 PM PDT</t>
   </si>
   <si>
     <t>Period</t>
@@ -473,7 +473,7 @@
     <t>11:00 PM EDT</t>
   </si>
   <si>
-    <t>2026-07-14 20:48:28 UTC</t>
+    <t>2026-07-14 21:15:43 UTC</t>
   </si>
   <si>
     <t>2026-07-14T20:08:45+00:00</t>
@@ -1206,7 +1206,7 @@
         <v>7.5</v>
       </c>
       <c r="R2">
-        <v>8.699999999999999</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="S2">
         <v>0</v>
@@ -1227,10 +1227,10 @@
         <v>6</v>
       </c>
       <c r="Y2">
-        <v>3.7</v>
+        <v>3.8</v>
       </c>
       <c r="Z2">
-        <v>91.09999999999999</v>
+        <v>91.2</v>
       </c>
       <c r="AA2" t="s">
         <v>66</v>
@@ -1275,13 +1275,13 @@
         <v>67</v>
       </c>
       <c r="AO2">
-        <v>17.9</v>
+        <v>18</v>
       </c>
       <c r="AP2">
-        <v>-0.02</v>
+        <v>0.1</v>
       </c>
       <c r="AQ2">
-        <v>-0.13</v>
+        <v>0.21</v>
       </c>
       <c r="AR2">
         <v>0</v>
@@ -1299,13 +1299,13 @@
         <v>68</v>
       </c>
       <c r="AW2">
-        <v>11.4</v>
+        <v>11.3</v>
       </c>
       <c r="AX2" t="s">
         <v>69</v>
       </c>
       <c r="AY2">
-        <v>39.7</v>
+        <v>67</v>
       </c>
       <c r="AZ2">
         <v>5</v>
@@ -1693,19 +1693,19 @@
         <v>151</v>
       </c>
       <c r="J2">
-        <v>39.7</v>
+        <v>67</v>
       </c>
       <c r="K2">
-        <v>3.2</v>
+        <v>2.7</v>
       </c>
       <c r="L2">
         <v>5</v>
       </c>
       <c r="M2">
-        <v>0.87</v>
+        <v>0.89</v>
       </c>
       <c r="N2">
-        <v>0.61</v>
+        <v>0.65</v>
       </c>
       <c r="O2">
         <v>0</v>
@@ -1714,7 +1714,7 @@
         <v>0.8</v>
       </c>
       <c r="Q2">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
       <c r="R2">
         <v>100</v>
@@ -1735,16 +1735,16 @@
         <v>1</v>
       </c>
       <c r="X2">
-        <v>0.5874</v>
+        <v>0.6336000000000001</v>
       </c>
       <c r="Y2">
-        <v>-0.02</v>
+        <v>0.1</v>
       </c>
       <c r="Z2">
-        <v>-0.13</v>
+        <v>0.21</v>
       </c>
       <c r="AA2">
-        <v>5.3</v>
+        <v>5.5</v>
       </c>
       <c r="AB2">
         <v>92</v>
@@ -1804,7 +1804,7 @@
         <v>9.4</v>
       </c>
       <c r="AU2">
-        <v>20.7</v>
+        <v>20.8</v>
       </c>
       <c r="AV2" t="s">
         <v>63</v>
@@ -1828,10 +1828,10 @@
         <v>2.9</v>
       </c>
       <c r="BC2">
-        <v>8.699999999999999</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="BD2">
-        <v>5.2</v>
+        <v>5.3</v>
       </c>
       <c r="BE2">
         <v>6.8</v>
@@ -1858,7 +1858,7 @@
         <v>158</v>
       </c>
       <c r="BM2">
-        <v>2026</v>
+        <v>2027</v>
       </c>
       <c r="BN2" t="s">
         <v>59</v>
@@ -1873,7 +1873,7 @@
         <v>1.086</v>
       </c>
       <c r="BR2">
-        <v>87.59999999999999</v>
+        <v>87.7</v>
       </c>
       <c r="BS2">
         <v>82.40000000000001</v>
@@ -1894,7 +1894,7 @@
         <v>68</v>
       </c>
       <c r="BY2">
-        <v>10.2</v>
+        <v>10</v>
       </c>
       <c r="BZ2" t="s">
         <v>68</v>
@@ -1903,13 +1903,13 @@
         <v>91</v>
       </c>
       <c r="CB2">
-        <v>86.8</v>
+        <v>86.90000000000001</v>
       </c>
       <c r="CC2">
         <v>10</v>
       </c>
       <c r="CD2">
-        <v>9.199999999999999</v>
+        <v>9.300000000000001</v>
       </c>
     </row>
     <row r="3" spans="1:82">
@@ -1941,16 +1941,16 @@
         <v>151</v>
       </c>
       <c r="J3">
-        <v>39.7</v>
+        <v>67</v>
       </c>
       <c r="K3">
-        <v>4.2</v>
+        <v>3.7</v>
       </c>
       <c r="L3">
         <v>5</v>
       </c>
       <c r="M3">
-        <v>0.71</v>
+        <v>0.68</v>
       </c>
       <c r="N3">
         <v>1.06</v>
@@ -1983,22 +1983,22 @@
         <v>1</v>
       </c>
       <c r="X3">
-        <v>0.4972</v>
+        <v>0.5364</v>
       </c>
       <c r="Y3">
-        <v>-0.02</v>
+        <v>0.08</v>
       </c>
       <c r="Z3">
-        <v>-0.11</v>
+        <v>0.18</v>
       </c>
       <c r="AA3">
-        <v>6</v>
+        <v>5.9</v>
       </c>
       <c r="AB3">
-        <v>91.5</v>
+        <v>91.7</v>
       </c>
       <c r="AC3">
-        <v>79.7</v>
+        <v>79.8</v>
       </c>
       <c r="AD3">
         <v>0.98</v>
@@ -2079,7 +2079,7 @@
         <v>8.4</v>
       </c>
       <c r="BD3">
-        <v>5</v>
+        <v>5.1</v>
       </c>
       <c r="BE3">
         <v>6.5</v>
@@ -2124,7 +2124,7 @@
         <v>84.2</v>
       </c>
       <c r="BS3">
-        <v>79.09999999999999</v>
+        <v>79.2</v>
       </c>
       <c r="BT3">
         <v>59.7</v>
@@ -2142,7 +2142,7 @@
         <v>68</v>
       </c>
       <c r="BY3">
-        <v>10.5</v>
+        <v>10.3</v>
       </c>
       <c r="BZ3" t="s">
         <v>68</v>
@@ -2157,7 +2157,7 @@
         <v>10</v>
       </c>
       <c r="CD3">
-        <v>8.5</v>
+        <v>8.6</v>
       </c>
     </row>
     <row r="4" spans="1:82">
@@ -2189,19 +2189,19 @@
         <v>151</v>
       </c>
       <c r="J4">
-        <v>39.7</v>
+        <v>67</v>
       </c>
       <c r="K4">
-        <v>5.2</v>
+        <v>4.7</v>
       </c>
       <c r="L4">
         <v>5</v>
       </c>
       <c r="M4">
-        <v>1.33</v>
+        <v>1.31</v>
       </c>
       <c r="N4">
-        <v>1.18</v>
+        <v>1.16</v>
       </c>
       <c r="O4">
         <v>0</v>
@@ -2231,22 +2231,22 @@
         <v>1</v>
       </c>
       <c r="X4">
-        <v>0.4209</v>
+        <v>0.454</v>
       </c>
       <c r="Y4">
-        <v>-0.02</v>
+        <v>0.07000000000000001</v>
       </c>
       <c r="Z4">
-        <v>-0.1</v>
+        <v>0.15</v>
       </c>
       <c r="AA4">
-        <v>8.9</v>
+        <v>8.699999999999999</v>
       </c>
       <c r="AB4">
-        <v>89.7</v>
+        <v>89.90000000000001</v>
       </c>
       <c r="AC4">
-        <v>78.2</v>
+        <v>78.3</v>
       </c>
       <c r="AD4">
         <v>0.98</v>
@@ -2348,13 +2348,13 @@
         <v>0.09</v>
       </c>
       <c r="BK4">
-        <v>1.1589</v>
+        <v>1.1588</v>
       </c>
       <c r="BL4" t="s">
         <v>158</v>
       </c>
       <c r="BM4">
-        <v>1631</v>
+        <v>1632</v>
       </c>
       <c r="BN4" t="s">
         <v>59</v>
@@ -2369,7 +2369,7 @@
         <v>1.075</v>
       </c>
       <c r="BR4">
-        <v>83.09999999999999</v>
+        <v>83.2</v>
       </c>
       <c r="BS4">
         <v>78</v>
@@ -2381,7 +2381,7 @@
         <v>57.4</v>
       </c>
       <c r="BV4">
-        <v>54.9</v>
+        <v>54.8</v>
       </c>
       <c r="BW4">
         <v>8.9</v>
@@ -2390,7 +2390,7 @@
         <v>68</v>
       </c>
       <c r="BY4">
-        <v>11.4</v>
+        <v>11.3</v>
       </c>
       <c r="BZ4" t="s">
         <v>68</v>
@@ -2437,19 +2437,19 @@
         <v>151</v>
       </c>
       <c r="J5">
-        <v>39.7</v>
+        <v>67</v>
       </c>
       <c r="K5">
-        <v>6.2</v>
+        <v>5.7</v>
       </c>
       <c r="L5">
         <v>5</v>
       </c>
       <c r="M5">
-        <v>1.83</v>
+        <v>1.81</v>
       </c>
       <c r="N5">
-        <v>1.31</v>
+        <v>1.29</v>
       </c>
       <c r="O5">
         <v>0</v>
@@ -2479,22 +2479,22 @@
         <v>1</v>
       </c>
       <c r="X5">
-        <v>0.3563</v>
+        <v>0.3843</v>
       </c>
       <c r="Y5">
-        <v>-0.01</v>
+        <v>0.06</v>
       </c>
       <c r="Z5">
-        <v>-0.08</v>
+        <v>0.13</v>
       </c>
       <c r="AA5">
-        <v>11.3</v>
+        <v>11.1</v>
       </c>
       <c r="AB5">
-        <v>89.40000000000001</v>
+        <v>89.5</v>
       </c>
       <c r="AC5">
-        <v>76.40000000000001</v>
+        <v>76.5</v>
       </c>
       <c r="AD5">
         <v>0.98</v>
@@ -2512,7 +2512,7 @@
         <v>61</v>
       </c>
       <c r="AI5">
-        <v>80.8</v>
+        <v>80.90000000000001</v>
       </c>
       <c r="AJ5">
         <v>81.59999999999999</v>
@@ -2521,7 +2521,7 @@
         <v>68.3</v>
       </c>
       <c r="AL5">
-        <v>67</v>
+        <v>66.90000000000001</v>
       </c>
       <c r="AM5">
         <v>1012</v>
@@ -2548,7 +2548,7 @@
         <v>8.9</v>
       </c>
       <c r="AU5">
-        <v>17.1</v>
+        <v>17.2</v>
       </c>
       <c r="AV5" t="s">
         <v>63</v>
@@ -2620,7 +2620,7 @@
         <v>81.3</v>
       </c>
       <c r="BS5">
-        <v>76.2</v>
+        <v>76.3</v>
       </c>
       <c r="BT5">
         <v>58.7</v>
@@ -2629,7 +2629,7 @@
         <v>56.8</v>
       </c>
       <c r="BV5">
-        <v>58.4</v>
+        <v>58.3</v>
       </c>
       <c r="BW5">
         <v>7.9</v>
@@ -2638,7 +2638,7 @@
         <v>68</v>
       </c>
       <c r="BY5">
-        <v>10.1</v>
+        <v>10</v>
       </c>
       <c r="BZ5" t="s">
         <v>68</v>
@@ -2760,7 +2760,7 @@
         <v>64</v>
       </c>
       <c r="G2">
-        <v>91.09999999999999</v>
+        <v>91.2</v>
       </c>
       <c r="H2">
         <v>8</v>
@@ -2769,7 +2769,7 @@
         <v>6</v>
       </c>
       <c r="J2">
-        <v>3.7</v>
+        <v>3.8</v>
       </c>
       <c r="K2">
         <v>5</v>

</xml_diff>

<commit_message>
Update MLB weather 2026-07-14 02:25 PM PT
</commit_message>
<xml_diff>
--- a/mlb_weather_professional_v4_2026_07_14.xlsx
+++ b/mlb_weather_professional_v4_2026_07_14.xlsx
@@ -209,7 +209,7 @@
     <t>Clear</t>
   </si>
   <si>
-    <t>9.4 mph from SW</t>
+    <t>🟢 8.8 mph Out to RF</t>
   </si>
   <si>
     <t>SW</t>
@@ -224,13 +224,13 @@
     <t>🟢 Good</t>
   </si>
   <si>
-    <t>STEADY</t>
+    <t>IMPROVING RAPIDLY</t>
   </si>
   <si>
     <t>LOW</t>
   </si>
   <si>
-    <t>2026-07-14 02:16:23 PM PDT</t>
+    <t>2026-07-14 02:25:42 PM PDT</t>
   </si>
   <si>
     <t>Period</t>
@@ -473,7 +473,7 @@
     <t>11:00 PM EDT</t>
   </si>
   <si>
-    <t>2026-07-14 21:16:23 UTC</t>
+    <t>2026-07-14 21:25:42 UTC</t>
   </si>
   <si>
     <t>2026-07-14T20:08:45+00:00</t>
@@ -960,7 +960,7 @@
     <col min="10" max="10" width="20.7109375" customWidth="1"/>
     <col min="11" max="11" width="27.7109375" customWidth="1"/>
     <col min="12" max="12" width="33.7109375" customWidth="1"/>
-    <col min="13" max="13" width="18.7109375" customWidth="1"/>
+    <col min="13" max="13" width="21.7109375" customWidth="1"/>
     <col min="14" max="15" width="28.7109375" customWidth="1"/>
     <col min="16" max="18" width="32.7109375" customWidth="1"/>
     <col min="19" max="19" width="29.7109375" customWidth="1"/>
@@ -982,7 +982,7 @@
     <col min="37" max="37" width="22.7109375" customWidth="1"/>
     <col min="38" max="38" width="17.7109375" customWidth="1"/>
     <col min="39" max="39" width="15.7109375" customWidth="1"/>
-    <col min="40" max="40" width="16.7109375" customWidth="1"/>
+    <col min="40" max="40" width="19.7109375" customWidth="1"/>
     <col min="41" max="41" width="34.7109375" customWidth="1"/>
     <col min="42" max="42" width="21.7109375" customWidth="1"/>
     <col min="43" max="43" width="23.7109375" customWidth="1"/>
@@ -1257,7 +1257,7 @@
         <v>1.1528</v>
       </c>
       <c r="AI2">
-        <v>1822</v>
+        <v>1823</v>
       </c>
       <c r="AJ2">
         <v>1012.3</v>
@@ -1275,13 +1275,13 @@
         <v>67</v>
       </c>
       <c r="AO2">
-        <v>0</v>
+        <v>18</v>
       </c>
       <c r="AP2">
-        <v>0.1</v>
+        <v>0.17</v>
       </c>
       <c r="AQ2">
-        <v>0.21</v>
+        <v>0.27</v>
       </c>
       <c r="AR2">
         <v>0</v>
@@ -1305,7 +1305,7 @@
         <v>69</v>
       </c>
       <c r="AY2">
-        <v>67.59999999999999</v>
+        <v>77</v>
       </c>
       <c r="AZ2">
         <v>5</v>
@@ -1693,10 +1693,10 @@
         <v>151</v>
       </c>
       <c r="J2">
-        <v>67.59999999999999</v>
+        <v>77</v>
       </c>
       <c r="K2">
-        <v>2.7</v>
+        <v>2.6</v>
       </c>
       <c r="L2">
         <v>5</v>
@@ -1705,7 +1705,7 @@
         <v>0.89</v>
       </c>
       <c r="N2">
-        <v>0.65</v>
+        <v>0.66</v>
       </c>
       <c r="O2">
         <v>0</v>
@@ -1735,13 +1735,13 @@
         <v>1</v>
       </c>
       <c r="X2">
-        <v>0.6348</v>
+        <v>0.6514</v>
       </c>
       <c r="Y2">
-        <v>0.1</v>
+        <v>0.17</v>
       </c>
       <c r="Z2">
-        <v>0.21</v>
+        <v>0.27</v>
       </c>
       <c r="AA2">
         <v>5.5</v>
@@ -1750,7 +1750,7 @@
         <v>92</v>
       </c>
       <c r="AC2">
-        <v>83</v>
+        <v>83.09999999999999</v>
       </c>
       <c r="AD2">
         <v>0.98</v>
@@ -1774,7 +1774,7 @@
         <v>90.09999999999999</v>
       </c>
       <c r="AK2">
-        <v>68.59999999999999</v>
+        <v>68.5</v>
       </c>
       <c r="AL2">
         <v>52.1</v>
@@ -1941,16 +1941,16 @@
         <v>151</v>
       </c>
       <c r="J3">
-        <v>67.59999999999999</v>
+        <v>77</v>
       </c>
       <c r="K3">
-        <v>3.7</v>
+        <v>3.6</v>
       </c>
       <c r="L3">
         <v>5</v>
       </c>
       <c r="M3">
-        <v>0.68</v>
+        <v>0.67</v>
       </c>
       <c r="N3">
         <v>1.06</v>
@@ -1983,13 +1983,13 @@
         <v>1</v>
       </c>
       <c r="X3">
-        <v>0.5373</v>
+        <v>0.5514</v>
       </c>
       <c r="Y3">
-        <v>0.09</v>
+        <v>0.14</v>
       </c>
       <c r="Z3">
-        <v>0.18</v>
+        <v>0.23</v>
       </c>
       <c r="AA3">
         <v>5.9</v>
@@ -2106,7 +2106,7 @@
         <v>158</v>
       </c>
       <c r="BM3">
-        <v>1789</v>
+        <v>1790</v>
       </c>
       <c r="BN3" t="s">
         <v>59</v>
@@ -2189,16 +2189,16 @@
         <v>151</v>
       </c>
       <c r="J4">
-        <v>67.59999999999999</v>
+        <v>77</v>
       </c>
       <c r="K4">
-        <v>4.7</v>
+        <v>4.6</v>
       </c>
       <c r="L4">
         <v>5</v>
       </c>
       <c r="M4">
-        <v>1.31</v>
+        <v>1.3</v>
       </c>
       <c r="N4">
         <v>1.16</v>
@@ -2231,13 +2231,13 @@
         <v>1</v>
       </c>
       <c r="X4">
-        <v>0.4548</v>
+        <v>0.4668</v>
       </c>
       <c r="Y4">
-        <v>0.07000000000000001</v>
+        <v>0.12</v>
       </c>
       <c r="Z4">
-        <v>0.15</v>
+        <v>0.19</v>
       </c>
       <c r="AA4">
         <v>8.699999999999999</v>
@@ -2437,19 +2437,19 @@
         <v>151</v>
       </c>
       <c r="J5">
-        <v>67.59999999999999</v>
+        <v>77</v>
       </c>
       <c r="K5">
-        <v>5.7</v>
+        <v>5.6</v>
       </c>
       <c r="L5">
         <v>5</v>
       </c>
       <c r="M5">
-        <v>1.81</v>
+        <v>1.8</v>
       </c>
       <c r="N5">
-        <v>1.29</v>
+        <v>1.28</v>
       </c>
       <c r="O5">
         <v>0</v>
@@ -2479,13 +2479,13 @@
         <v>1</v>
       </c>
       <c r="X5">
-        <v>0.385</v>
+        <v>0.3951</v>
       </c>
       <c r="Y5">
-        <v>0.06</v>
+        <v>0.1</v>
       </c>
       <c r="Z5">
-        <v>0.13</v>
+        <v>0.16</v>
       </c>
       <c r="AA5">
         <v>11.1</v>
@@ -2545,7 +2545,7 @@
         <v>793</v>
       </c>
       <c r="AT5">
-        <v>8.9</v>
+        <v>9</v>
       </c>
       <c r="AU5">
         <v>17.2</v>
@@ -2563,7 +2563,7 @@
         <v>3.1</v>
       </c>
       <c r="AZ5">
-        <v>8.9</v>
+        <v>9</v>
       </c>
       <c r="BA5">
         <v>7.2</v>
@@ -2781,7 +2781,7 @@
         <v>86.09999999999999</v>
       </c>
       <c r="N2">
-        <v>1822</v>
+        <v>1823</v>
       </c>
       <c r="O2" t="s">
         <v>59</v>

</xml_diff>

<commit_message>
Update MLB weather 2026-07-14 02:28 PM PT
</commit_message>
<xml_diff>
--- a/mlb_weather_professional_v4_2026_07_14.xlsx
+++ b/mlb_weather_professional_v4_2026_07_14.xlsx
@@ -230,7 +230,7 @@
     <t>LOW</t>
   </si>
   <si>
-    <t>2026-07-14 02:25:42 PM PDT</t>
+    <t>2026-07-14 02:28:02 PM PDT</t>
   </si>
   <si>
     <t>Period</t>
@@ -473,7 +473,7 @@
     <t>11:00 PM EDT</t>
   </si>
   <si>
-    <t>2026-07-14 21:25:42 UTC</t>
+    <t>2026-07-14 21:28:02 UTC</t>
   </si>
   <si>
     <t>2026-07-14T20:08:45+00:00</t>
@@ -1212,7 +1212,7 @@
         <v>0</v>
       </c>
       <c r="T2">
-        <v>62.5</v>
+        <v>62.6</v>
       </c>
       <c r="U2" t="s">
         <v>64</v>
@@ -1254,7 +1254,7 @@
         <v>0.4</v>
       </c>
       <c r="AH2">
-        <v>1.1528</v>
+        <v>1.1527</v>
       </c>
       <c r="AI2">
         <v>1823</v>
@@ -1278,10 +1278,10 @@
         <v>18</v>
       </c>
       <c r="AP2">
-        <v>0.17</v>
+        <v>0.18</v>
       </c>
       <c r="AQ2">
-        <v>0.27</v>
+        <v>0.28</v>
       </c>
       <c r="AR2">
         <v>0</v>
@@ -1305,7 +1305,7 @@
         <v>69</v>
       </c>
       <c r="AY2">
-        <v>77</v>
+        <v>79.3</v>
       </c>
       <c r="AZ2">
         <v>5</v>
@@ -1693,16 +1693,16 @@
         <v>151</v>
       </c>
       <c r="J2">
-        <v>77</v>
+        <v>79.3</v>
       </c>
       <c r="K2">
-        <v>2.6</v>
+        <v>2.5</v>
       </c>
       <c r="L2">
         <v>5</v>
       </c>
       <c r="M2">
-        <v>0.89</v>
+        <v>0.9</v>
       </c>
       <c r="N2">
         <v>0.66</v>
@@ -1735,16 +1735,16 @@
         <v>1</v>
       </c>
       <c r="X2">
-        <v>0.6514</v>
+        <v>0.6556999999999999</v>
       </c>
       <c r="Y2">
-        <v>0.17</v>
+        <v>0.18</v>
       </c>
       <c r="Z2">
-        <v>0.27</v>
+        <v>0.28</v>
       </c>
       <c r="AA2">
-        <v>5.5</v>
+        <v>5.6</v>
       </c>
       <c r="AB2">
         <v>92</v>
@@ -1894,7 +1894,7 @@
         <v>68</v>
       </c>
       <c r="BY2">
-        <v>10</v>
+        <v>9.9</v>
       </c>
       <c r="BZ2" t="s">
         <v>68</v>
@@ -1941,10 +1941,10 @@
         <v>151</v>
       </c>
       <c r="J3">
-        <v>77</v>
+        <v>79.3</v>
       </c>
       <c r="K3">
-        <v>3.6</v>
+        <v>3.5</v>
       </c>
       <c r="L3">
         <v>5</v>
@@ -1983,13 +1983,13 @@
         <v>1</v>
       </c>
       <c r="X3">
-        <v>0.5514</v>
+        <v>0.555</v>
       </c>
       <c r="Y3">
-        <v>0.14</v>
+        <v>0.16</v>
       </c>
       <c r="Z3">
-        <v>0.23</v>
+        <v>0.24</v>
       </c>
       <c r="AA3">
         <v>5.9</v>
@@ -2100,7 +2100,7 @@
         <v>0.09</v>
       </c>
       <c r="BK3">
-        <v>1.1538</v>
+        <v>1.1537</v>
       </c>
       <c r="BL3" t="s">
         <v>158</v>
@@ -2189,16 +2189,16 @@
         <v>151</v>
       </c>
       <c r="J4">
-        <v>77</v>
+        <v>79.3</v>
       </c>
       <c r="K4">
-        <v>4.6</v>
+        <v>4.5</v>
       </c>
       <c r="L4">
         <v>5</v>
       </c>
       <c r="M4">
-        <v>1.3</v>
+        <v>1.29</v>
       </c>
       <c r="N4">
         <v>1.16</v>
@@ -2231,13 +2231,13 @@
         <v>1</v>
       </c>
       <c r="X4">
-        <v>0.4668</v>
+        <v>0.4698</v>
       </c>
       <c r="Y4">
-        <v>0.12</v>
+        <v>0.13</v>
       </c>
       <c r="Z4">
-        <v>0.19</v>
+        <v>0.2</v>
       </c>
       <c r="AA4">
         <v>8.699999999999999</v>
@@ -2437,10 +2437,10 @@
         <v>151</v>
       </c>
       <c r="J5">
-        <v>77</v>
+        <v>79.3</v>
       </c>
       <c r="K5">
-        <v>5.6</v>
+        <v>5.5</v>
       </c>
       <c r="L5">
         <v>5</v>
@@ -2479,13 +2479,13 @@
         <v>1</v>
       </c>
       <c r="X5">
-        <v>0.3951</v>
+        <v>0.3977</v>
       </c>
       <c r="Y5">
-        <v>0.1</v>
+        <v>0.11</v>
       </c>
       <c r="Z5">
-        <v>0.16</v>
+        <v>0.17</v>
       </c>
       <c r="AA5">
         <v>11.1</v>
@@ -2754,7 +2754,7 @@
         <v>58</v>
       </c>
       <c r="E2">
-        <v>62.5</v>
+        <v>62.6</v>
       </c>
       <c r="F2" t="s">
         <v>64</v>

</xml_diff>

<commit_message>
Update MLB weather 2026-07-14 02:51 PM PT
</commit_message>
<xml_diff>
--- a/mlb_weather_professional_v4_2026_07_14.xlsx
+++ b/mlb_weather_professional_v4_2026_07_14.xlsx
@@ -230,7 +230,7 @@
     <t>LOW</t>
   </si>
   <si>
-    <t>2026-07-14 02:34:37 PM PDT</t>
+    <t>2026-07-14 02:51:42 PM PDT</t>
   </si>
   <si>
     <t>Period</t>
@@ -473,10 +473,10 @@
     <t>11:00 PM EDT</t>
   </si>
   <si>
-    <t>2026-07-14 21:34:37 UTC</t>
-  </si>
-  <si>
-    <t>2026-07-14T20:08:45+00:00</t>
+    <t>2026-07-14 21:51:42 UTC</t>
+  </si>
+  <si>
+    <t>2026-07-14T20:53:25+00:00</t>
   </si>
   <si>
     <t>YES</t>
@@ -1188,7 +1188,7 @@
         <v>88.5</v>
       </c>
       <c r="L2">
-        <v>52.8</v>
+        <v>54.7</v>
       </c>
       <c r="M2" t="s">
         <v>62</v>
@@ -1212,7 +1212,7 @@
         <v>0</v>
       </c>
       <c r="T2">
-        <v>62.1</v>
+        <v>62.3</v>
       </c>
       <c r="U2" t="s">
         <v>64</v>
@@ -1227,7 +1227,7 @@
         <v>6</v>
       </c>
       <c r="Y2">
-        <v>3.6</v>
+        <v>3.7</v>
       </c>
       <c r="Z2">
         <v>89.59999999999999</v>
@@ -1248,40 +1248,40 @@
         <v>0</v>
       </c>
       <c r="AF2">
-        <v>4.2</v>
+        <v>4.6</v>
       </c>
       <c r="AG2">
-        <v>0.4</v>
+        <v>0.5</v>
       </c>
       <c r="AH2">
-        <v>1.1546</v>
+        <v>1.1538</v>
       </c>
       <c r="AI2">
-        <v>1771</v>
+        <v>1782</v>
       </c>
       <c r="AJ2">
-        <v>1012.4</v>
+        <v>1012.1</v>
       </c>
       <c r="AK2">
-        <v>68</v>
+        <v>69.2</v>
       </c>
       <c r="AL2">
         <v>85.40000000000001</v>
       </c>
       <c r="AM2">
-        <v>58.2</v>
+        <v>60.3</v>
       </c>
       <c r="AN2" t="s">
         <v>67</v>
       </c>
       <c r="AO2">
-        <v>16.6</v>
+        <v>17.3</v>
       </c>
       <c r="AP2">
-        <v>0.1</v>
+        <v>0.01</v>
       </c>
       <c r="AQ2">
-        <v>0.11</v>
+        <v>0.18</v>
       </c>
       <c r="AR2">
         <v>0</v>
@@ -1293,7 +1293,7 @@
         <v>68</v>
       </c>
       <c r="AU2">
-        <v>10.3</v>
+        <v>11.8</v>
       </c>
       <c r="AV2" t="s">
         <v>68</v>
@@ -1305,7 +1305,7 @@
         <v>69</v>
       </c>
       <c r="AY2">
-        <v>85.90000000000001</v>
+        <v>58.3</v>
       </c>
       <c r="AZ2">
         <v>5</v>
@@ -1693,25 +1693,25 @@
         <v>151</v>
       </c>
       <c r="J2">
-        <v>85.90000000000001</v>
+        <v>58.3</v>
       </c>
       <c r="K2">
-        <v>2.4</v>
+        <v>2.1</v>
       </c>
       <c r="L2">
         <v>5</v>
       </c>
       <c r="M2">
-        <v>0.13</v>
+        <v>0.1</v>
       </c>
       <c r="N2">
-        <v>0.57</v>
+        <v>0.54</v>
       </c>
       <c r="O2">
         <v>0</v>
       </c>
       <c r="P2">
-        <v>0.9</v>
+        <v>1.2</v>
       </c>
       <c r="Q2">
         <v>0.3</v>
@@ -1735,22 +1735,22 @@
         <v>1</v>
       </c>
       <c r="X2">
-        <v>0.6677999999999999</v>
+        <v>0.7002</v>
       </c>
       <c r="Y2">
-        <v>0.1</v>
+        <v>0.01</v>
       </c>
       <c r="Z2">
-        <v>0.11</v>
+        <v>0.18</v>
       </c>
       <c r="AA2">
-        <v>2.2</v>
+        <v>2</v>
       </c>
       <c r="AB2">
-        <v>91.59999999999999</v>
+        <v>91.7</v>
       </c>
       <c r="AC2">
-        <v>82</v>
+        <v>82.2</v>
       </c>
       <c r="AD2">
         <v>0.98</v>
@@ -1771,19 +1771,19 @@
         <v>88.5</v>
       </c>
       <c r="AJ2">
-        <v>88.2</v>
+        <v>89.8</v>
       </c>
       <c r="AK2">
-        <v>68.09999999999999</v>
+        <v>69.3</v>
       </c>
       <c r="AL2">
-        <v>52.8</v>
+        <v>54.7</v>
       </c>
       <c r="AM2">
-        <v>1012.5</v>
+        <v>1012.1</v>
       </c>
       <c r="AN2">
-        <v>1014.8</v>
+        <v>1014.3</v>
       </c>
       <c r="AO2">
         <v>0</v>
@@ -1798,13 +1798,13 @@
         <v>63</v>
       </c>
       <c r="AS2">
-        <v>1026</v>
+        <v>1178</v>
       </c>
       <c r="AT2">
         <v>9.199999999999999</v>
       </c>
       <c r="AU2">
-        <v>20.3</v>
+        <v>20.4</v>
       </c>
       <c r="AV2" t="s">
         <v>63</v>
@@ -1852,13 +1852,13 @@
         <v>0.09</v>
       </c>
       <c r="BK2">
-        <v>1.148</v>
+        <v>1.1471</v>
       </c>
       <c r="BL2" t="s">
         <v>158</v>
       </c>
       <c r="BM2">
-        <v>1974</v>
+        <v>1989</v>
       </c>
       <c r="BN2" t="s">
         <v>59</v>
@@ -1867,28 +1867,28 @@
         <v>60</v>
       </c>
       <c r="BP2">
-        <v>85</v>
+        <v>85.2</v>
       </c>
       <c r="BQ2">
         <v>1.084</v>
       </c>
       <c r="BR2">
-        <v>86.7</v>
+        <v>86.90000000000001</v>
       </c>
       <c r="BS2">
-        <v>81.59999999999999</v>
+        <v>81.7</v>
       </c>
       <c r="BT2">
         <v>60.4</v>
       </c>
       <c r="BU2">
-        <v>58.5</v>
+        <v>58.7</v>
       </c>
       <c r="BV2">
-        <v>47.5</v>
+        <v>46.4</v>
       </c>
       <c r="BW2">
-        <v>10.3</v>
+        <v>11.8</v>
       </c>
       <c r="BX2" t="s">
         <v>68</v>
@@ -1941,28 +1941,28 @@
         <v>151</v>
       </c>
       <c r="J3">
-        <v>85.90000000000001</v>
+        <v>58.3</v>
       </c>
       <c r="K3">
-        <v>3.4</v>
+        <v>3.1</v>
       </c>
       <c r="L3">
         <v>5</v>
       </c>
       <c r="M3">
-        <v>1.22</v>
+        <v>1.24</v>
       </c>
       <c r="N3">
-        <v>1.13</v>
+        <v>1.12</v>
       </c>
       <c r="O3">
         <v>0</v>
       </c>
       <c r="P3">
-        <v>5.4</v>
+        <v>6.1</v>
       </c>
       <c r="Q3">
-        <v>0.5</v>
+        <v>0.6</v>
       </c>
       <c r="R3">
         <v>100</v>
@@ -1983,22 +1983,22 @@
         <v>1</v>
       </c>
       <c r="X3">
-        <v>0.5653</v>
+        <v>0.5927</v>
       </c>
       <c r="Y3">
-        <v>0.08</v>
+        <v>0.01</v>
       </c>
       <c r="Z3">
-        <v>0.1</v>
+        <v>0.15</v>
       </c>
       <c r="AA3">
         <v>8.300000000000001</v>
       </c>
       <c r="AB3">
-        <v>88.5</v>
+        <v>88.40000000000001</v>
       </c>
       <c r="AC3">
-        <v>77.90000000000001</v>
+        <v>78.09999999999999</v>
       </c>
       <c r="AD3">
         <v>0.98</v>
@@ -2019,19 +2019,19 @@
         <v>84.7</v>
       </c>
       <c r="AJ3">
-        <v>83.8</v>
+        <v>85.8</v>
       </c>
       <c r="AK3">
-        <v>67.8</v>
+        <v>69.3</v>
       </c>
       <c r="AL3">
-        <v>58.9</v>
+        <v>61.4</v>
       </c>
       <c r="AM3">
-        <v>1012.3</v>
+        <v>1011.8</v>
       </c>
       <c r="AN3">
-        <v>1014.6</v>
+        <v>1014.1</v>
       </c>
       <c r="AO3">
         <v>0</v>
@@ -2046,13 +2046,13 @@
         <v>47.5</v>
       </c>
       <c r="AS3">
-        <v>917</v>
+        <v>1164</v>
       </c>
       <c r="AT3">
         <v>8.800000000000001</v>
       </c>
       <c r="AU3">
-        <v>17.3</v>
+        <v>17.4</v>
       </c>
       <c r="AV3" t="s">
         <v>63</v>
@@ -2100,13 +2100,13 @@
         <v>0.09</v>
       </c>
       <c r="BK3">
-        <v>1.156</v>
+        <v>1.1549</v>
       </c>
       <c r="BL3" t="s">
         <v>158</v>
       </c>
       <c r="BM3">
-        <v>1729</v>
+        <v>1745</v>
       </c>
       <c r="BN3" t="s">
         <v>59</v>
@@ -2115,28 +2115,28 @@
         <v>60</v>
       </c>
       <c r="BP3">
-        <v>81.5</v>
+        <v>81.7</v>
       </c>
       <c r="BQ3">
         <v>1.076</v>
       </c>
       <c r="BR3">
-        <v>83.2</v>
+        <v>83.40000000000001</v>
       </c>
       <c r="BS3">
-        <v>78.2</v>
+        <v>78.5</v>
       </c>
       <c r="BT3">
         <v>59.4</v>
       </c>
       <c r="BU3">
-        <v>57.5</v>
+        <v>57.7</v>
       </c>
       <c r="BV3">
-        <v>54.4</v>
+        <v>53</v>
       </c>
       <c r="BW3">
-        <v>9.199999999999999</v>
+        <v>11.6</v>
       </c>
       <c r="BX3" t="s">
         <v>68</v>
@@ -2189,28 +2189,28 @@
         <v>151</v>
       </c>
       <c r="J4">
-        <v>85.90000000000001</v>
+        <v>58.3</v>
       </c>
       <c r="K4">
-        <v>4.4</v>
+        <v>4.1</v>
       </c>
       <c r="L4">
         <v>5</v>
       </c>
       <c r="M4">
-        <v>1.78</v>
+        <v>1.79</v>
       </c>
       <c r="N4">
-        <v>1.18</v>
+        <v>1.2</v>
       </c>
       <c r="O4">
         <v>0</v>
       </c>
       <c r="P4">
-        <v>7.1</v>
+        <v>7.3</v>
       </c>
       <c r="Q4">
-        <v>0.4</v>
+        <v>0.6</v>
       </c>
       <c r="R4">
         <v>100</v>
@@ -2231,19 +2231,19 @@
         <v>1</v>
       </c>
       <c r="X4">
-        <v>0.4785</v>
+        <v>0.5017</v>
       </c>
       <c r="Y4">
-        <v>0.07000000000000001</v>
+        <v>0.01</v>
       </c>
       <c r="Z4">
-        <v>0.08</v>
+        <v>0.13</v>
       </c>
       <c r="AA4">
-        <v>10.6</v>
+        <v>10.8</v>
       </c>
       <c r="AB4">
-        <v>87.59999999999999</v>
+        <v>87.5</v>
       </c>
       <c r="AC4">
         <v>77.09999999999999</v>
@@ -2267,19 +2267,19 @@
         <v>82.5</v>
       </c>
       <c r="AJ4">
-        <v>81.40000000000001</v>
+        <v>82.8</v>
       </c>
       <c r="AK4">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="AL4">
-        <v>63.5</v>
+        <v>65.3</v>
       </c>
       <c r="AM4">
-        <v>1012.4</v>
+        <v>1012.3</v>
       </c>
       <c r="AN4">
-        <v>1014.7</v>
+        <v>1014.6</v>
       </c>
       <c r="AO4">
         <v>0</v>
@@ -2294,13 +2294,13 @@
         <v>39.5</v>
       </c>
       <c r="AS4">
-        <v>867</v>
+        <v>1069</v>
       </c>
       <c r="AT4">
         <v>9.1</v>
       </c>
       <c r="AU4">
-        <v>18.1</v>
+        <v>18</v>
       </c>
       <c r="AV4" t="s">
         <v>63</v>
@@ -2348,13 +2348,13 @@
         <v>0.09</v>
       </c>
       <c r="BK4">
-        <v>1.1606</v>
+        <v>1.1601</v>
       </c>
       <c r="BL4" t="s">
         <v>159</v>
       </c>
       <c r="BM4">
-        <v>1583</v>
+        <v>1586</v>
       </c>
       <c r="BN4" t="s">
         <v>59</v>
@@ -2363,7 +2363,7 @@
         <v>60</v>
       </c>
       <c r="BP4">
-        <v>80.90000000000001</v>
+        <v>81</v>
       </c>
       <c r="BQ4">
         <v>1.074</v>
@@ -2375,22 +2375,22 @@
         <v>77.59999999999999</v>
       </c>
       <c r="BT4">
-        <v>59.2</v>
+        <v>59.1</v>
       </c>
       <c r="BU4">
-        <v>57.2</v>
+        <v>57.3</v>
       </c>
       <c r="BV4">
-        <v>56.1</v>
+        <v>55.2</v>
       </c>
       <c r="BW4">
-        <v>8.699999999999999</v>
+        <v>10.7</v>
       </c>
       <c r="BX4" t="s">
         <v>68</v>
       </c>
       <c r="BY4">
-        <v>13.8</v>
+        <v>13.9</v>
       </c>
       <c r="BZ4" t="s">
         <v>68</v>
@@ -2437,28 +2437,28 @@
         <v>151</v>
       </c>
       <c r="J5">
-        <v>85.90000000000001</v>
+        <v>58.3</v>
       </c>
       <c r="K5">
-        <v>5.4</v>
+        <v>5.1</v>
       </c>
       <c r="L5">
         <v>5</v>
       </c>
       <c r="M5">
-        <v>1.8</v>
+        <v>1.81</v>
       </c>
       <c r="N5">
-        <v>1.22</v>
+        <v>1.27</v>
       </c>
       <c r="O5">
         <v>0</v>
       </c>
       <c r="P5">
-        <v>7.9</v>
+        <v>8</v>
       </c>
       <c r="Q5">
-        <v>0.4</v>
+        <v>0.5</v>
       </c>
       <c r="R5">
         <v>100</v>
@@ -2479,22 +2479,22 @@
         <v>1</v>
       </c>
       <c r="X5">
-        <v>0.405</v>
+        <v>0.4247</v>
       </c>
       <c r="Y5">
-        <v>0.06</v>
+        <v>0.01</v>
       </c>
       <c r="Z5">
-        <v>0.07000000000000001</v>
+        <v>0.11</v>
       </c>
       <c r="AA5">
-        <v>10.9</v>
+        <v>11.1</v>
       </c>
       <c r="AB5">
-        <v>89.2</v>
+        <v>89.09999999999999</v>
       </c>
       <c r="AC5">
-        <v>76.5</v>
+        <v>76.40000000000001</v>
       </c>
       <c r="AD5">
         <v>0.98</v>
@@ -2515,22 +2515,22 @@
         <v>80.5</v>
       </c>
       <c r="AJ5">
-        <v>80.7</v>
+        <v>81.5</v>
       </c>
       <c r="AK5">
-        <v>68.2</v>
+        <v>68.8</v>
       </c>
       <c r="AL5">
-        <v>67.5</v>
+        <v>69.2</v>
       </c>
       <c r="AM5">
         <v>1012.1</v>
       </c>
       <c r="AN5">
-        <v>1014.3</v>
+        <v>1014.4</v>
       </c>
       <c r="AO5">
-        <v>0</v>
+        <v>0.6</v>
       </c>
       <c r="AP5">
         <v>0</v>
@@ -2542,13 +2542,13 @@
         <v>36.3</v>
       </c>
       <c r="AS5">
-        <v>788</v>
+        <v>911</v>
       </c>
       <c r="AT5">
-        <v>9.1</v>
+        <v>9</v>
       </c>
       <c r="AU5">
-        <v>17.5</v>
+        <v>17.3</v>
       </c>
       <c r="AV5" t="s">
         <v>63</v>
@@ -2563,7 +2563,7 @@
         <v>3.1</v>
       </c>
       <c r="AZ5">
-        <v>9.1</v>
+        <v>9</v>
       </c>
       <c r="BA5">
         <v>7.3</v>
@@ -2596,13 +2596,13 @@
         <v>0.09</v>
       </c>
       <c r="BK5">
-        <v>1.1645</v>
+        <v>1.1643</v>
       </c>
       <c r="BL5" t="s">
         <v>159</v>
       </c>
       <c r="BM5">
-        <v>1461</v>
+        <v>1459</v>
       </c>
       <c r="BN5" t="s">
         <v>59</v>
@@ -2611,13 +2611,13 @@
         <v>60</v>
       </c>
       <c r="BP5">
-        <v>79.7</v>
+        <v>79.59999999999999</v>
       </c>
       <c r="BQ5">
         <v>1.071</v>
       </c>
       <c r="BR5">
-        <v>81.40000000000001</v>
+        <v>81.3</v>
       </c>
       <c r="BS5">
         <v>76.3</v>
@@ -2626,13 +2626,13 @@
         <v>58.7</v>
       </c>
       <c r="BU5">
-        <v>56.7</v>
+        <v>56.8</v>
       </c>
       <c r="BV5">
-        <v>58.5</v>
+        <v>58.1</v>
       </c>
       <c r="BW5">
-        <v>7.9</v>
+        <v>9.1</v>
       </c>
       <c r="BX5" t="s">
         <v>68</v>
@@ -2647,7 +2647,7 @@
         <v>82</v>
       </c>
       <c r="CB5">
-        <v>78.3</v>
+        <v>78.2</v>
       </c>
       <c r="CC5">
         <v>10</v>
@@ -2754,7 +2754,7 @@
         <v>58</v>
       </c>
       <c r="E2">
-        <v>62.1</v>
+        <v>62.3</v>
       </c>
       <c r="F2" t="s">
         <v>64</v>
@@ -2769,7 +2769,7 @@
         <v>6</v>
       </c>
       <c r="J2">
-        <v>3.6</v>
+        <v>3.7</v>
       </c>
       <c r="K2">
         <v>5</v>
@@ -2781,7 +2781,7 @@
         <v>85.40000000000001</v>
       </c>
       <c r="N2">
-        <v>1771</v>
+        <v>1782</v>
       </c>
       <c r="O2" t="s">
         <v>59</v>

</xml_diff>

<commit_message>
Update MLB weather 2026-07-14 02:55 PM PT
</commit_message>
<xml_diff>
--- a/mlb_weather_professional_v4_2026_07_14.xlsx
+++ b/mlb_weather_professional_v4_2026_07_14.xlsx
@@ -230,7 +230,7 @@
     <t>LOW</t>
   </si>
   <si>
-    <t>2026-07-14 02:51:42 PM PDT</t>
+    <t>2026-07-14 02:55:45 PM PDT</t>
   </si>
   <si>
     <t>Period</t>
@@ -473,7 +473,7 @@
     <t>11:00 PM EDT</t>
   </si>
   <si>
-    <t>2026-07-14 21:51:42 UTC</t>
+    <t>2026-07-14 21:55:45 UTC</t>
   </si>
   <si>
     <t>2026-07-14T20:53:25+00:00</t>
@@ -1200,10 +1200,10 @@
         <v>63</v>
       </c>
       <c r="P2">
-        <v>2.8</v>
+        <v>2.4</v>
       </c>
       <c r="Q2">
-        <v>7.4</v>
+        <v>7.1</v>
       </c>
       <c r="R2">
         <v>8.6</v>
@@ -1275,13 +1275,13 @@
         <v>67</v>
       </c>
       <c r="AO2">
-        <v>17.3</v>
+        <v>17</v>
       </c>
       <c r="AP2">
-        <v>0.01</v>
+        <v>0.04</v>
       </c>
       <c r="AQ2">
-        <v>0.18</v>
+        <v>0.16</v>
       </c>
       <c r="AR2">
         <v>0</v>
@@ -1305,7 +1305,7 @@
         <v>69</v>
       </c>
       <c r="AY2">
-        <v>58.3</v>
+        <v>62.3</v>
       </c>
       <c r="AZ2">
         <v>5</v>
@@ -1693,7 +1693,7 @@
         <v>151</v>
       </c>
       <c r="J2">
-        <v>58.3</v>
+        <v>62.3</v>
       </c>
       <c r="K2">
         <v>2.1</v>
@@ -1702,7 +1702,7 @@
         <v>5</v>
       </c>
       <c r="M2">
-        <v>0.1</v>
+        <v>0.11</v>
       </c>
       <c r="N2">
         <v>0.54</v>
@@ -1735,22 +1735,22 @@
         <v>1</v>
       </c>
       <c r="X2">
-        <v>0.7002</v>
+        <v>0.7081</v>
       </c>
       <c r="Y2">
-        <v>0.01</v>
+        <v>0.04</v>
       </c>
       <c r="Z2">
-        <v>0.18</v>
+        <v>0.16</v>
       </c>
       <c r="AA2">
-        <v>2</v>
+        <v>2.1</v>
       </c>
       <c r="AB2">
         <v>91.7</v>
       </c>
       <c r="AC2">
-        <v>82.2</v>
+        <v>81.8</v>
       </c>
       <c r="AD2">
         <v>0.98</v>
@@ -1810,31 +1810,31 @@
         <v>63</v>
       </c>
       <c r="AW2">
-        <v>225</v>
+        <v>227.8</v>
       </c>
       <c r="AX2">
-        <v>7.5</v>
+        <v>7.3</v>
       </c>
       <c r="AY2">
-        <v>3.2</v>
+        <v>2.7</v>
       </c>
       <c r="AZ2">
         <v>9.199999999999999</v>
       </c>
       <c r="BA2">
-        <v>7.4</v>
+        <v>7.1</v>
       </c>
       <c r="BB2">
-        <v>2.8</v>
+        <v>2.4</v>
       </c>
       <c r="BC2">
         <v>8.6</v>
       </c>
       <c r="BD2">
-        <v>5.1</v>
+        <v>5.5</v>
       </c>
       <c r="BE2">
-        <v>6.6</v>
+        <v>6.4</v>
       </c>
       <c r="BF2">
         <v>0.8</v>
@@ -1867,25 +1867,25 @@
         <v>60</v>
       </c>
       <c r="BP2">
-        <v>85.2</v>
+        <v>84.59999999999999</v>
       </c>
       <c r="BQ2">
-        <v>1.084</v>
+        <v>1.083</v>
       </c>
       <c r="BR2">
-        <v>86.90000000000001</v>
+        <v>86.59999999999999</v>
       </c>
       <c r="BS2">
-        <v>81.7</v>
+        <v>81.09999999999999</v>
       </c>
       <c r="BT2">
-        <v>60.4</v>
+        <v>60.5</v>
       </c>
       <c r="BU2">
-        <v>58.7</v>
+        <v>58.6</v>
       </c>
       <c r="BV2">
-        <v>46.4</v>
+        <v>46.5</v>
       </c>
       <c r="BW2">
         <v>11.8</v>
@@ -1941,7 +1941,7 @@
         <v>151</v>
       </c>
       <c r="J3">
-        <v>58.3</v>
+        <v>62.3</v>
       </c>
       <c r="K3">
         <v>3.1</v>
@@ -1950,7 +1950,7 @@
         <v>5</v>
       </c>
       <c r="M3">
-        <v>1.24</v>
+        <v>1.23</v>
       </c>
       <c r="N3">
         <v>1.12</v>
@@ -1983,22 +1983,22 @@
         <v>1</v>
       </c>
       <c r="X3">
-        <v>0.5927</v>
+        <v>0.5994</v>
       </c>
       <c r="Y3">
-        <v>0.01</v>
+        <v>0.03</v>
       </c>
       <c r="Z3">
-        <v>0.15</v>
+        <v>0.14</v>
       </c>
       <c r="AA3">
         <v>8.300000000000001</v>
       </c>
       <c r="AB3">
-        <v>88.40000000000001</v>
+        <v>88.5</v>
       </c>
       <c r="AC3">
-        <v>78.09999999999999</v>
+        <v>78.3</v>
       </c>
       <c r="AD3">
         <v>0.98</v>
@@ -2058,31 +2058,31 @@
         <v>63</v>
       </c>
       <c r="AW3">
-        <v>225</v>
+        <v>223.4</v>
       </c>
       <c r="AX3">
-        <v>7.2</v>
+        <v>7.4</v>
       </c>
       <c r="AY3">
-        <v>3</v>
+        <v>3.2</v>
       </c>
       <c r="AZ3">
         <v>8.800000000000001</v>
       </c>
       <c r="BA3">
-        <v>7.1</v>
+        <v>7.2</v>
       </c>
       <c r="BB3">
-        <v>2.7</v>
+        <v>2.9</v>
       </c>
       <c r="BC3">
         <v>8.199999999999999</v>
       </c>
       <c r="BD3">
-        <v>4.9</v>
+        <v>4.7</v>
       </c>
       <c r="BE3">
-        <v>6.3</v>
+        <v>6.5</v>
       </c>
       <c r="BF3">
         <v>0.8</v>
@@ -2115,19 +2115,19 @@
         <v>60</v>
       </c>
       <c r="BP3">
-        <v>81.7</v>
+        <v>82</v>
       </c>
       <c r="BQ3">
-        <v>1.076</v>
+        <v>1.077</v>
       </c>
       <c r="BR3">
-        <v>83.40000000000001</v>
+        <v>83.59999999999999</v>
       </c>
       <c r="BS3">
-        <v>78.5</v>
+        <v>78.8</v>
       </c>
       <c r="BT3">
-        <v>59.4</v>
+        <v>59.3</v>
       </c>
       <c r="BU3">
         <v>57.7</v>
@@ -2189,7 +2189,7 @@
         <v>151</v>
       </c>
       <c r="J4">
-        <v>58.3</v>
+        <v>62.3</v>
       </c>
       <c r="K4">
         <v>4.1</v>
@@ -2198,7 +2198,7 @@
         <v>5</v>
       </c>
       <c r="M4">
-        <v>1.79</v>
+        <v>1.78</v>
       </c>
       <c r="N4">
         <v>1.2</v>
@@ -2207,7 +2207,7 @@
         <v>0</v>
       </c>
       <c r="P4">
-        <v>7.3</v>
+        <v>7.2</v>
       </c>
       <c r="Q4">
         <v>0.6</v>
@@ -2231,13 +2231,13 @@
         <v>1</v>
       </c>
       <c r="X4">
-        <v>0.5017</v>
+        <v>0.5074</v>
       </c>
       <c r="Y4">
-        <v>0.01</v>
+        <v>0.03</v>
       </c>
       <c r="Z4">
-        <v>0.13</v>
+        <v>0.12</v>
       </c>
       <c r="AA4">
         <v>10.8</v>
@@ -2246,7 +2246,7 @@
         <v>87.5</v>
       </c>
       <c r="AC4">
-        <v>77.09999999999999</v>
+        <v>77.3</v>
       </c>
       <c r="AD4">
         <v>0.98</v>
@@ -2306,28 +2306,28 @@
         <v>63</v>
       </c>
       <c r="AW4">
-        <v>225</v>
+        <v>223.8</v>
       </c>
       <c r="AX4">
-        <v>7.5</v>
+        <v>7.6</v>
       </c>
       <c r="AY4">
-        <v>3.1</v>
+        <v>3.3</v>
       </c>
       <c r="AZ4">
         <v>9.1</v>
       </c>
       <c r="BA4">
-        <v>7.3</v>
+        <v>7.4</v>
       </c>
       <c r="BB4">
-        <v>2.8</v>
+        <v>2.9</v>
       </c>
       <c r="BC4">
         <v>8.5</v>
       </c>
       <c r="BD4">
-        <v>5.1</v>
+        <v>4.9</v>
       </c>
       <c r="BE4">
         <v>6.6</v>
@@ -2363,16 +2363,16 @@
         <v>60</v>
       </c>
       <c r="BP4">
-        <v>81</v>
+        <v>81.2</v>
       </c>
       <c r="BQ4">
-        <v>1.074</v>
+        <v>1.075</v>
       </c>
       <c r="BR4">
-        <v>82.7</v>
+        <v>82.8</v>
       </c>
       <c r="BS4">
-        <v>77.59999999999999</v>
+        <v>77.90000000000001</v>
       </c>
       <c r="BT4">
         <v>59.1</v>
@@ -2437,7 +2437,7 @@
         <v>151</v>
       </c>
       <c r="J5">
-        <v>58.3</v>
+        <v>62.3</v>
       </c>
       <c r="K5">
         <v>5.1</v>
@@ -2479,13 +2479,13 @@
         <v>1</v>
       </c>
       <c r="X5">
-        <v>0.4247</v>
+        <v>0.4295</v>
       </c>
       <c r="Y5">
-        <v>0.01</v>
+        <v>0.02</v>
       </c>
       <c r="Z5">
-        <v>0.11</v>
+        <v>0.1</v>
       </c>
       <c r="AA5">
         <v>11.1</v>
@@ -2494,7 +2494,7 @@
         <v>89.09999999999999</v>
       </c>
       <c r="AC5">
-        <v>76.40000000000001</v>
+        <v>76.2</v>
       </c>
       <c r="AD5">
         <v>0.98</v>
@@ -2554,31 +2554,31 @@
         <v>63</v>
       </c>
       <c r="AW5">
-        <v>225</v>
+        <v>226.1</v>
       </c>
       <c r="AX5">
-        <v>7.4</v>
+        <v>7.3</v>
       </c>
       <c r="AY5">
-        <v>3.1</v>
+        <v>2.9</v>
       </c>
       <c r="AZ5">
         <v>9</v>
       </c>
       <c r="BA5">
-        <v>7.3</v>
+        <v>7.2</v>
       </c>
       <c r="BB5">
-        <v>2.8</v>
+        <v>2.6</v>
       </c>
       <c r="BC5">
         <v>8.4</v>
       </c>
       <c r="BD5">
-        <v>5.1</v>
+        <v>5.2</v>
       </c>
       <c r="BE5">
-        <v>6.5</v>
+        <v>6.4</v>
       </c>
       <c r="BF5">
         <v>0.8</v>
@@ -2611,22 +2611,22 @@
         <v>60</v>
       </c>
       <c r="BP5">
-        <v>79.59999999999999</v>
+        <v>79.40000000000001</v>
       </c>
       <c r="BQ5">
         <v>1.071</v>
       </c>
       <c r="BR5">
-        <v>81.3</v>
+        <v>81.2</v>
       </c>
       <c r="BS5">
-        <v>76.3</v>
+        <v>76</v>
       </c>
       <c r="BT5">
         <v>58.7</v>
       </c>
       <c r="BU5">
-        <v>56.8</v>
+        <v>56.7</v>
       </c>
       <c r="BV5">
         <v>58.1</v>

</xml_diff>

<commit_message>
Update MLB weather 2026-07-14 03:07 PM PT
</commit_message>
<xml_diff>
--- a/mlb_weather_professional_v4_2026_07_14.xlsx
+++ b/mlb_weather_professional_v4_2026_07_14.xlsx
@@ -12,7 +12,7 @@
     <sheet name="HR Weather" sheetId="3" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Game Summary'!$A$1:$AZ$2</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Game Summary'!$A$1:$BB$2</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Hourly Detail'!$A$1:$CD$5</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'HR Weather'!$A$1:$Q$2</definedName>
   </definedNames>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="405" uniqueCount="160">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="410" uniqueCount="163">
   <si>
     <t>Date</t>
   </si>
@@ -77,6 +77,12 @@
     <t>First Pitch Wind Toward RF MPH</t>
   </si>
   <si>
+    <t>Official MLB Wind Text</t>
+  </si>
+  <si>
+    <t>Wind Data Source</t>
+  </si>
+  <si>
     <t>First Pitch Precipitation %</t>
   </si>
   <si>
@@ -215,10 +221,13 @@
     <t>SW</t>
   </si>
   <si>
+    <t>FORECAST MODEL</t>
+  </si>
+  <si>
     <t>B+</t>
   </si>
   <si>
-    <t>Density 80 | Wind 65 | Temp 64 | Altitude 62 | Confidence 90%</t>
+    <t>Density 80 | Wind 64 | Temp 64 | Altitude 62 | Confidence 90%</t>
   </si>
   <si>
     <t>🟢 Good</t>
@@ -230,7 +239,7 @@
     <t>LOW</t>
   </si>
   <si>
-    <t>2026-07-14 02:55:45 PM PDT</t>
+    <t>2026-07-14 03:07:25 PM PDT</t>
   </si>
   <si>
     <t>Period</t>
@@ -473,7 +482,7 @@
     <t>11:00 PM EDT</t>
   </si>
   <si>
-    <t>2026-07-14 21:55:45 UTC</t>
+    <t>2026-07-14 22:07:25 UTC</t>
   </si>
   <si>
     <t>2026-07-14T20:53:25+00:00</t>
@@ -946,7 +955,7 @@
   <sheetPr>
     <tabColor rgb="FF70AD47"/>
   </sheetPr>
-  <dimension ref="A1:AZ2"/>
+  <dimension ref="A1:BB2"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="12.7109375" customWidth="1"/>
@@ -963,39 +972,41 @@
     <col min="13" max="13" width="21.7109375" customWidth="1"/>
     <col min="14" max="15" width="28.7109375" customWidth="1"/>
     <col min="16" max="18" width="32.7109375" customWidth="1"/>
-    <col min="19" max="19" width="29.7109375" customWidth="1"/>
-    <col min="20" max="20" width="22.7109375" customWidth="1"/>
-    <col min="21" max="21" width="19.7109375" customWidth="1"/>
-    <col min="22" max="22" width="34.7109375" customWidth="1"/>
-    <col min="23" max="23" width="30.7109375" customWidth="1"/>
+    <col min="19" max="19" width="24.7109375" customWidth="1"/>
+    <col min="20" max="20" width="18.7109375" customWidth="1"/>
+    <col min="21" max="21" width="29.7109375" customWidth="1"/>
+    <col min="22" max="22" width="22.7109375" customWidth="1"/>
+    <col min="23" max="23" width="19.7109375" customWidth="1"/>
     <col min="24" max="24" width="34.7109375" customWidth="1"/>
-    <col min="25" max="25" width="23.7109375" customWidth="1"/>
-    <col min="26" max="26" width="24.7109375" customWidth="1"/>
-    <col min="27" max="27" width="19.7109375" customWidth="1"/>
-    <col min="28" max="28" width="32.7109375" customWidth="1"/>
-    <col min="29" max="29" width="30.7109375" customWidth="1"/>
-    <col min="30" max="32" width="34.7109375" customWidth="1"/>
-    <col min="33" max="33" width="32.7109375" customWidth="1"/>
-    <col min="34" max="34" width="28.7109375" customWidth="1"/>
-    <col min="35" max="35" width="30.7109375" customWidth="1"/>
-    <col min="36" max="36" width="23.7109375" customWidth="1"/>
-    <col min="37" max="37" width="22.7109375" customWidth="1"/>
-    <col min="38" max="38" width="17.7109375" customWidth="1"/>
-    <col min="39" max="39" width="15.7109375" customWidth="1"/>
-    <col min="40" max="40" width="19.7109375" customWidth="1"/>
-    <col min="41" max="41" width="34.7109375" customWidth="1"/>
-    <col min="42" max="42" width="21.7109375" customWidth="1"/>
-    <col min="43" max="43" width="23.7109375" customWidth="1"/>
-    <col min="44" max="44" width="33.7109375" customWidth="1"/>
-    <col min="45" max="45" width="32.7109375" customWidth="1"/>
-    <col min="46" max="46" width="16.7109375" customWidth="1"/>
-    <col min="47" max="48" width="22.7109375" customWidth="1"/>
-    <col min="49" max="50" width="28.7109375" customWidth="1"/>
-    <col min="51" max="51" width="22.7109375" customWidth="1"/>
-    <col min="52" max="52" width="18.7109375" customWidth="1"/>
+    <col min="25" max="25" width="30.7109375" customWidth="1"/>
+    <col min="26" max="26" width="34.7109375" customWidth="1"/>
+    <col min="27" max="27" width="23.7109375" customWidth="1"/>
+    <col min="28" max="28" width="24.7109375" customWidth="1"/>
+    <col min="29" max="29" width="19.7109375" customWidth="1"/>
+    <col min="30" max="30" width="32.7109375" customWidth="1"/>
+    <col min="31" max="31" width="30.7109375" customWidth="1"/>
+    <col min="32" max="34" width="34.7109375" customWidth="1"/>
+    <col min="35" max="35" width="32.7109375" customWidth="1"/>
+    <col min="36" max="36" width="28.7109375" customWidth="1"/>
+    <col min="37" max="37" width="30.7109375" customWidth="1"/>
+    <col min="38" max="38" width="23.7109375" customWidth="1"/>
+    <col min="39" max="39" width="22.7109375" customWidth="1"/>
+    <col min="40" max="40" width="17.7109375" customWidth="1"/>
+    <col min="41" max="41" width="15.7109375" customWidth="1"/>
+    <col min="42" max="42" width="19.7109375" customWidth="1"/>
+    <col min="43" max="43" width="34.7109375" customWidth="1"/>
+    <col min="44" max="44" width="21.7109375" customWidth="1"/>
+    <col min="45" max="45" width="23.7109375" customWidth="1"/>
+    <col min="46" max="46" width="33.7109375" customWidth="1"/>
+    <col min="47" max="47" width="32.7109375" customWidth="1"/>
+    <col min="48" max="48" width="16.7109375" customWidth="1"/>
+    <col min="49" max="50" width="22.7109375" customWidth="1"/>
+    <col min="51" max="52" width="28.7109375" customWidth="1"/>
+    <col min="53" max="53" width="22.7109375" customWidth="1"/>
+    <col min="54" max="54" width="18.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:52" ht="34" customHeight="1">
+    <row r="1" spans="1:54" ht="34" customHeight="1">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1152,37 +1163,43 @@
       <c r="AZ1" s="1" t="s">
         <v>51</v>
       </c>
+      <c r="BA1" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="BB1" s="1" t="s">
+        <v>53</v>
+      </c>
     </row>
-    <row r="2" spans="1:52">
+    <row r="2" spans="1:54">
       <c r="A2" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="B2" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="C2" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="D2" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="E2" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="F2" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="G2" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="H2" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="I2" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="J2" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="K2">
         <v>88.5</v>
@@ -1191,13 +1208,13 @@
         <v>54.7</v>
       </c>
       <c r="M2" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="N2">
         <v>9.199999999999999</v>
       </c>
       <c r="O2" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="P2">
         <v>2.4</v>
@@ -1208,131 +1225,134 @@
       <c r="R2">
         <v>8.6</v>
       </c>
-      <c r="S2">
+      <c r="T2" t="s">
+        <v>66</v>
+      </c>
+      <c r="U2">
         <v>0</v>
       </c>
-      <c r="T2">
-        <v>62.3</v>
-      </c>
-      <c r="U2" t="s">
-        <v>64</v>
-      </c>
-      <c r="V2" t="s">
-        <v>65</v>
-      </c>
-      <c r="W2">
+      <c r="V2">
+        <v>62.2</v>
+      </c>
+      <c r="W2" t="s">
+        <v>67</v>
+      </c>
+      <c r="X2" t="s">
+        <v>68</v>
+      </c>
+      <c r="Y2">
         <v>8</v>
       </c>
-      <c r="X2">
+      <c r="Z2">
         <v>6</v>
       </c>
-      <c r="Y2">
+      <c r="AA2">
         <v>3.7</v>
       </c>
-      <c r="Z2">
-        <v>89.59999999999999</v>
-      </c>
-      <c r="AA2" t="s">
-        <v>66</v>
-      </c>
       <c r="AB2">
-        <v>6.5</v>
-      </c>
-      <c r="AC2">
+        <v>89.7</v>
+      </c>
+      <c r="AC2" t="s">
+        <v>69</v>
+      </c>
+      <c r="AD2">
+        <v>6.4</v>
+      </c>
+      <c r="AE2">
         <v>5</v>
       </c>
-      <c r="AD2">
+      <c r="AF2">
         <v>100</v>
       </c>
-      <c r="AE2">
+      <c r="AG2">
         <v>0</v>
       </c>
-      <c r="AF2">
-        <v>4.6</v>
-      </c>
-      <c r="AG2">
+      <c r="AH2">
+        <v>4.3</v>
+      </c>
+      <c r="AI2">
         <v>0.5</v>
       </c>
-      <c r="AH2">
-        <v>1.1538</v>
-      </c>
-      <c r="AI2">
-        <v>1782</v>
-      </c>
       <c r="AJ2">
+        <v>1.1537</v>
+      </c>
+      <c r="AK2">
+        <v>1783</v>
+      </c>
+      <c r="AL2">
         <v>1012.1</v>
       </c>
-      <c r="AK2">
+      <c r="AM2">
         <v>69.2</v>
       </c>
-      <c r="AL2">
+      <c r="AN2">
         <v>85.40000000000001</v>
       </c>
-      <c r="AM2">
+      <c r="AO2">
         <v>60.3</v>
       </c>
-      <c r="AN2" t="s">
-        <v>67</v>
-      </c>
-      <c r="AO2">
+      <c r="AP2" t="s">
+        <v>70</v>
+      </c>
+      <c r="AQ2">
         <v>17</v>
       </c>
-      <c r="AP2">
-        <v>0.04</v>
-      </c>
-      <c r="AQ2">
-        <v>0.16</v>
-      </c>
       <c r="AR2">
+        <v>0.14</v>
+      </c>
+      <c r="AS2">
+        <v>0.12</v>
+      </c>
+      <c r="AT2">
         <v>0</v>
       </c>
-      <c r="AS2">
+      <c r="AU2">
         <v>0</v>
       </c>
-      <c r="AT2" t="s">
-        <v>68</v>
-      </c>
-      <c r="AU2">
+      <c r="AV2" t="s">
+        <v>71</v>
+      </c>
+      <c r="AW2">
         <v>11.8</v>
       </c>
-      <c r="AV2" t="s">
-        <v>68</v>
-      </c>
-      <c r="AW2">
+      <c r="AX2" t="s">
+        <v>71</v>
+      </c>
+      <c r="AY2">
         <v>14.2</v>
       </c>
-      <c r="AX2" t="s">
-        <v>69</v>
-      </c>
-      <c r="AY2">
-        <v>62.3</v>
-      </c>
-      <c r="AZ2">
+      <c r="AZ2" t="s">
+        <v>72</v>
+      </c>
+      <c r="BA2">
+        <v>74</v>
+      </c>
+      <c r="BB2">
         <v>5</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:AZ2"/>
+  <autoFilter ref="A1:BB2"/>
   <conditionalFormatting sqref="B2">
     <cfRule type="expression" dxfId="0" priority="1">
-      <formula>OR(ISNUMBER(SEARCH("Elite",$AA2)),ISNUMBER(SEARCH("Excellent",$AA2)),ISNUMBER(SEARCH("Very Good",$AA2)),ISNUMBER(SEARCH("Good",$AA2)))</formula>
+      <formula>OR(ISNUMBER(SEARCH("Elite",$AC2)),ISNUMBER(SEARCH("Excellent",$AC2)),ISNUMBER(SEARCH("Very Good",$AC2)),ISNUMBER(SEARCH("Good",$AC2)))</formula>
     </cfRule>
     <cfRule type="expression" dxfId="1" priority="2">
-      <formula>ISNUMBER(SEARCH("Neutral",$AA2))</formula>
+      <formula>ISNUMBER(SEARCH("Neutral",$AC2))</formula>
     </cfRule>
     <cfRule type="expression" dxfId="2" priority="3">
-      <formula>OR(ISNUMBER(SEARCH("Below Average",$AA2)),ISNUMBER(SEARCH("Poor",$AA2)))</formula>
+      <formula>OR(ISNUMBER(SEARCH("Below Average",$AC2)),ISNUMBER(SEARCH("Poor",$AC2)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C2">
     <cfRule type="expression" dxfId="0" priority="4">
-      <formula>OR(ISNUMBER(SEARCH("Elite",$AA2)),ISNUMBER(SEARCH("Excellent",$AA2)),ISNUMBER(SEARCH("Very Good",$AA2)),ISNUMBER(SEARCH("Good",$AA2)))</formula>
+      <formula>OR(ISNUMBER(SEARCH("Elite",$AC2)),ISNUMBER(SEARCH("Excellent",$AC2)),ISNUMBER(SEARCH("Very Good",$AC2)),ISNUMBER(SEARCH("Good",$AC2)))</formula>
     </cfRule>
     <cfRule type="expression" dxfId="1" priority="5">
-      <formula>ISNUMBER(SEARCH("Neutral",$AA2))</formula>
+      <formula>ISNUMBER(SEARCH("Neutral",$AC2))</formula>
     </cfRule>
     <cfRule type="expression" dxfId="2" priority="6">
-      <formula>OR(ISNUMBER(SEARCH("Below Average",$AA2)),ISNUMBER(SEARCH("Poor",$AA2)))</formula>
+      <formula>OR(ISNUMBER(SEARCH("Below Average",$AC2)),ISNUMBER(SEARCH("Poor",$AC2)))</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1430,279 +1450,279 @@
         <v>6</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>70</v>
+        <v>73</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>71</v>
+        <v>74</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="H1" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>76</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="K1" s="1" t="s">
+        <v>77</v>
+      </c>
+      <c r="L1" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="M1" s="1" t="s">
+        <v>78</v>
+      </c>
+      <c r="N1" s="1" t="s">
+        <v>79</v>
+      </c>
+      <c r="O1" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="P1" s="1" t="s">
+        <v>81</v>
+      </c>
+      <c r="Q1" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="R1" s="1" t="s">
+        <v>83</v>
+      </c>
+      <c r="S1" s="1" t="s">
+        <v>84</v>
+      </c>
+      <c r="T1" s="1" t="s">
+        <v>85</v>
+      </c>
+      <c r="U1" s="1" t="s">
+        <v>86</v>
+      </c>
+      <c r="V1" s="1" t="s">
+        <v>87</v>
+      </c>
+      <c r="W1" s="1" t="s">
+        <v>88</v>
+      </c>
+      <c r="X1" s="1" t="s">
+        <v>89</v>
+      </c>
+      <c r="Y1" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="Z1" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="AA1" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="AB1" s="1" t="s">
+        <v>93</v>
+      </c>
+      <c r="AC1" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="AD1" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="AE1" s="1" t="s">
+        <v>96</v>
+      </c>
+      <c r="AF1" s="1" t="s">
+        <v>97</v>
+      </c>
+      <c r="AG1" s="1" t="s">
+        <v>98</v>
+      </c>
+      <c r="AH1" s="1" t="s">
+        <v>99</v>
+      </c>
+      <c r="AI1" s="1" t="s">
+        <v>100</v>
+      </c>
+      <c r="AJ1" s="1" t="s">
+        <v>101</v>
+      </c>
+      <c r="AK1" s="1" t="s">
+        <v>102</v>
+      </c>
+      <c r="AL1" s="1" t="s">
+        <v>103</v>
+      </c>
+      <c r="AM1" s="1" t="s">
+        <v>104</v>
+      </c>
+      <c r="AN1" s="1" t="s">
+        <v>105</v>
+      </c>
+      <c r="AO1" s="1" t="s">
+        <v>106</v>
+      </c>
+      <c r="AP1" s="1" t="s">
+        <v>107</v>
+      </c>
+      <c r="AQ1" s="1" t="s">
+        <v>108</v>
+      </c>
+      <c r="AR1" s="1" t="s">
+        <v>109</v>
+      </c>
+      <c r="AS1" s="1" t="s">
+        <v>110</v>
+      </c>
+      <c r="AT1" s="1" t="s">
+        <v>111</v>
+      </c>
+      <c r="AU1" s="1" t="s">
+        <v>112</v>
+      </c>
+      <c r="AV1" s="1" t="s">
+        <v>113</v>
+      </c>
+      <c r="AW1" s="1" t="s">
+        <v>114</v>
+      </c>
+      <c r="AX1" s="1" t="s">
+        <v>115</v>
+      </c>
+      <c r="AY1" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="AZ1" s="1" t="s">
+        <v>117</v>
+      </c>
+      <c r="BA1" s="1" t="s">
+        <v>118</v>
+      </c>
+      <c r="BB1" s="1" t="s">
+        <v>119</v>
+      </c>
+      <c r="BC1" s="1" t="s">
+        <v>120</v>
+      </c>
+      <c r="BD1" s="1" t="s">
+        <v>121</v>
+      </c>
+      <c r="BE1" s="1" t="s">
+        <v>122</v>
+      </c>
+      <c r="BF1" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="BG1" s="1" t="s">
+        <v>124</v>
+      </c>
+      <c r="BH1" s="1" t="s">
+        <v>125</v>
+      </c>
+      <c r="BI1" s="1" t="s">
+        <v>126</v>
+      </c>
+      <c r="BJ1" s="1" t="s">
+        <v>127</v>
+      </c>
+      <c r="BK1" s="1" t="s">
+        <v>128</v>
+      </c>
+      <c r="BL1" s="1" t="s">
+        <v>129</v>
+      </c>
+      <c r="BM1" s="1" t="s">
+        <v>130</v>
+      </c>
+      <c r="BN1" s="1" t="s">
+        <v>131</v>
+      </c>
+      <c r="BO1" s="1" t="s">
+        <v>132</v>
+      </c>
+      <c r="BP1" s="1" t="s">
+        <v>133</v>
+      </c>
+      <c r="BQ1" s="1" t="s">
+        <v>134</v>
+      </c>
+      <c r="BR1" s="1" t="s">
+        <v>135</v>
+      </c>
+      <c r="BS1" s="1" t="s">
+        <v>136</v>
+      </c>
+      <c r="BT1" s="1" t="s">
+        <v>137</v>
+      </c>
+      <c r="BU1" s="1" t="s">
+        <v>138</v>
+      </c>
+      <c r="BV1" s="1" t="s">
+        <v>139</v>
+      </c>
+      <c r="BW1" s="1" t="s">
+        <v>140</v>
+      </c>
+      <c r="BX1" s="1" t="s">
+        <v>141</v>
+      </c>
+      <c r="BY1" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="BZ1" s="1" t="s">
         <v>49</v>
       </c>
-      <c r="I1" s="1" t="s">
-        <v>73</v>
-      </c>
-      <c r="J1" s="1" t="s">
-        <v>50</v>
-      </c>
-      <c r="K1" s="1" t="s">
-        <v>74</v>
-      </c>
-      <c r="L1" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="M1" s="1" t="s">
-        <v>75</v>
-      </c>
-      <c r="N1" s="1" t="s">
-        <v>76</v>
-      </c>
-      <c r="O1" s="1" t="s">
-        <v>77</v>
-      </c>
-      <c r="P1" s="1" t="s">
-        <v>78</v>
-      </c>
-      <c r="Q1" s="1" t="s">
-        <v>79</v>
-      </c>
-      <c r="R1" s="1" t="s">
-        <v>80</v>
-      </c>
-      <c r="S1" s="1" t="s">
-        <v>81</v>
-      </c>
-      <c r="T1" s="1" t="s">
-        <v>82</v>
-      </c>
-      <c r="U1" s="1" t="s">
-        <v>83</v>
-      </c>
-      <c r="V1" s="1" t="s">
-        <v>84</v>
-      </c>
-      <c r="W1" s="1" t="s">
-        <v>85</v>
-      </c>
-      <c r="X1" s="1" t="s">
-        <v>86</v>
-      </c>
-      <c r="Y1" s="1" t="s">
-        <v>87</v>
-      </c>
-      <c r="Z1" s="1" t="s">
-        <v>88</v>
-      </c>
-      <c r="AA1" s="1" t="s">
-        <v>89</v>
-      </c>
-      <c r="AB1" s="1" t="s">
-        <v>90</v>
-      </c>
-      <c r="AC1" s="1" t="s">
-        <v>91</v>
-      </c>
-      <c r="AD1" s="1" t="s">
-        <v>92</v>
-      </c>
-      <c r="AE1" s="1" t="s">
-        <v>93</v>
-      </c>
-      <c r="AF1" s="1" t="s">
-        <v>94</v>
-      </c>
-      <c r="AG1" s="1" t="s">
-        <v>95</v>
-      </c>
-      <c r="AH1" s="1" t="s">
-        <v>96</v>
-      </c>
-      <c r="AI1" s="1" t="s">
-        <v>97</v>
-      </c>
-      <c r="AJ1" s="1" t="s">
-        <v>98</v>
-      </c>
-      <c r="AK1" s="1" t="s">
-        <v>99</v>
-      </c>
-      <c r="AL1" s="1" t="s">
-        <v>100</v>
-      </c>
-      <c r="AM1" s="1" t="s">
-        <v>101</v>
-      </c>
-      <c r="AN1" s="1" t="s">
-        <v>102</v>
-      </c>
-      <c r="AO1" s="1" t="s">
-        <v>103</v>
-      </c>
-      <c r="AP1" s="1" t="s">
-        <v>104</v>
-      </c>
-      <c r="AQ1" s="1" t="s">
-        <v>105</v>
-      </c>
-      <c r="AR1" s="1" t="s">
-        <v>106</v>
-      </c>
-      <c r="AS1" s="1" t="s">
-        <v>107</v>
-      </c>
-      <c r="AT1" s="1" t="s">
-        <v>108</v>
-      </c>
-      <c r="AU1" s="1" t="s">
-        <v>109</v>
-      </c>
-      <c r="AV1" s="1" t="s">
-        <v>110</v>
-      </c>
-      <c r="AW1" s="1" t="s">
-        <v>111</v>
-      </c>
-      <c r="AX1" s="1" t="s">
-        <v>112</v>
-      </c>
-      <c r="AY1" s="1" t="s">
-        <v>113</v>
-      </c>
-      <c r="AZ1" s="1" t="s">
-        <v>114</v>
-      </c>
-      <c r="BA1" s="1" t="s">
-        <v>115</v>
-      </c>
-      <c r="BB1" s="1" t="s">
-        <v>116</v>
-      </c>
-      <c r="BC1" s="1" t="s">
-        <v>117</v>
-      </c>
-      <c r="BD1" s="1" t="s">
-        <v>118</v>
-      </c>
-      <c r="BE1" s="1" t="s">
-        <v>119</v>
-      </c>
-      <c r="BF1" s="1" t="s">
-        <v>120</v>
-      </c>
-      <c r="BG1" s="1" t="s">
-        <v>121</v>
-      </c>
-      <c r="BH1" s="1" t="s">
-        <v>122</v>
-      </c>
-      <c r="BI1" s="1" t="s">
-        <v>123</v>
-      </c>
-      <c r="BJ1" s="1" t="s">
-        <v>124</v>
-      </c>
-      <c r="BK1" s="1" t="s">
-        <v>125</v>
-      </c>
-      <c r="BL1" s="1" t="s">
-        <v>126</v>
-      </c>
-      <c r="BM1" s="1" t="s">
-        <v>127</v>
-      </c>
-      <c r="BN1" s="1" t="s">
-        <v>128</v>
-      </c>
-      <c r="BO1" s="1" t="s">
-        <v>129</v>
-      </c>
-      <c r="BP1" s="1" t="s">
-        <v>130</v>
-      </c>
-      <c r="BQ1" s="1" t="s">
-        <v>131</v>
-      </c>
-      <c r="BR1" s="1" t="s">
-        <v>132</v>
-      </c>
-      <c r="BS1" s="1" t="s">
-        <v>133</v>
-      </c>
-      <c r="BT1" s="1" t="s">
-        <v>134</v>
-      </c>
-      <c r="BU1" s="1" t="s">
-        <v>135</v>
-      </c>
-      <c r="BV1" s="1" t="s">
-        <v>136</v>
-      </c>
-      <c r="BW1" s="1" t="s">
-        <v>137</v>
-      </c>
-      <c r="BX1" s="1" t="s">
-        <v>138</v>
-      </c>
-      <c r="BY1" s="1" t="s">
-        <v>48</v>
-      </c>
-      <c r="BZ1" s="1" t="s">
-        <v>47</v>
-      </c>
       <c r="CA1" s="1" t="s">
-        <v>139</v>
+        <v>142</v>
       </c>
       <c r="CB1" s="1" t="s">
-        <v>140</v>
+        <v>143</v>
       </c>
       <c r="CC1" s="1" t="s">
-        <v>141</v>
+        <v>144</v>
       </c>
       <c r="CD1" s="1" t="s">
-        <v>142</v>
+        <v>145</v>
       </c>
     </row>
     <row r="2" spans="1:82">
       <c r="A2" t="s">
+        <v>57</v>
+      </c>
+      <c r="B2" t="s">
         <v>55</v>
       </c>
-      <c r="B2" t="s">
-        <v>53</v>
-      </c>
       <c r="C2" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="D2" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="E2" t="s">
-        <v>143</v>
+        <v>146</v>
       </c>
       <c r="F2" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="G2" t="s">
-        <v>150</v>
+        <v>153</v>
       </c>
       <c r="H2" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="I2" t="s">
-        <v>151</v>
+        <v>154</v>
       </c>
       <c r="J2">
-        <v>62.3</v>
+        <v>74</v>
       </c>
       <c r="K2">
-        <v>2.1</v>
+        <v>1.9</v>
       </c>
       <c r="L2">
         <v>5</v>
       </c>
       <c r="M2">
-        <v>0.11</v>
+        <v>0.15</v>
       </c>
       <c r="N2">
         <v>0.54</v>
@@ -1711,7 +1731,7 @@
         <v>0</v>
       </c>
       <c r="P2">
-        <v>1.2</v>
+        <v>0.8</v>
       </c>
       <c r="Q2">
         <v>0.3</v>
@@ -1723,34 +1743,34 @@
         <v>0</v>
       </c>
       <c r="T2" t="s">
-        <v>152</v>
+        <v>155</v>
       </c>
       <c r="U2" t="s">
-        <v>153</v>
+        <v>156</v>
       </c>
       <c r="V2" t="s">
-        <v>154</v>
+        <v>157</v>
       </c>
       <c r="W2">
         <v>1</v>
       </c>
       <c r="X2">
-        <v>0.7081</v>
+        <v>0.7315</v>
       </c>
       <c r="Y2">
-        <v>0.04</v>
+        <v>0.14</v>
       </c>
       <c r="Z2">
-        <v>0.16</v>
+        <v>0.12</v>
       </c>
       <c r="AA2">
-        <v>2.1</v>
+        <v>2.2</v>
       </c>
       <c r="AB2">
         <v>91.7</v>
       </c>
       <c r="AC2">
-        <v>81.8</v>
+        <v>81.7</v>
       </c>
       <c r="AD2">
         <v>0.98</v>
@@ -1765,7 +1785,7 @@
         <v>1.6</v>
       </c>
       <c r="AH2" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="AI2">
         <v>88.5</v>
@@ -1807,10 +1827,10 @@
         <v>20.4</v>
       </c>
       <c r="AV2" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="AW2">
-        <v>227.8</v>
+        <v>227.9</v>
       </c>
       <c r="AX2">
         <v>7.3</v>
@@ -1855,16 +1875,16 @@
         <v>1.1471</v>
       </c>
       <c r="BL2" t="s">
-        <v>158</v>
+        <v>161</v>
       </c>
       <c r="BM2">
         <v>1989</v>
       </c>
       <c r="BN2" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="BO2" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="BP2">
         <v>84.59999999999999</v>
@@ -1876,28 +1896,28 @@
         <v>86.59999999999999</v>
       </c>
       <c r="BS2">
-        <v>81.09999999999999</v>
+        <v>81</v>
       </c>
       <c r="BT2">
         <v>60.5</v>
       </c>
       <c r="BU2">
-        <v>58.6</v>
+        <v>58.5</v>
       </c>
       <c r="BV2">
-        <v>46.5</v>
+        <v>46.4</v>
       </c>
       <c r="BW2">
         <v>11.8</v>
       </c>
       <c r="BX2" t="s">
-        <v>68</v>
+        <v>71</v>
       </c>
       <c r="BY2">
         <v>13.4</v>
       </c>
       <c r="BZ2" t="s">
-        <v>68</v>
+        <v>71</v>
       </c>
       <c r="CA2">
         <v>91</v>
@@ -1914,52 +1934,52 @@
     </row>
     <row r="3" spans="1:82">
       <c r="A3" t="s">
+        <v>57</v>
+      </c>
+      <c r="B3" t="s">
         <v>55</v>
       </c>
-      <c r="B3" t="s">
-        <v>53</v>
-      </c>
       <c r="C3" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="D3" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="E3" t="s">
-        <v>144</v>
+        <v>147</v>
       </c>
       <c r="F3" t="s">
-        <v>147</v>
+        <v>150</v>
       </c>
       <c r="G3" t="s">
-        <v>150</v>
+        <v>153</v>
       </c>
       <c r="H3" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="I3" t="s">
-        <v>151</v>
+        <v>154</v>
       </c>
       <c r="J3">
-        <v>62.3</v>
+        <v>74</v>
       </c>
       <c r="K3">
-        <v>3.1</v>
+        <v>2.9</v>
       </c>
       <c r="L3">
         <v>5</v>
       </c>
       <c r="M3">
-        <v>1.23</v>
+        <v>1.21</v>
       </c>
       <c r="N3">
-        <v>1.12</v>
+        <v>1.13</v>
       </c>
       <c r="O3">
         <v>0</v>
       </c>
       <c r="P3">
-        <v>6.1</v>
+        <v>5.9</v>
       </c>
       <c r="Q3">
         <v>0.6</v>
@@ -1971,28 +1991,28 @@
         <v>0</v>
       </c>
       <c r="T3" t="s">
-        <v>152</v>
+        <v>155</v>
       </c>
       <c r="U3" t="s">
-        <v>154</v>
+        <v>157</v>
       </c>
       <c r="V3" t="s">
-        <v>155</v>
+        <v>158</v>
       </c>
       <c r="W3">
         <v>1</v>
       </c>
       <c r="X3">
-        <v>0.5994</v>
+        <v>0.6192</v>
       </c>
       <c r="Y3">
-        <v>0.03</v>
+        <v>0.12</v>
       </c>
       <c r="Z3">
-        <v>0.14</v>
+        <v>0.1</v>
       </c>
       <c r="AA3">
-        <v>8.300000000000001</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="AB3">
         <v>88.5</v>
@@ -2013,7 +2033,7 @@
         <v>1.6</v>
       </c>
       <c r="AH3" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="AI3">
         <v>84.7</v>
@@ -2022,7 +2042,7 @@
         <v>85.8</v>
       </c>
       <c r="AK3">
-        <v>69.3</v>
+        <v>69.40000000000001</v>
       </c>
       <c r="AL3">
         <v>61.4</v>
@@ -2055,13 +2075,13 @@
         <v>17.4</v>
       </c>
       <c r="AV3" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="AW3">
-        <v>223.4</v>
+        <v>223.6</v>
       </c>
       <c r="AX3">
-        <v>7.4</v>
+        <v>7.3</v>
       </c>
       <c r="AY3">
         <v>3.2</v>
@@ -2079,10 +2099,10 @@
         <v>8.199999999999999</v>
       </c>
       <c r="BD3">
-        <v>4.7</v>
+        <v>4.8</v>
       </c>
       <c r="BE3">
-        <v>6.5</v>
+        <v>6.4</v>
       </c>
       <c r="BF3">
         <v>0.8</v>
@@ -2100,19 +2120,19 @@
         <v>0.09</v>
       </c>
       <c r="BK3">
-        <v>1.1549</v>
+        <v>1.1548</v>
       </c>
       <c r="BL3" t="s">
-        <v>158</v>
+        <v>161</v>
       </c>
       <c r="BM3">
-        <v>1745</v>
+        <v>1746</v>
       </c>
       <c r="BN3" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="BO3" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="BP3">
         <v>82</v>
@@ -2139,13 +2159,13 @@
         <v>11.6</v>
       </c>
       <c r="BX3" t="s">
-        <v>68</v>
+        <v>71</v>
       </c>
       <c r="BY3">
         <v>14.2</v>
       </c>
       <c r="BZ3" t="s">
-        <v>68</v>
+        <v>71</v>
       </c>
       <c r="CA3">
         <v>87</v>
@@ -2162,55 +2182,55 @@
     </row>
     <row r="4" spans="1:82">
       <c r="A4" t="s">
+        <v>57</v>
+      </c>
+      <c r="B4" t="s">
         <v>55</v>
       </c>
-      <c r="B4" t="s">
-        <v>53</v>
-      </c>
       <c r="C4" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="D4" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="E4" t="s">
-        <v>145</v>
+        <v>148</v>
       </c>
       <c r="F4" t="s">
-        <v>148</v>
+        <v>151</v>
       </c>
       <c r="G4" t="s">
-        <v>150</v>
+        <v>153</v>
       </c>
       <c r="H4" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="I4" t="s">
-        <v>151</v>
+        <v>154</v>
       </c>
       <c r="J4">
-        <v>62.3</v>
+        <v>74</v>
       </c>
       <c r="K4">
-        <v>4.1</v>
+        <v>3.9</v>
       </c>
       <c r="L4">
         <v>5</v>
       </c>
       <c r="M4">
-        <v>1.78</v>
+        <v>1.77</v>
       </c>
       <c r="N4">
-        <v>1.2</v>
+        <v>1.21</v>
       </c>
       <c r="O4">
         <v>0</v>
       </c>
       <c r="P4">
-        <v>7.2</v>
+        <v>7.1</v>
       </c>
       <c r="Q4">
-        <v>0.6</v>
+        <v>0.5</v>
       </c>
       <c r="R4">
         <v>100</v>
@@ -2219,31 +2239,31 @@
         <v>0</v>
       </c>
       <c r="T4" t="s">
-        <v>152</v>
+        <v>155</v>
       </c>
       <c r="U4" t="s">
-        <v>155</v>
+        <v>158</v>
       </c>
       <c r="V4" t="s">
-        <v>156</v>
+        <v>159</v>
       </c>
       <c r="W4">
         <v>1</v>
       </c>
       <c r="X4">
-        <v>0.5074</v>
+        <v>0.5241</v>
       </c>
       <c r="Y4">
-        <v>0.03</v>
+        <v>0.1</v>
       </c>
       <c r="Z4">
-        <v>0.12</v>
+        <v>0.08</v>
       </c>
       <c r="AA4">
-        <v>10.8</v>
+        <v>10.7</v>
       </c>
       <c r="AB4">
-        <v>87.5</v>
+        <v>87.59999999999999</v>
       </c>
       <c r="AC4">
         <v>77.3</v>
@@ -2261,7 +2281,7 @@
         <v>1.6</v>
       </c>
       <c r="AH4" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="AI4">
         <v>82.5</v>
@@ -2270,7 +2290,7 @@
         <v>82.8</v>
       </c>
       <c r="AK4">
-        <v>69</v>
+        <v>69.09999999999999</v>
       </c>
       <c r="AL4">
         <v>65.3</v>
@@ -2303,10 +2323,10 @@
         <v>18</v>
       </c>
       <c r="AV4" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="AW4">
-        <v>223.8</v>
+        <v>223.9</v>
       </c>
       <c r="AX4">
         <v>7.6</v>
@@ -2327,7 +2347,7 @@
         <v>8.5</v>
       </c>
       <c r="BD4">
-        <v>4.9</v>
+        <v>5</v>
       </c>
       <c r="BE4">
         <v>6.6</v>
@@ -2351,16 +2371,16 @@
         <v>1.1601</v>
       </c>
       <c r="BL4" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
       <c r="BM4">
-        <v>1586</v>
+        <v>1587</v>
       </c>
       <c r="BN4" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="BO4" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="BP4">
         <v>81.2</v>
@@ -2387,19 +2407,19 @@
         <v>10.7</v>
       </c>
       <c r="BX4" t="s">
-        <v>68</v>
+        <v>71</v>
       </c>
       <c r="BY4">
-        <v>13.9</v>
+        <v>13.8</v>
       </c>
       <c r="BZ4" t="s">
-        <v>68</v>
+        <v>71</v>
       </c>
       <c r="CA4">
         <v>85</v>
       </c>
       <c r="CB4">
-        <v>79.5</v>
+        <v>79.59999999999999</v>
       </c>
       <c r="CC4">
         <v>10</v>
@@ -2410,52 +2430,52 @@
     </row>
     <row r="5" spans="1:82">
       <c r="A5" t="s">
+        <v>57</v>
+      </c>
+      <c r="B5" t="s">
         <v>55</v>
       </c>
-      <c r="B5" t="s">
-        <v>53</v>
-      </c>
       <c r="C5" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="D5" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="E5" t="s">
-        <v>146</v>
+        <v>149</v>
       </c>
       <c r="F5" t="s">
-        <v>149</v>
+        <v>152</v>
       </c>
       <c r="G5" t="s">
-        <v>150</v>
+        <v>153</v>
       </c>
       <c r="H5" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="I5" t="s">
-        <v>151</v>
+        <v>154</v>
       </c>
       <c r="J5">
-        <v>62.3</v>
+        <v>74</v>
       </c>
       <c r="K5">
-        <v>5.1</v>
+        <v>4.9</v>
       </c>
       <c r="L5">
         <v>5</v>
       </c>
       <c r="M5">
-        <v>1.81</v>
+        <v>1.79</v>
       </c>
       <c r="N5">
-        <v>1.27</v>
+        <v>1.28</v>
       </c>
       <c r="O5">
         <v>0</v>
       </c>
       <c r="P5">
-        <v>8</v>
+        <v>7.9</v>
       </c>
       <c r="Q5">
         <v>0.5</v>
@@ -2467,31 +2487,31 @@
         <v>0</v>
       </c>
       <c r="T5" t="s">
-        <v>152</v>
+        <v>155</v>
       </c>
       <c r="U5" t="s">
-        <v>156</v>
+        <v>159</v>
       </c>
       <c r="V5" t="s">
-        <v>157</v>
+        <v>160</v>
       </c>
       <c r="W5">
         <v>1</v>
       </c>
       <c r="X5">
-        <v>0.4295</v>
+        <v>0.4436</v>
       </c>
       <c r="Y5">
-        <v>0.02</v>
+        <v>0.09</v>
       </c>
       <c r="Z5">
-        <v>0.1</v>
+        <v>0.07000000000000001</v>
       </c>
       <c r="AA5">
-        <v>11.1</v>
+        <v>11</v>
       </c>
       <c r="AB5">
-        <v>89.09999999999999</v>
+        <v>89.2</v>
       </c>
       <c r="AC5">
         <v>76.2</v>
@@ -2509,7 +2529,7 @@
         <v>1.6</v>
       </c>
       <c r="AH5" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="AI5">
         <v>80.5</v>
@@ -2551,10 +2571,10 @@
         <v>17.3</v>
       </c>
       <c r="AV5" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="AW5">
-        <v>226.1</v>
+        <v>226.2</v>
       </c>
       <c r="AX5">
         <v>7.3</v>
@@ -2599,16 +2619,16 @@
         <v>1.1643</v>
       </c>
       <c r="BL5" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
       <c r="BM5">
         <v>1459</v>
       </c>
       <c r="BN5" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="BO5" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="BP5">
         <v>79.40000000000001</v>
@@ -2635,19 +2655,19 @@
         <v>9.1</v>
       </c>
       <c r="BX5" t="s">
-        <v>68</v>
+        <v>71</v>
       </c>
       <c r="BY5">
         <v>10.7</v>
       </c>
       <c r="BZ5" t="s">
-        <v>68</v>
+        <v>71</v>
       </c>
       <c r="CA5">
         <v>82</v>
       </c>
       <c r="CB5">
-        <v>78.2</v>
+        <v>78.3</v>
       </c>
       <c r="CC5">
         <v>10</v>
@@ -2701,66 +2721,66 @@
         <v>6</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="G1" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="I1" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="H1" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="I1" s="1" t="s">
-        <v>23</v>
-      </c>
       <c r="J1" s="1" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="K1" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="L1" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="L1" s="1" t="s">
-        <v>26</v>
-      </c>
       <c r="M1" s="1" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="N1" s="1" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="O1" s="1" t="s">
         <v>7</v>
       </c>
       <c r="P1" s="1" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="Q1" s="1" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
     </row>
     <row r="2" spans="1:17">
       <c r="A2" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="B2" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="C2" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="D2" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="E2">
-        <v>62.3</v>
+        <v>62.2</v>
       </c>
       <c r="F2" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="G2">
-        <v>89.59999999999999</v>
+        <v>89.7</v>
       </c>
       <c r="H2">
         <v>8</v>
@@ -2775,19 +2795,19 @@
         <v>5</v>
       </c>
       <c r="L2" t="s">
-        <v>66</v>
+        <v>69</v>
       </c>
       <c r="M2">
         <v>85.40000000000001</v>
       </c>
       <c r="N2">
-        <v>1782</v>
+        <v>1783</v>
       </c>
       <c r="O2" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="P2" t="s">
-        <v>68</v>
+        <v>71</v>
       </c>
       <c r="Q2">
         <v>5</v>

</xml_diff>

<commit_message>
Update MLB weather 2026-07-14 03:12 PM PT
</commit_message>
<xml_diff>
--- a/mlb_weather_professional_v4_2026_07_14.xlsx
+++ b/mlb_weather_professional_v4_2026_07_14.xlsx
@@ -227,7 +227,7 @@
     <t>B+</t>
   </si>
   <si>
-    <t>Density 80 | Wind 64 | Temp 64 | Altitude 62 | Confidence 90%</t>
+    <t>Density 80 | Wind 65 | Temp 64 | Altitude 62 | Confidence 90%</t>
   </si>
   <si>
     <t>🟢 Good</t>
@@ -239,7 +239,7 @@
     <t>LOW</t>
   </si>
   <si>
-    <t>2026-07-14 03:07:25 PM PDT</t>
+    <t>2026-07-14 03:12:42 PM PDT</t>
   </si>
   <si>
     <t>Period</t>
@@ -482,7 +482,7 @@
     <t>11:00 PM EDT</t>
   </si>
   <si>
-    <t>2026-07-14 22:07:25 UTC</t>
+    <t>2026-07-14 22:12:42 UTC</t>
   </si>
   <si>
     <t>2026-07-14T20:53:25+00:00</t>
@@ -1232,7 +1232,7 @@
         <v>0</v>
       </c>
       <c r="V2">
-        <v>62.2</v>
+        <v>62.3</v>
       </c>
       <c r="W2" t="s">
         <v>67</v>
@@ -1256,7 +1256,7 @@
         <v>69</v>
       </c>
       <c r="AD2">
-        <v>6.4</v>
+        <v>6.5</v>
       </c>
       <c r="AE2">
         <v>5</v>
@@ -1295,13 +1295,13 @@
         <v>70</v>
       </c>
       <c r="AQ2">
-        <v>17</v>
+        <v>17.1</v>
       </c>
       <c r="AR2">
-        <v>0.14</v>
+        <v>0.25</v>
       </c>
       <c r="AS2">
-        <v>0.12</v>
+        <v>0.2</v>
       </c>
       <c r="AT2">
         <v>0</v>
@@ -1319,13 +1319,13 @@
         <v>71</v>
       </c>
       <c r="AY2">
-        <v>14.2</v>
+        <v>14.1</v>
       </c>
       <c r="AZ2" t="s">
         <v>72</v>
       </c>
       <c r="BA2">
-        <v>74</v>
+        <v>79.3</v>
       </c>
       <c r="BB2">
         <v>5</v>
@@ -1713,16 +1713,16 @@
         <v>154</v>
       </c>
       <c r="J2">
-        <v>74</v>
+        <v>79.3</v>
       </c>
       <c r="K2">
-        <v>1.9</v>
+        <v>1.8</v>
       </c>
       <c r="L2">
         <v>5</v>
       </c>
       <c r="M2">
-        <v>0.15</v>
+        <v>0.19</v>
       </c>
       <c r="N2">
         <v>0.54</v>
@@ -1755,19 +1755,19 @@
         <v>1</v>
       </c>
       <c r="X2">
-        <v>0.7315</v>
+        <v>0.7423</v>
       </c>
       <c r="Y2">
-        <v>0.14</v>
+        <v>0.25</v>
       </c>
       <c r="Z2">
-        <v>0.12</v>
+        <v>0.2</v>
       </c>
       <c r="AA2">
-        <v>2.2</v>
+        <v>2.4</v>
       </c>
       <c r="AB2">
-        <v>91.7</v>
+        <v>91.59999999999999</v>
       </c>
       <c r="AC2">
         <v>81.7</v>
@@ -1830,7 +1830,7 @@
         <v>65</v>
       </c>
       <c r="AW2">
-        <v>227.9</v>
+        <v>228</v>
       </c>
       <c r="AX2">
         <v>7.3</v>
@@ -1914,7 +1914,7 @@
         <v>71</v>
       </c>
       <c r="BY2">
-        <v>13.4</v>
+        <v>13.3</v>
       </c>
       <c r="BZ2" t="s">
         <v>71</v>
@@ -1961,19 +1961,19 @@
         <v>154</v>
       </c>
       <c r="J3">
-        <v>74</v>
+        <v>79.3</v>
       </c>
       <c r="K3">
-        <v>2.9</v>
+        <v>2.8</v>
       </c>
       <c r="L3">
         <v>5</v>
       </c>
       <c r="M3">
-        <v>1.21</v>
+        <v>1.19</v>
       </c>
       <c r="N3">
-        <v>1.13</v>
+        <v>1.12</v>
       </c>
       <c r="O3">
         <v>0</v>
@@ -2003,19 +2003,19 @@
         <v>1</v>
       </c>
       <c r="X3">
-        <v>0.6192</v>
+        <v>0.6283</v>
       </c>
       <c r="Y3">
-        <v>0.12</v>
+        <v>0.21</v>
       </c>
       <c r="Z3">
-        <v>0.1</v>
+        <v>0.17</v>
       </c>
       <c r="AA3">
-        <v>8.199999999999999</v>
+        <v>8.1</v>
       </c>
       <c r="AB3">
-        <v>88.5</v>
+        <v>88.59999999999999</v>
       </c>
       <c r="AC3">
         <v>78.3</v>
@@ -2042,7 +2042,7 @@
         <v>85.8</v>
       </c>
       <c r="AK3">
-        <v>69.40000000000001</v>
+        <v>69.3</v>
       </c>
       <c r="AL3">
         <v>61.4</v>
@@ -2102,7 +2102,7 @@
         <v>4.8</v>
       </c>
       <c r="BE3">
-        <v>6.4</v>
+        <v>6.5</v>
       </c>
       <c r="BF3">
         <v>0.8</v>
@@ -2150,7 +2150,7 @@
         <v>59.3</v>
       </c>
       <c r="BU3">
-        <v>57.7</v>
+        <v>57.8</v>
       </c>
       <c r="BV3">
         <v>53</v>
@@ -2162,7 +2162,7 @@
         <v>71</v>
       </c>
       <c r="BY3">
-        <v>14.2</v>
+        <v>14.1</v>
       </c>
       <c r="BZ3" t="s">
         <v>71</v>
@@ -2209,19 +2209,19 @@
         <v>154</v>
       </c>
       <c r="J4">
-        <v>74</v>
+        <v>79.3</v>
       </c>
       <c r="K4">
-        <v>3.9</v>
+        <v>3.8</v>
       </c>
       <c r="L4">
         <v>5</v>
       </c>
       <c r="M4">
-        <v>1.77</v>
+        <v>1.75</v>
       </c>
       <c r="N4">
-        <v>1.21</v>
+        <v>1.2</v>
       </c>
       <c r="O4">
         <v>0</v>
@@ -2251,16 +2251,16 @@
         <v>1</v>
       </c>
       <c r="X4">
-        <v>0.5241</v>
+        <v>0.5319</v>
       </c>
       <c r="Y4">
-        <v>0.1</v>
+        <v>0.18</v>
       </c>
       <c r="Z4">
-        <v>0.08</v>
+        <v>0.15</v>
       </c>
       <c r="AA4">
-        <v>10.7</v>
+        <v>10.6</v>
       </c>
       <c r="AB4">
         <v>87.59999999999999</v>
@@ -2290,7 +2290,7 @@
         <v>82.8</v>
       </c>
       <c r="AK4">
-        <v>69.09999999999999</v>
+        <v>69</v>
       </c>
       <c r="AL4">
         <v>65.3</v>
@@ -2457,19 +2457,19 @@
         <v>154</v>
       </c>
       <c r="J5">
-        <v>74</v>
+        <v>79.3</v>
       </c>
       <c r="K5">
-        <v>4.9</v>
+        <v>4.8</v>
       </c>
       <c r="L5">
         <v>5</v>
       </c>
       <c r="M5">
-        <v>1.79</v>
+        <v>1.78</v>
       </c>
       <c r="N5">
-        <v>1.28</v>
+        <v>1.27</v>
       </c>
       <c r="O5">
         <v>0</v>
@@ -2499,16 +2499,16 @@
         <v>1</v>
       </c>
       <c r="X5">
-        <v>0.4436</v>
+        <v>0.4502</v>
       </c>
       <c r="Y5">
-        <v>0.09</v>
+        <v>0.15</v>
       </c>
       <c r="Z5">
-        <v>0.07000000000000001</v>
+        <v>0.12</v>
       </c>
       <c r="AA5">
-        <v>11</v>
+        <v>10.9</v>
       </c>
       <c r="AB5">
         <v>89.2</v>
@@ -2565,7 +2565,7 @@
         <v>911</v>
       </c>
       <c r="AT5">
-        <v>9</v>
+        <v>9.1</v>
       </c>
       <c r="AU5">
         <v>17.3</v>
@@ -2774,7 +2774,7 @@
         <v>60</v>
       </c>
       <c r="E2">
-        <v>62.2</v>
+        <v>62.3</v>
       </c>
       <c r="F2" t="s">
         <v>67</v>

</xml_diff>

<commit_message>
Update MLB weather 2026-07-14 03:15 PM PT
</commit_message>
<xml_diff>
--- a/mlb_weather_professional_v4_2026_07_14.xlsx
+++ b/mlb_weather_professional_v4_2026_07_14.xlsx
@@ -215,7 +215,7 @@
     <t>Clear</t>
   </si>
   <si>
-    <t>🟢 8.6 mph Out to RF</t>
+    <t>🟢 8.5 mph Out to RF</t>
   </si>
   <si>
     <t>SW</t>
@@ -227,7 +227,7 @@
     <t>B+</t>
   </si>
   <si>
-    <t>Density 80 | Wind 65 | Temp 64 | Altitude 62 | Confidence 90%</t>
+    <t>Density 80 | Wind 64 | Temp 64 | Altitude 62 | Confidence 90%</t>
   </si>
   <si>
     <t>🟢 Good</t>
@@ -239,7 +239,7 @@
     <t>LOW</t>
   </si>
   <si>
-    <t>2026-07-14 03:12:42 PM PDT</t>
+    <t>2026-07-14 03:15:03 PM PDT</t>
   </si>
   <si>
     <t>Period</t>
@@ -482,7 +482,7 @@
     <t>11:00 PM EDT</t>
   </si>
   <si>
-    <t>2026-07-14 22:12:42 UTC</t>
+    <t>2026-07-14 22:15:03 UTC</t>
   </si>
   <si>
     <t>2026-07-14T20:53:25+00:00</t>
@@ -1223,7 +1223,7 @@
         <v>7.1</v>
       </c>
       <c r="R2">
-        <v>8.6</v>
+        <v>8.5</v>
       </c>
       <c r="T2" t="s">
         <v>66</v>
@@ -1232,7 +1232,7 @@
         <v>0</v>
       </c>
       <c r="V2">
-        <v>62.3</v>
+        <v>62.2</v>
       </c>
       <c r="W2" t="s">
         <v>67</v>
@@ -1256,7 +1256,7 @@
         <v>69</v>
       </c>
       <c r="AD2">
-        <v>6.5</v>
+        <v>6.4</v>
       </c>
       <c r="AE2">
         <v>5</v>
@@ -1283,7 +1283,7 @@
         <v>1012.1</v>
       </c>
       <c r="AM2">
-        <v>69.2</v>
+        <v>69.3</v>
       </c>
       <c r="AN2">
         <v>85.40000000000001</v>
@@ -1295,13 +1295,13 @@
         <v>70</v>
       </c>
       <c r="AQ2">
-        <v>17.1</v>
+        <v>17</v>
       </c>
       <c r="AR2">
-        <v>0.25</v>
+        <v>0.15</v>
       </c>
       <c r="AS2">
-        <v>0.2</v>
+        <v>0.09</v>
       </c>
       <c r="AT2">
         <v>0</v>
@@ -1319,13 +1319,13 @@
         <v>71</v>
       </c>
       <c r="AY2">
-        <v>14.1</v>
+        <v>14.2</v>
       </c>
       <c r="AZ2" t="s">
         <v>72</v>
       </c>
       <c r="BA2">
-        <v>79.3</v>
+        <v>81.59999999999999</v>
       </c>
       <c r="BB2">
         <v>5</v>
@@ -1713,16 +1713,16 @@
         <v>154</v>
       </c>
       <c r="J2">
-        <v>79.3</v>
+        <v>81.59999999999999</v>
       </c>
       <c r="K2">
-        <v>1.8</v>
+        <v>1.7</v>
       </c>
       <c r="L2">
         <v>5</v>
       </c>
       <c r="M2">
-        <v>0.19</v>
+        <v>0.15</v>
       </c>
       <c r="N2">
         <v>0.54</v>
@@ -1731,7 +1731,7 @@
         <v>0</v>
       </c>
       <c r="P2">
-        <v>0.8</v>
+        <v>0.9</v>
       </c>
       <c r="Q2">
         <v>0.3</v>
@@ -1755,19 +1755,19 @@
         <v>1</v>
       </c>
       <c r="X2">
-        <v>0.7423</v>
+        <v>0.7471</v>
       </c>
       <c r="Y2">
-        <v>0.25</v>
+        <v>0.15</v>
       </c>
       <c r="Z2">
-        <v>0.2</v>
+        <v>0.09</v>
       </c>
       <c r="AA2">
-        <v>2.4</v>
+        <v>2.2</v>
       </c>
       <c r="AB2">
-        <v>91.59999999999999</v>
+        <v>91.7</v>
       </c>
       <c r="AC2">
         <v>81.7</v>
@@ -1794,7 +1794,7 @@
         <v>89.8</v>
       </c>
       <c r="AK2">
-        <v>69.3</v>
+        <v>69.40000000000001</v>
       </c>
       <c r="AL2">
         <v>54.7</v>
@@ -1830,10 +1830,10 @@
         <v>65</v>
       </c>
       <c r="AW2">
-        <v>228</v>
+        <v>228.2</v>
       </c>
       <c r="AX2">
-        <v>7.3</v>
+        <v>7.2</v>
       </c>
       <c r="AY2">
         <v>2.7</v>
@@ -1848,7 +1848,7 @@
         <v>2.4</v>
       </c>
       <c r="BC2">
-        <v>8.6</v>
+        <v>8.5</v>
       </c>
       <c r="BD2">
         <v>5.5</v>
@@ -1893,7 +1893,7 @@
         <v>1.083</v>
       </c>
       <c r="BR2">
-        <v>86.59999999999999</v>
+        <v>86.5</v>
       </c>
       <c r="BS2">
         <v>81</v>
@@ -1961,25 +1961,25 @@
         <v>154</v>
       </c>
       <c r="J3">
-        <v>79.3</v>
+        <v>81.59999999999999</v>
       </c>
       <c r="K3">
-        <v>2.8</v>
+        <v>2.7</v>
       </c>
       <c r="L3">
         <v>5</v>
       </c>
       <c r="M3">
-        <v>1.19</v>
+        <v>1.21</v>
       </c>
       <c r="N3">
-        <v>1.12</v>
+        <v>1.13</v>
       </c>
       <c r="O3">
         <v>0</v>
       </c>
       <c r="P3">
-        <v>5.9</v>
+        <v>5.7</v>
       </c>
       <c r="Q3">
         <v>0.6</v>
@@ -2003,19 +2003,19 @@
         <v>1</v>
       </c>
       <c r="X3">
-        <v>0.6283</v>
+        <v>0.6324</v>
       </c>
       <c r="Y3">
-        <v>0.21</v>
+        <v>0.13</v>
       </c>
       <c r="Z3">
-        <v>0.17</v>
+        <v>0.08</v>
       </c>
       <c r="AA3">
-        <v>8.1</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="AB3">
-        <v>88.59999999999999</v>
+        <v>88.5</v>
       </c>
       <c r="AC3">
         <v>78.3</v>
@@ -2042,7 +2042,7 @@
         <v>85.8</v>
       </c>
       <c r="AK3">
-        <v>69.3</v>
+        <v>69.40000000000001</v>
       </c>
       <c r="AL3">
         <v>61.4</v>
@@ -2078,7 +2078,7 @@
         <v>65</v>
       </c>
       <c r="AW3">
-        <v>223.6</v>
+        <v>223.7</v>
       </c>
       <c r="AX3">
         <v>7.3</v>
@@ -2102,7 +2102,7 @@
         <v>4.8</v>
       </c>
       <c r="BE3">
-        <v>6.5</v>
+        <v>6.4</v>
       </c>
       <c r="BF3">
         <v>0.8</v>
@@ -2141,19 +2141,19 @@
         <v>1.077</v>
       </c>
       <c r="BR3">
-        <v>83.59999999999999</v>
+        <v>83.5</v>
       </c>
       <c r="BS3">
-        <v>78.8</v>
+        <v>78.7</v>
       </c>
       <c r="BT3">
         <v>59.3</v>
       </c>
       <c r="BU3">
-        <v>57.8</v>
+        <v>57.7</v>
       </c>
       <c r="BV3">
-        <v>53</v>
+        <v>52.9</v>
       </c>
       <c r="BW3">
         <v>11.6</v>
@@ -2162,7 +2162,7 @@
         <v>71</v>
       </c>
       <c r="BY3">
-        <v>14.1</v>
+        <v>14.2</v>
       </c>
       <c r="BZ3" t="s">
         <v>71</v>
@@ -2209,25 +2209,25 @@
         <v>154</v>
       </c>
       <c r="J4">
-        <v>79.3</v>
+        <v>81.59999999999999</v>
       </c>
       <c r="K4">
-        <v>3.8</v>
+        <v>3.7</v>
       </c>
       <c r="L4">
         <v>5</v>
       </c>
       <c r="M4">
-        <v>1.75</v>
+        <v>1.77</v>
       </c>
       <c r="N4">
-        <v>1.2</v>
+        <v>1.21</v>
       </c>
       <c r="O4">
         <v>0</v>
       </c>
       <c r="P4">
-        <v>7.1</v>
+        <v>7</v>
       </c>
       <c r="Q4">
         <v>0.5</v>
@@ -2251,16 +2251,16 @@
         <v>1</v>
       </c>
       <c r="X4">
-        <v>0.5319</v>
+        <v>0.5353</v>
       </c>
       <c r="Y4">
-        <v>0.18</v>
+        <v>0.11</v>
       </c>
       <c r="Z4">
-        <v>0.15</v>
+        <v>0.07000000000000001</v>
       </c>
       <c r="AA4">
-        <v>10.6</v>
+        <v>10.7</v>
       </c>
       <c r="AB4">
         <v>87.59999999999999</v>
@@ -2290,10 +2290,10 @@
         <v>82.8</v>
       </c>
       <c r="AK4">
-        <v>69</v>
+        <v>69.09999999999999</v>
       </c>
       <c r="AL4">
-        <v>65.3</v>
+        <v>65.40000000000001</v>
       </c>
       <c r="AM4">
         <v>1012.3</v>
@@ -2326,10 +2326,10 @@
         <v>65</v>
       </c>
       <c r="AW4">
-        <v>223.9</v>
+        <v>224.1</v>
       </c>
       <c r="AX4">
-        <v>7.6</v>
+        <v>7.5</v>
       </c>
       <c r="AY4">
         <v>3.3</v>
@@ -2392,7 +2392,7 @@
         <v>82.8</v>
       </c>
       <c r="BS4">
-        <v>77.90000000000001</v>
+        <v>77.8</v>
       </c>
       <c r="BT4">
         <v>59.1</v>
@@ -2457,25 +2457,25 @@
         <v>154</v>
       </c>
       <c r="J5">
-        <v>79.3</v>
+        <v>81.59999999999999</v>
       </c>
       <c r="K5">
-        <v>4.8</v>
+        <v>4.7</v>
       </c>
       <c r="L5">
         <v>5</v>
       </c>
       <c r="M5">
-        <v>1.78</v>
+        <v>1.79</v>
       </c>
       <c r="N5">
-        <v>1.27</v>
+        <v>1.28</v>
       </c>
       <c r="O5">
         <v>0</v>
       </c>
       <c r="P5">
-        <v>7.9</v>
+        <v>7.8</v>
       </c>
       <c r="Q5">
         <v>0.5</v>
@@ -2499,16 +2499,16 @@
         <v>1</v>
       </c>
       <c r="X5">
-        <v>0.4502</v>
+        <v>0.4532</v>
       </c>
       <c r="Y5">
-        <v>0.15</v>
+        <v>0.09</v>
       </c>
       <c r="Z5">
-        <v>0.12</v>
+        <v>0.06</v>
       </c>
       <c r="AA5">
-        <v>10.9</v>
+        <v>11</v>
       </c>
       <c r="AB5">
         <v>89.2</v>
@@ -2565,16 +2565,16 @@
         <v>911</v>
       </c>
       <c r="AT5">
-        <v>9.1</v>
+        <v>9</v>
       </c>
       <c r="AU5">
-        <v>17.3</v>
+        <v>17.4</v>
       </c>
       <c r="AV5" t="s">
         <v>65</v>
       </c>
       <c r="AW5">
-        <v>226.2</v>
+        <v>226.3</v>
       </c>
       <c r="AX5">
         <v>7.3</v>
@@ -2586,7 +2586,7 @@
         <v>9</v>
       </c>
       <c r="BA5">
-        <v>7.2</v>
+        <v>7.1</v>
       </c>
       <c r="BB5">
         <v>2.6</v>
@@ -2774,7 +2774,7 @@
         <v>60</v>
       </c>
       <c r="E2">
-        <v>62.3</v>
+        <v>62.2</v>
       </c>
       <c r="F2" t="s">
         <v>67</v>

</xml_diff>

<commit_message>
Update MLB weather 2026-07-14 04:30 PM PT
</commit_message>
<xml_diff>
--- a/mlb_weather_professional_v4_2026_07_14.xlsx
+++ b/mlb_weather_professional_v4_2026_07_14.xlsx
@@ -215,7 +215,7 @@
     <t>Clear</t>
   </si>
   <si>
-    <t>🟢 8.5 mph Out to RF</t>
+    <t>🟢 8.6 mph Out to RF</t>
   </si>
   <si>
     <t>SW</t>
@@ -227,7 +227,7 @@
     <t>B+</t>
   </si>
   <si>
-    <t>Density 80 | Wind 64 | Temp 64 | Altitude 62 | Confidence 90%</t>
+    <t>Density 80 | Wind 65 | Temp 64 | Altitude 62 | Confidence 88%</t>
   </si>
   <si>
     <t>🟢 Good</t>
@@ -239,7 +239,7 @@
     <t>LOW</t>
   </si>
   <si>
-    <t>2026-07-14 03:15:03 PM PDT</t>
+    <t>2026-07-14 04:30:55 PM PDT</t>
   </si>
   <si>
     <t>Period</t>
@@ -482,10 +482,10 @@
     <t>11:00 PM EDT</t>
   </si>
   <si>
-    <t>2026-07-14 22:15:03 UTC</t>
-  </si>
-  <si>
-    <t>2026-07-14T20:53:25+00:00</t>
+    <t>2026-07-14 23:30:55 UTC</t>
+  </si>
+  <si>
+    <t>2026-07-14T21:58:43+00:00</t>
   </si>
   <si>
     <t>YES</t>
@@ -1202,28 +1202,28 @@
         <v>63</v>
       </c>
       <c r="K2">
-        <v>88.5</v>
+        <v>87.8</v>
       </c>
       <c r="L2">
-        <v>54.7</v>
+        <v>56.3</v>
       </c>
       <c r="M2" t="s">
         <v>64</v>
       </c>
       <c r="N2">
-        <v>9.199999999999999</v>
+        <v>9.300000000000001</v>
       </c>
       <c r="O2" t="s">
         <v>65</v>
       </c>
       <c r="P2">
-        <v>2.4</v>
+        <v>2.6</v>
       </c>
       <c r="Q2">
-        <v>7.1</v>
+        <v>7.3</v>
       </c>
       <c r="R2">
-        <v>8.5</v>
+        <v>8.6</v>
       </c>
       <c r="T2" t="s">
         <v>66</v>
@@ -1232,7 +1232,7 @@
         <v>0</v>
       </c>
       <c r="V2">
-        <v>62.2</v>
+        <v>62.1</v>
       </c>
       <c r="W2" t="s">
         <v>67</v>
@@ -1241,22 +1241,22 @@
         <v>68</v>
       </c>
       <c r="Y2">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="Z2">
         <v>6</v>
       </c>
       <c r="AA2">
-        <v>3.7</v>
+        <v>3.6</v>
       </c>
       <c r="AB2">
-        <v>89.7</v>
+        <v>88.2</v>
       </c>
       <c r="AC2" t="s">
         <v>69</v>
       </c>
       <c r="AD2">
-        <v>6.4</v>
+        <v>6.5</v>
       </c>
       <c r="AE2">
         <v>5</v>
@@ -1268,40 +1268,40 @@
         <v>0</v>
       </c>
       <c r="AH2">
-        <v>4.3</v>
+        <v>3.8</v>
       </c>
       <c r="AI2">
         <v>0.5</v>
       </c>
       <c r="AJ2">
-        <v>1.1537</v>
+        <v>1.1547</v>
       </c>
       <c r="AK2">
-        <v>1783</v>
+        <v>1751</v>
       </c>
       <c r="AL2">
-        <v>1012.1</v>
+        <v>1012.2</v>
       </c>
       <c r="AM2">
-        <v>69.3</v>
+        <v>69.40000000000001</v>
       </c>
       <c r="AN2">
-        <v>85.40000000000001</v>
+        <v>85</v>
       </c>
       <c r="AO2">
-        <v>60.3</v>
+        <v>61.6</v>
       </c>
       <c r="AP2" t="s">
         <v>70</v>
       </c>
       <c r="AQ2">
-        <v>17</v>
+        <v>16.6</v>
       </c>
       <c r="AR2">
-        <v>0.15</v>
+        <v>0.29</v>
       </c>
       <c r="AS2">
-        <v>0.09</v>
+        <v>0.26</v>
       </c>
       <c r="AT2">
         <v>0</v>
@@ -1313,19 +1313,19 @@
         <v>71</v>
       </c>
       <c r="AW2">
-        <v>11.8</v>
+        <v>12</v>
       </c>
       <c r="AX2" t="s">
         <v>71</v>
       </c>
       <c r="AY2">
-        <v>14.2</v>
+        <v>15.4</v>
       </c>
       <c r="AZ2" t="s">
         <v>72</v>
       </c>
       <c r="BA2">
-        <v>81.59999999999999</v>
+        <v>92.2</v>
       </c>
       <c r="BB2">
         <v>5</v>
@@ -1713,28 +1713,28 @@
         <v>154</v>
       </c>
       <c r="J2">
-        <v>81.59999999999999</v>
+        <v>92.2</v>
       </c>
       <c r="K2">
-        <v>1.7</v>
+        <v>0.5</v>
       </c>
       <c r="L2">
         <v>5</v>
       </c>
       <c r="M2">
-        <v>0.15</v>
+        <v>0.98</v>
       </c>
       <c r="N2">
-        <v>0.54</v>
+        <v>0.55</v>
       </c>
       <c r="O2">
         <v>0</v>
       </c>
       <c r="P2">
-        <v>0.9</v>
+        <v>1.9</v>
       </c>
       <c r="Q2">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
       <c r="R2">
         <v>100</v>
@@ -1755,22 +1755,22 @@
         <v>1</v>
       </c>
       <c r="X2">
-        <v>0.7471</v>
+        <v>0.9224</v>
       </c>
       <c r="Y2">
-        <v>0.15</v>
+        <v>0.29</v>
       </c>
       <c r="Z2">
-        <v>0.09</v>
+        <v>0.26</v>
       </c>
       <c r="AA2">
-        <v>2.2</v>
+        <v>5.6</v>
       </c>
       <c r="AB2">
-        <v>91.7</v>
+        <v>89</v>
       </c>
       <c r="AC2">
-        <v>81.7</v>
+        <v>81</v>
       </c>
       <c r="AD2">
         <v>0.98</v>
@@ -1788,22 +1788,22 @@
         <v>63</v>
       </c>
       <c r="AI2">
-        <v>88.5</v>
+        <v>87.8</v>
       </c>
       <c r="AJ2">
-        <v>89.8</v>
+        <v>87.40000000000001</v>
       </c>
       <c r="AK2">
         <v>69.40000000000001</v>
       </c>
       <c r="AL2">
-        <v>54.7</v>
+        <v>56.3</v>
       </c>
       <c r="AM2">
-        <v>1012.1</v>
+        <v>1012.3</v>
       </c>
       <c r="AN2">
-        <v>1014.3</v>
+        <v>1014.5</v>
       </c>
       <c r="AO2">
         <v>0</v>
@@ -1815,46 +1815,46 @@
         <v>0</v>
       </c>
       <c r="AR2">
-        <v>63</v>
+        <v>55.7</v>
       </c>
       <c r="AS2">
-        <v>1178</v>
+        <v>1274</v>
       </c>
       <c r="AT2">
-        <v>9.199999999999999</v>
+        <v>9.300000000000001</v>
       </c>
       <c r="AU2">
-        <v>20.4</v>
+        <v>21.8</v>
       </c>
       <c r="AV2" t="s">
         <v>65</v>
       </c>
       <c r="AW2">
-        <v>228.2</v>
+        <v>227.1</v>
       </c>
       <c r="AX2">
-        <v>7.2</v>
+        <v>7.4</v>
       </c>
       <c r="AY2">
-        <v>2.7</v>
+        <v>2.9</v>
       </c>
       <c r="AZ2">
-        <v>9.199999999999999</v>
+        <v>9.300000000000001</v>
       </c>
       <c r="BA2">
-        <v>7.1</v>
+        <v>7.3</v>
       </c>
       <c r="BB2">
-        <v>2.4</v>
+        <v>2.6</v>
       </c>
       <c r="BC2">
-        <v>8.5</v>
+        <v>8.6</v>
       </c>
       <c r="BD2">
         <v>5.5</v>
       </c>
       <c r="BE2">
-        <v>6.4</v>
+        <v>6.5</v>
       </c>
       <c r="BF2">
         <v>0.8</v>
@@ -1872,13 +1872,13 @@
         <v>0.09</v>
       </c>
       <c r="BK2">
-        <v>1.1471</v>
+        <v>1.1488</v>
       </c>
       <c r="BL2" t="s">
         <v>161</v>
       </c>
       <c r="BM2">
-        <v>1989</v>
+        <v>1933</v>
       </c>
       <c r="BN2" t="s">
         <v>61</v>
@@ -1887,34 +1887,34 @@
         <v>62</v>
       </c>
       <c r="BP2">
-        <v>84.59999999999999</v>
+        <v>84.8</v>
       </c>
       <c r="BQ2">
         <v>1.083</v>
       </c>
       <c r="BR2">
-        <v>86.5</v>
+        <v>86.7</v>
       </c>
       <c r="BS2">
-        <v>81</v>
+        <v>81.2</v>
       </c>
       <c r="BT2">
-        <v>60.5</v>
+        <v>60.4</v>
       </c>
       <c r="BU2">
         <v>58.5</v>
       </c>
       <c r="BV2">
-        <v>46.4</v>
+        <v>46</v>
       </c>
       <c r="BW2">
-        <v>11.8</v>
+        <v>12</v>
       </c>
       <c r="BX2" t="s">
         <v>71</v>
       </c>
       <c r="BY2">
-        <v>13.3</v>
+        <v>15.4</v>
       </c>
       <c r="BZ2" t="s">
         <v>71</v>
@@ -1923,13 +1923,13 @@
         <v>91</v>
       </c>
       <c r="CB2">
-        <v>85.5</v>
+        <v>84.3</v>
       </c>
       <c r="CC2">
         <v>10</v>
       </c>
       <c r="CD2">
-        <v>8.9</v>
+        <v>9.1</v>
       </c>
     </row>
     <row r="3" spans="1:82">
@@ -1961,28 +1961,28 @@
         <v>154</v>
       </c>
       <c r="J3">
-        <v>81.59999999999999</v>
+        <v>92.2</v>
       </c>
       <c r="K3">
-        <v>2.7</v>
+        <v>1.5</v>
       </c>
       <c r="L3">
         <v>5</v>
       </c>
       <c r="M3">
-        <v>1.21</v>
+        <v>1.86</v>
       </c>
       <c r="N3">
-        <v>1.13</v>
+        <v>1.07</v>
       </c>
       <c r="O3">
         <v>0</v>
       </c>
       <c r="P3">
-        <v>5.7</v>
+        <v>4</v>
       </c>
       <c r="Q3">
-        <v>0.6</v>
+        <v>0.7</v>
       </c>
       <c r="R3">
         <v>100</v>
@@ -2003,22 +2003,22 @@
         <v>1</v>
       </c>
       <c r="X3">
-        <v>0.6324</v>
+        <v>0.7808</v>
       </c>
       <c r="Y3">
-        <v>0.13</v>
+        <v>0.25</v>
       </c>
       <c r="Z3">
-        <v>0.08</v>
+        <v>0.22</v>
       </c>
       <c r="AA3">
-        <v>8.199999999999999</v>
+        <v>10.6</v>
       </c>
       <c r="AB3">
-        <v>88.5</v>
+        <v>86.90000000000001</v>
       </c>
       <c r="AC3">
-        <v>78.3</v>
+        <v>77.59999999999999</v>
       </c>
       <c r="AD3">
         <v>0.98</v>
@@ -2036,22 +2036,22 @@
         <v>63</v>
       </c>
       <c r="AI3">
+        <v>84.3</v>
+      </c>
+      <c r="AJ3">
         <v>84.7</v>
       </c>
-      <c r="AJ3">
-        <v>85.8</v>
-      </c>
       <c r="AK3">
-        <v>69.40000000000001</v>
+        <v>69.59999999999999</v>
       </c>
       <c r="AL3">
-        <v>61.4</v>
+        <v>63</v>
       </c>
       <c r="AM3">
-        <v>1011.8</v>
+        <v>1012</v>
       </c>
       <c r="AN3">
-        <v>1014.1</v>
+        <v>1014.3</v>
       </c>
       <c r="AO3">
         <v>0</v>
@@ -2063,43 +2063,43 @@
         <v>0</v>
       </c>
       <c r="AR3">
-        <v>47.5</v>
+        <v>42.6</v>
       </c>
       <c r="AS3">
-        <v>1164</v>
+        <v>1266</v>
       </c>
       <c r="AT3">
-        <v>8.800000000000001</v>
+        <v>8.9</v>
       </c>
       <c r="AU3">
-        <v>17.4</v>
+        <v>17.9</v>
       </c>
       <c r="AV3" t="s">
         <v>65</v>
       </c>
       <c r="AW3">
-        <v>223.7</v>
+        <v>225.3</v>
       </c>
       <c r="AX3">
         <v>7.3</v>
       </c>
       <c r="AY3">
-        <v>3.2</v>
+        <v>3</v>
       </c>
       <c r="AZ3">
-        <v>8.800000000000001</v>
+        <v>8.9</v>
       </c>
       <c r="BA3">
-        <v>7.2</v>
+        <v>7.1</v>
       </c>
       <c r="BB3">
-        <v>2.9</v>
+        <v>2.7</v>
       </c>
       <c r="BC3">
-        <v>8.199999999999999</v>
+        <v>8.300000000000001</v>
       </c>
       <c r="BD3">
-        <v>4.8</v>
+        <v>5</v>
       </c>
       <c r="BE3">
         <v>6.4</v>
@@ -2120,13 +2120,13 @@
         <v>0.09</v>
       </c>
       <c r="BK3">
-        <v>1.1548</v>
+        <v>1.1559</v>
       </c>
       <c r="BL3" t="s">
         <v>161</v>
       </c>
       <c r="BM3">
-        <v>1746</v>
+        <v>1711</v>
       </c>
       <c r="BN3" t="s">
         <v>61</v>
@@ -2135,34 +2135,34 @@
         <v>62</v>
       </c>
       <c r="BP3">
-        <v>82</v>
+        <v>81.8</v>
       </c>
       <c r="BQ3">
-        <v>1.077</v>
+        <v>1.076</v>
       </c>
       <c r="BR3">
         <v>83.5</v>
       </c>
       <c r="BS3">
-        <v>78.7</v>
+        <v>78.40000000000001</v>
       </c>
       <c r="BT3">
-        <v>59.3</v>
+        <v>59.4</v>
       </c>
       <c r="BU3">
         <v>57.7</v>
       </c>
       <c r="BV3">
-        <v>52.9</v>
+        <v>52.8</v>
       </c>
       <c r="BW3">
-        <v>11.6</v>
+        <v>12</v>
       </c>
       <c r="BX3" t="s">
         <v>71</v>
       </c>
       <c r="BY3">
-        <v>14.2</v>
+        <v>15.1</v>
       </c>
       <c r="BZ3" t="s">
         <v>71</v>
@@ -2171,13 +2171,13 @@
         <v>87</v>
       </c>
       <c r="CB3">
-        <v>81.90000000000001</v>
+        <v>81.09999999999999</v>
       </c>
       <c r="CC3">
         <v>10</v>
       </c>
       <c r="CD3">
-        <v>8.199999999999999</v>
+        <v>8.4</v>
       </c>
     </row>
     <row r="4" spans="1:82">
@@ -2209,25 +2209,25 @@
         <v>154</v>
       </c>
       <c r="J4">
-        <v>81.59999999999999</v>
+        <v>92.2</v>
       </c>
       <c r="K4">
-        <v>3.7</v>
+        <v>2.5</v>
       </c>
       <c r="L4">
         <v>5</v>
       </c>
       <c r="M4">
-        <v>1.77</v>
+        <v>1.74</v>
       </c>
       <c r="N4">
-        <v>1.21</v>
+        <v>1.19</v>
       </c>
       <c r="O4">
         <v>0</v>
       </c>
       <c r="P4">
-        <v>7</v>
+        <v>5.5</v>
       </c>
       <c r="Q4">
         <v>0.5</v>
@@ -2251,22 +2251,22 @@
         <v>1</v>
       </c>
       <c r="X4">
-        <v>0.5353</v>
+        <v>0.6609</v>
       </c>
       <c r="Y4">
-        <v>0.11</v>
+        <v>0.21</v>
       </c>
       <c r="Z4">
-        <v>0.07000000000000001</v>
+        <v>0.19</v>
       </c>
       <c r="AA4">
-        <v>10.7</v>
+        <v>10.5</v>
       </c>
       <c r="AB4">
-        <v>87.59999999999999</v>
+        <v>87.8</v>
       </c>
       <c r="AC4">
-        <v>77.3</v>
+        <v>77.09999999999999</v>
       </c>
       <c r="AD4">
         <v>0.98</v>
@@ -2287,13 +2287,13 @@
         <v>82.5</v>
       </c>
       <c r="AJ4">
-        <v>82.8</v>
+        <v>82.90000000000001</v>
       </c>
       <c r="AK4">
-        <v>69.09999999999999</v>
+        <v>69.2</v>
       </c>
       <c r="AL4">
-        <v>65.40000000000001</v>
+        <v>65.7</v>
       </c>
       <c r="AM4">
         <v>1012.3</v>
@@ -2311,46 +2311,46 @@
         <v>0</v>
       </c>
       <c r="AR4">
-        <v>39.5</v>
+        <v>38.3</v>
       </c>
       <c r="AS4">
-        <v>1069</v>
+        <v>1148</v>
       </c>
       <c r="AT4">
         <v>9.1</v>
       </c>
       <c r="AU4">
-        <v>18</v>
+        <v>17.8</v>
       </c>
       <c r="AV4" t="s">
         <v>65</v>
       </c>
       <c r="AW4">
-        <v>224.1</v>
+        <v>225.6</v>
       </c>
       <c r="AX4">
-        <v>7.5</v>
+        <v>7.4</v>
       </c>
       <c r="AY4">
-        <v>3.3</v>
+        <v>3</v>
       </c>
       <c r="AZ4">
         <v>9.1</v>
       </c>
       <c r="BA4">
-        <v>7.4</v>
+        <v>7.3</v>
       </c>
       <c r="BB4">
-        <v>2.9</v>
+        <v>2.7</v>
       </c>
       <c r="BC4">
         <v>8.5</v>
       </c>
       <c r="BD4">
-        <v>5</v>
+        <v>5.2</v>
       </c>
       <c r="BE4">
-        <v>6.6</v>
+        <v>6.5</v>
       </c>
       <c r="BF4">
         <v>0.8</v>
@@ -2374,7 +2374,7 @@
         <v>162</v>
       </c>
       <c r="BM4">
-        <v>1587</v>
+        <v>1586</v>
       </c>
       <c r="BN4" t="s">
         <v>61</v>
@@ -2383,19 +2383,19 @@
         <v>62</v>
       </c>
       <c r="BP4">
-        <v>81.2</v>
+        <v>80.90000000000001</v>
       </c>
       <c r="BQ4">
-        <v>1.075</v>
+        <v>1.074</v>
       </c>
       <c r="BR4">
-        <v>82.8</v>
+        <v>82.7</v>
       </c>
       <c r="BS4">
-        <v>77.8</v>
+        <v>77.5</v>
       </c>
       <c r="BT4">
-        <v>59.1</v>
+        <v>59.2</v>
       </c>
       <c r="BU4">
         <v>57.3</v>
@@ -2404,13 +2404,13 @@
         <v>55.2</v>
       </c>
       <c r="BW4">
-        <v>10.7</v>
+        <v>11.5</v>
       </c>
       <c r="BX4" t="s">
         <v>71</v>
       </c>
       <c r="BY4">
-        <v>13.8</v>
+        <v>13.5</v>
       </c>
       <c r="BZ4" t="s">
         <v>71</v>
@@ -2425,7 +2425,7 @@
         <v>10</v>
       </c>
       <c r="CD4">
-        <v>8.699999999999999</v>
+        <v>8.800000000000001</v>
       </c>
     </row>
     <row r="5" spans="1:82">
@@ -2457,25 +2457,25 @@
         <v>154</v>
       </c>
       <c r="J5">
-        <v>81.59999999999999</v>
+        <v>92.2</v>
       </c>
       <c r="K5">
-        <v>4.7</v>
+        <v>3.5</v>
       </c>
       <c r="L5">
         <v>5</v>
       </c>
       <c r="M5">
-        <v>1.79</v>
+        <v>1.64</v>
       </c>
       <c r="N5">
-        <v>1.28</v>
+        <v>1.25</v>
       </c>
       <c r="O5">
         <v>0</v>
       </c>
       <c r="P5">
-        <v>7.8</v>
+        <v>7.5</v>
       </c>
       <c r="Q5">
         <v>0.5</v>
@@ -2499,22 +2499,22 @@
         <v>1</v>
       </c>
       <c r="X5">
-        <v>0.4532</v>
+        <v>0.5595</v>
       </c>
       <c r="Y5">
-        <v>0.09</v>
+        <v>0.18</v>
       </c>
       <c r="Z5">
-        <v>0.06</v>
+        <v>0.16</v>
       </c>
       <c r="AA5">
-        <v>11</v>
+        <v>10.3</v>
       </c>
       <c r="AB5">
-        <v>89.2</v>
+        <v>89.90000000000001</v>
       </c>
       <c r="AC5">
-        <v>76.2</v>
+        <v>76.5</v>
       </c>
       <c r="AD5">
         <v>0.98</v>
@@ -2532,25 +2532,25 @@
         <v>63</v>
       </c>
       <c r="AI5">
-        <v>80.5</v>
+        <v>80.59999999999999</v>
       </c>
       <c r="AJ5">
-        <v>81.5</v>
+        <v>82.2</v>
       </c>
       <c r="AK5">
-        <v>68.8</v>
+        <v>69.2</v>
       </c>
       <c r="AL5">
-        <v>69.2</v>
+        <v>69.90000000000001</v>
       </c>
       <c r="AM5">
         <v>1012.1</v>
       </c>
       <c r="AN5">
-        <v>1014.4</v>
+        <v>1014.3</v>
       </c>
       <c r="AO5">
-        <v>0.6</v>
+        <v>1.1</v>
       </c>
       <c r="AP5">
         <v>0</v>
@@ -2559,13 +2559,13 @@
         <v>0</v>
       </c>
       <c r="AR5">
-        <v>36.3</v>
+        <v>34.9</v>
       </c>
       <c r="AS5">
-        <v>911</v>
+        <v>1063</v>
       </c>
       <c r="AT5">
-        <v>9</v>
+        <v>9.1</v>
       </c>
       <c r="AU5">
         <v>17.4</v>
@@ -2574,7 +2574,7 @@
         <v>65</v>
       </c>
       <c r="AW5">
-        <v>226.3</v>
+        <v>226.6</v>
       </c>
       <c r="AX5">
         <v>7.3</v>
@@ -2583,19 +2583,19 @@
         <v>2.9</v>
       </c>
       <c r="AZ5">
-        <v>9</v>
+        <v>9.1</v>
       </c>
       <c r="BA5">
-        <v>7.1</v>
+        <v>7.2</v>
       </c>
       <c r="BB5">
         <v>2.6</v>
       </c>
       <c r="BC5">
-        <v>8.4</v>
+        <v>8.5</v>
       </c>
       <c r="BD5">
-        <v>5.2</v>
+        <v>5.3</v>
       </c>
       <c r="BE5">
         <v>6.4</v>
@@ -2616,13 +2616,13 @@
         <v>0.09</v>
       </c>
       <c r="BK5">
-        <v>1.1643</v>
+        <v>1.1639</v>
       </c>
       <c r="BL5" t="s">
         <v>162</v>
       </c>
       <c r="BM5">
-        <v>1459</v>
+        <v>1468</v>
       </c>
       <c r="BN5" t="s">
         <v>61</v>
@@ -2631,34 +2631,34 @@
         <v>62</v>
       </c>
       <c r="BP5">
-        <v>79.40000000000001</v>
+        <v>79.5</v>
       </c>
       <c r="BQ5">
         <v>1.071</v>
       </c>
       <c r="BR5">
-        <v>81.2</v>
+        <v>81.40000000000001</v>
       </c>
       <c r="BS5">
-        <v>76</v>
+        <v>76.09999999999999</v>
       </c>
       <c r="BT5">
-        <v>58.7</v>
+        <v>58.8</v>
       </c>
       <c r="BU5">
-        <v>56.7</v>
+        <v>56.8</v>
       </c>
       <c r="BV5">
-        <v>58.1</v>
+        <v>57.6</v>
       </c>
       <c r="BW5">
-        <v>9.1</v>
+        <v>10.6</v>
       </c>
       <c r="BX5" t="s">
         <v>71</v>
       </c>
       <c r="BY5">
-        <v>10.7</v>
+        <v>10</v>
       </c>
       <c r="BZ5" t="s">
         <v>71</v>
@@ -2667,13 +2667,13 @@
         <v>82</v>
       </c>
       <c r="CB5">
-        <v>78.3</v>
+        <v>78.40000000000001</v>
       </c>
       <c r="CC5">
         <v>10</v>
       </c>
       <c r="CD5">
-        <v>8.6</v>
+        <v>8.699999999999999</v>
       </c>
     </row>
   </sheetData>
@@ -2774,22 +2774,22 @@
         <v>60</v>
       </c>
       <c r="E2">
-        <v>62.2</v>
+        <v>62.1</v>
       </c>
       <c r="F2" t="s">
         <v>67</v>
       </c>
       <c r="G2">
-        <v>89.7</v>
+        <v>88.2</v>
       </c>
       <c r="H2">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="I2">
         <v>6</v>
       </c>
       <c r="J2">
-        <v>3.7</v>
+        <v>3.6</v>
       </c>
       <c r="K2">
         <v>5</v>
@@ -2798,10 +2798,10 @@
         <v>69</v>
       </c>
       <c r="M2">
-        <v>85.40000000000001</v>
+        <v>85</v>
       </c>
       <c r="N2">
-        <v>1783</v>
+        <v>1751</v>
       </c>
       <c r="O2" t="s">
         <v>61</v>

</xml_diff>

<commit_message>
Update MLB weather 2026-07-14 04:31 PM PT
</commit_message>
<xml_diff>
--- a/mlb_weather_professional_v4_2026_07_14.xlsx
+++ b/mlb_weather_professional_v4_2026_07_14.xlsx
@@ -227,7 +227,7 @@
     <t>B+</t>
   </si>
   <si>
-    <t>Density 80 | Wind 65 | Temp 64 | Altitude 62 | Confidence 88%</t>
+    <t>Density 79 | Wind 65 | Temp 63 | Altitude 62 | Confidence 87%</t>
   </si>
   <si>
     <t>🟢 Good</t>
@@ -239,7 +239,7 @@
     <t>LOW</t>
   </si>
   <si>
-    <t>2026-07-14 04:30:55 PM PDT</t>
+    <t>2026-07-14 04:31:26 PM PDT</t>
   </si>
   <si>
     <t>Period</t>
@@ -482,7 +482,7 @@
     <t>11:00 PM EDT</t>
   </si>
   <si>
-    <t>2026-07-14 23:30:55 UTC</t>
+    <t>2026-07-14 23:31:26 UTC</t>
   </si>
   <si>
     <t>2026-07-14T21:58:43+00:00</t>
@@ -1202,7 +1202,7 @@
         <v>63</v>
       </c>
       <c r="K2">
-        <v>87.8</v>
+        <v>87.5</v>
       </c>
       <c r="L2">
         <v>56.3</v>
@@ -1211,13 +1211,13 @@
         <v>64</v>
       </c>
       <c r="N2">
-        <v>9.300000000000001</v>
+        <v>9.199999999999999</v>
       </c>
       <c r="O2" t="s">
         <v>65</v>
       </c>
       <c r="P2">
-        <v>2.6</v>
+        <v>2.7</v>
       </c>
       <c r="Q2">
         <v>7.3</v>
@@ -1232,7 +1232,7 @@
         <v>0</v>
       </c>
       <c r="V2">
-        <v>62.1</v>
+        <v>61.9</v>
       </c>
       <c r="W2" t="s">
         <v>67</v>
@@ -1244,13 +1244,13 @@
         <v>7</v>
       </c>
       <c r="Z2">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="AA2">
         <v>3.6</v>
       </c>
       <c r="AB2">
-        <v>88.2</v>
+        <v>87.2</v>
       </c>
       <c r="AC2" t="s">
         <v>69</v>
@@ -1268,25 +1268,25 @@
         <v>0</v>
       </c>
       <c r="AH2">
-        <v>3.8</v>
+        <v>5</v>
       </c>
       <c r="AI2">
         <v>0.5</v>
       </c>
       <c r="AJ2">
-        <v>1.1547</v>
+        <v>1.1552</v>
       </c>
       <c r="AK2">
-        <v>1751</v>
+        <v>1738</v>
       </c>
       <c r="AL2">
         <v>1012.2</v>
       </c>
       <c r="AM2">
-        <v>69.40000000000001</v>
+        <v>69.2</v>
       </c>
       <c r="AN2">
-        <v>85</v>
+        <v>84.8</v>
       </c>
       <c r="AO2">
         <v>61.6</v>
@@ -1295,13 +1295,13 @@
         <v>70</v>
       </c>
       <c r="AQ2">
-        <v>16.6</v>
+        <v>16.2</v>
       </c>
       <c r="AR2">
-        <v>0.29</v>
+        <v>0.38</v>
       </c>
       <c r="AS2">
-        <v>0.26</v>
+        <v>0.15</v>
       </c>
       <c r="AT2">
         <v>0</v>
@@ -1319,13 +1319,13 @@
         <v>71</v>
       </c>
       <c r="AY2">
-        <v>15.4</v>
+        <v>16.8</v>
       </c>
       <c r="AZ2" t="s">
         <v>72</v>
       </c>
       <c r="BA2">
-        <v>92.2</v>
+        <v>92.7</v>
       </c>
       <c r="BB2">
         <v>5</v>
@@ -1713,7 +1713,7 @@
         <v>154</v>
       </c>
       <c r="J2">
-        <v>92.2</v>
+        <v>92.7</v>
       </c>
       <c r="K2">
         <v>0.5</v>
@@ -1722,16 +1722,16 @@
         <v>5</v>
       </c>
       <c r="M2">
-        <v>0.98</v>
+        <v>1.41</v>
       </c>
       <c r="N2">
-        <v>0.55</v>
+        <v>0.54</v>
       </c>
       <c r="O2">
         <v>0</v>
       </c>
       <c r="P2">
-        <v>1.9</v>
+        <v>3</v>
       </c>
       <c r="Q2">
         <v>0.4</v>
@@ -1755,22 +1755,22 @@
         <v>1</v>
       </c>
       <c r="X2">
-        <v>0.9224</v>
+        <v>0.9237</v>
       </c>
       <c r="Y2">
-        <v>0.29</v>
+        <v>0.38</v>
       </c>
       <c r="Z2">
-        <v>0.26</v>
+        <v>0.15</v>
       </c>
       <c r="AA2">
-        <v>5.6</v>
+        <v>7.3</v>
       </c>
       <c r="AB2">
-        <v>89</v>
+        <v>87.5</v>
       </c>
       <c r="AC2">
-        <v>81</v>
+        <v>80.3</v>
       </c>
       <c r="AD2">
         <v>0.98</v>
@@ -1788,13 +1788,13 @@
         <v>63</v>
       </c>
       <c r="AI2">
-        <v>87.8</v>
+        <v>87.5</v>
       </c>
       <c r="AJ2">
-        <v>87.40000000000001</v>
+        <v>86.2</v>
       </c>
       <c r="AK2">
-        <v>69.40000000000001</v>
+        <v>69.09999999999999</v>
       </c>
       <c r="AL2">
         <v>56.3</v>
@@ -1815,13 +1815,13 @@
         <v>0</v>
       </c>
       <c r="AR2">
-        <v>55.7</v>
+        <v>50.6</v>
       </c>
       <c r="AS2">
         <v>1274</v>
       </c>
       <c r="AT2">
-        <v>9.300000000000001</v>
+        <v>9.199999999999999</v>
       </c>
       <c r="AU2">
         <v>21.8</v>
@@ -1830,28 +1830,28 @@
         <v>65</v>
       </c>
       <c r="AW2">
-        <v>227.1</v>
+        <v>226.1</v>
       </c>
       <c r="AX2">
         <v>7.4</v>
       </c>
       <c r="AY2">
-        <v>2.9</v>
+        <v>3</v>
       </c>
       <c r="AZ2">
-        <v>9.300000000000001</v>
+        <v>9.199999999999999</v>
       </c>
       <c r="BA2">
         <v>7.3</v>
       </c>
       <c r="BB2">
-        <v>2.6</v>
+        <v>2.7</v>
       </c>
       <c r="BC2">
         <v>8.6</v>
       </c>
       <c r="BD2">
-        <v>5.5</v>
+        <v>5.3</v>
       </c>
       <c r="BE2">
         <v>6.5</v>
@@ -1872,13 +1872,13 @@
         <v>0.09</v>
       </c>
       <c r="BK2">
-        <v>1.1488</v>
+        <v>1.1496</v>
       </c>
       <c r="BL2" t="s">
         <v>161</v>
       </c>
       <c r="BM2">
-        <v>1933</v>
+        <v>1914</v>
       </c>
       <c r="BN2" t="s">
         <v>61</v>
@@ -1887,25 +1887,25 @@
         <v>62</v>
       </c>
       <c r="BP2">
-        <v>84.8</v>
+        <v>84.59999999999999</v>
       </c>
       <c r="BQ2">
         <v>1.083</v>
       </c>
       <c r="BR2">
-        <v>86.7</v>
+        <v>86.5</v>
       </c>
       <c r="BS2">
         <v>81.2</v>
       </c>
       <c r="BT2">
-        <v>60.4</v>
+        <v>60.2</v>
       </c>
       <c r="BU2">
-        <v>58.5</v>
+        <v>58.4</v>
       </c>
       <c r="BV2">
-        <v>46</v>
+        <v>46.6</v>
       </c>
       <c r="BW2">
         <v>12</v>
@@ -1914,7 +1914,7 @@
         <v>71</v>
       </c>
       <c r="BY2">
-        <v>15.4</v>
+        <v>16.8</v>
       </c>
       <c r="BZ2" t="s">
         <v>71</v>
@@ -1923,13 +1923,13 @@
         <v>91</v>
       </c>
       <c r="CB2">
-        <v>84.3</v>
+        <v>83.8</v>
       </c>
       <c r="CC2">
         <v>10</v>
       </c>
       <c r="CD2">
-        <v>9.1</v>
+        <v>8.9</v>
       </c>
     </row>
     <row r="3" spans="1:82">
@@ -1961,7 +1961,7 @@
         <v>154</v>
       </c>
       <c r="J3">
-        <v>92.2</v>
+        <v>92.7</v>
       </c>
       <c r="K3">
         <v>1.5</v>
@@ -1970,19 +1970,19 @@
         <v>5</v>
       </c>
       <c r="M3">
-        <v>1.86</v>
+        <v>1.89</v>
       </c>
       <c r="N3">
-        <v>1.07</v>
+        <v>1.09</v>
       </c>
       <c r="O3">
         <v>0</v>
       </c>
       <c r="P3">
-        <v>4</v>
+        <v>5.1</v>
       </c>
       <c r="Q3">
-        <v>0.7</v>
+        <v>0.6</v>
       </c>
       <c r="R3">
         <v>100</v>
@@ -2003,22 +2003,22 @@
         <v>1</v>
       </c>
       <c r="X3">
-        <v>0.7808</v>
+        <v>0.7819</v>
       </c>
       <c r="Y3">
-        <v>0.25</v>
+        <v>0.32</v>
       </c>
       <c r="Z3">
-        <v>0.22</v>
+        <v>0.13</v>
       </c>
       <c r="AA3">
-        <v>10.6</v>
+        <v>10.8</v>
       </c>
       <c r="AB3">
-        <v>86.90000000000001</v>
+        <v>86.59999999999999</v>
       </c>
       <c r="AC3">
-        <v>77.59999999999999</v>
+        <v>77.40000000000001</v>
       </c>
       <c r="AD3">
         <v>0.98</v>
@@ -2039,7 +2039,7 @@
         <v>84.3</v>
       </c>
       <c r="AJ3">
-        <v>84.7</v>
+        <v>84.40000000000001</v>
       </c>
       <c r="AK3">
         <v>69.59999999999999</v>
@@ -2063,7 +2063,7 @@
         <v>0</v>
       </c>
       <c r="AR3">
-        <v>42.6</v>
+        <v>42.4</v>
       </c>
       <c r="AS3">
         <v>1266</v>
@@ -2072,34 +2072,34 @@
         <v>8.9</v>
       </c>
       <c r="AU3">
-        <v>17.9</v>
+        <v>17.3</v>
       </c>
       <c r="AV3" t="s">
         <v>65</v>
       </c>
       <c r="AW3">
-        <v>225.3</v>
+        <v>224.3</v>
       </c>
       <c r="AX3">
         <v>7.3</v>
       </c>
       <c r="AY3">
-        <v>3</v>
+        <v>3.2</v>
       </c>
       <c r="AZ3">
         <v>8.9</v>
       </c>
       <c r="BA3">
-        <v>7.1</v>
+        <v>7.2</v>
       </c>
       <c r="BB3">
-        <v>2.7</v>
+        <v>2.8</v>
       </c>
       <c r="BC3">
         <v>8.300000000000001</v>
       </c>
       <c r="BD3">
-        <v>5</v>
+        <v>4.9</v>
       </c>
       <c r="BE3">
         <v>6.4</v>
@@ -2126,7 +2126,7 @@
         <v>161</v>
       </c>
       <c r="BM3">
-        <v>1711</v>
+        <v>1709</v>
       </c>
       <c r="BN3" t="s">
         <v>61</v>
@@ -2135,25 +2135,25 @@
         <v>62</v>
       </c>
       <c r="BP3">
-        <v>81.8</v>
+        <v>81.7</v>
       </c>
       <c r="BQ3">
         <v>1.076</v>
       </c>
       <c r="BR3">
-        <v>83.5</v>
+        <v>83.3</v>
       </c>
       <c r="BS3">
         <v>78.40000000000001</v>
       </c>
       <c r="BT3">
-        <v>59.4</v>
+        <v>59.3</v>
       </c>
       <c r="BU3">
         <v>57.7</v>
       </c>
       <c r="BV3">
-        <v>52.8</v>
+        <v>53.3</v>
       </c>
       <c r="BW3">
         <v>12</v>
@@ -2162,7 +2162,7 @@
         <v>71</v>
       </c>
       <c r="BY3">
-        <v>15.1</v>
+        <v>15.5</v>
       </c>
       <c r="BZ3" t="s">
         <v>71</v>
@@ -2177,7 +2177,7 @@
         <v>10</v>
       </c>
       <c r="CD3">
-        <v>8.4</v>
+        <v>8.300000000000001</v>
       </c>
     </row>
     <row r="4" spans="1:82">
@@ -2209,7 +2209,7 @@
         <v>154</v>
       </c>
       <c r="J4">
-        <v>92.2</v>
+        <v>92.7</v>
       </c>
       <c r="K4">
         <v>2.5</v>
@@ -2218,16 +2218,16 @@
         <v>5</v>
       </c>
       <c r="M4">
-        <v>1.74</v>
+        <v>2.02</v>
       </c>
       <c r="N4">
-        <v>1.19</v>
+        <v>1.23</v>
       </c>
       <c r="O4">
         <v>0</v>
       </c>
       <c r="P4">
-        <v>5.5</v>
+        <v>6.8</v>
       </c>
       <c r="Q4">
         <v>0.5</v>
@@ -2251,22 +2251,22 @@
         <v>1</v>
       </c>
       <c r="X4">
-        <v>0.6609</v>
+        <v>0.6619</v>
       </c>
       <c r="Y4">
-        <v>0.21</v>
+        <v>0.27</v>
       </c>
       <c r="Z4">
-        <v>0.19</v>
+        <v>0.11</v>
       </c>
       <c r="AA4">
-        <v>10.5</v>
+        <v>11.8</v>
       </c>
       <c r="AB4">
-        <v>87.8</v>
+        <v>86.7</v>
       </c>
       <c r="AC4">
-        <v>77.09999999999999</v>
+        <v>76.7</v>
       </c>
       <c r="AD4">
         <v>0.98</v>
@@ -2284,13 +2284,13 @@
         <v>63</v>
       </c>
       <c r="AI4">
-        <v>82.5</v>
+        <v>82.40000000000001</v>
       </c>
       <c r="AJ4">
-        <v>82.90000000000001</v>
+        <v>82.09999999999999</v>
       </c>
       <c r="AK4">
-        <v>69.2</v>
+        <v>68.90000000000001</v>
       </c>
       <c r="AL4">
         <v>65.7</v>
@@ -2311,46 +2311,46 @@
         <v>0</v>
       </c>
       <c r="AR4">
-        <v>38.3</v>
+        <v>40.6</v>
       </c>
       <c r="AS4">
         <v>1148</v>
       </c>
       <c r="AT4">
-        <v>9.1</v>
+        <v>9</v>
       </c>
       <c r="AU4">
-        <v>17.8</v>
+        <v>17.4</v>
       </c>
       <c r="AV4" t="s">
         <v>65</v>
       </c>
       <c r="AW4">
-        <v>225.6</v>
+        <v>224.2</v>
       </c>
       <c r="AX4">
-        <v>7.4</v>
+        <v>7.5</v>
       </c>
       <c r="AY4">
-        <v>3</v>
+        <v>3.2</v>
       </c>
       <c r="AZ4">
-        <v>9.1</v>
+        <v>9</v>
       </c>
       <c r="BA4">
         <v>7.3</v>
       </c>
       <c r="BB4">
-        <v>2.7</v>
+        <v>2.9</v>
       </c>
       <c r="BC4">
-        <v>8.5</v>
+        <v>8.4</v>
       </c>
       <c r="BD4">
-        <v>5.2</v>
+        <v>5</v>
       </c>
       <c r="BE4">
-        <v>6.5</v>
+        <v>6.6</v>
       </c>
       <c r="BF4">
         <v>0.8</v>
@@ -2368,13 +2368,13 @@
         <v>0.09</v>
       </c>
       <c r="BK4">
-        <v>1.1601</v>
+        <v>1.1606</v>
       </c>
       <c r="BL4" t="s">
         <v>162</v>
       </c>
       <c r="BM4">
-        <v>1586</v>
+        <v>1573</v>
       </c>
       <c r="BN4" t="s">
         <v>61</v>
@@ -2383,25 +2383,25 @@
         <v>62</v>
       </c>
       <c r="BP4">
-        <v>80.90000000000001</v>
+        <v>80.8</v>
       </c>
       <c r="BQ4">
         <v>1.074</v>
       </c>
       <c r="BR4">
-        <v>82.7</v>
+        <v>82.5</v>
       </c>
       <c r="BS4">
         <v>77.5</v>
       </c>
       <c r="BT4">
-        <v>59.2</v>
+        <v>59.1</v>
       </c>
       <c r="BU4">
-        <v>57.3</v>
+        <v>57.2</v>
       </c>
       <c r="BV4">
-        <v>55.2</v>
+        <v>55.9</v>
       </c>
       <c r="BW4">
         <v>11.5</v>
@@ -2410,7 +2410,7 @@
         <v>71</v>
       </c>
       <c r="BY4">
-        <v>13.5</v>
+        <v>14.6</v>
       </c>
       <c r="BZ4" t="s">
         <v>71</v>
@@ -2419,13 +2419,13 @@
         <v>85</v>
       </c>
       <c r="CB4">
-        <v>79.59999999999999</v>
+        <v>79.2</v>
       </c>
       <c r="CC4">
         <v>10</v>
       </c>
       <c r="CD4">
-        <v>8.800000000000001</v>
+        <v>8.6</v>
       </c>
     </row>
     <row r="5" spans="1:82">
@@ -2457,7 +2457,7 @@
         <v>154</v>
       </c>
       <c r="J5">
-        <v>92.2</v>
+        <v>92.7</v>
       </c>
       <c r="K5">
         <v>3.5</v>
@@ -2466,16 +2466,16 @@
         <v>5</v>
       </c>
       <c r="M5">
-        <v>1.64</v>
+        <v>2.05</v>
       </c>
       <c r="N5">
-        <v>1.25</v>
+        <v>1.29</v>
       </c>
       <c r="O5">
         <v>0</v>
       </c>
       <c r="P5">
-        <v>7.5</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="Q5">
         <v>0.5</v>
@@ -2499,22 +2499,22 @@
         <v>1</v>
       </c>
       <c r="X5">
-        <v>0.5595</v>
+        <v>0.5603</v>
       </c>
       <c r="Y5">
-        <v>0.18</v>
+        <v>0.23</v>
       </c>
       <c r="Z5">
-        <v>0.16</v>
+        <v>0.09</v>
       </c>
       <c r="AA5">
-        <v>10.3</v>
+        <v>12</v>
       </c>
       <c r="AB5">
-        <v>89.90000000000001</v>
+        <v>88.40000000000001</v>
       </c>
       <c r="AC5">
-        <v>76.5</v>
+        <v>76</v>
       </c>
       <c r="AD5">
         <v>0.98</v>
@@ -2532,13 +2532,13 @@
         <v>63</v>
       </c>
       <c r="AI5">
-        <v>80.59999999999999</v>
+        <v>80.3</v>
       </c>
       <c r="AJ5">
-        <v>82.2</v>
+        <v>81</v>
       </c>
       <c r="AK5">
-        <v>69.2</v>
+        <v>68.90000000000001</v>
       </c>
       <c r="AL5">
         <v>69.90000000000001</v>
@@ -2559,46 +2559,46 @@
         <v>0</v>
       </c>
       <c r="AR5">
-        <v>34.9</v>
+        <v>40.8</v>
       </c>
       <c r="AS5">
         <v>1063</v>
       </c>
       <c r="AT5">
-        <v>9.1</v>
+        <v>9</v>
       </c>
       <c r="AU5">
-        <v>17.4</v>
+        <v>17.2</v>
       </c>
       <c r="AV5" t="s">
         <v>65</v>
       </c>
       <c r="AW5">
-        <v>226.6</v>
+        <v>225.3</v>
       </c>
       <c r="AX5">
-        <v>7.3</v>
+        <v>7.4</v>
       </c>
       <c r="AY5">
-        <v>2.9</v>
+        <v>3</v>
       </c>
       <c r="AZ5">
-        <v>9.1</v>
+        <v>9</v>
       </c>
       <c r="BA5">
         <v>7.2</v>
       </c>
       <c r="BB5">
-        <v>2.6</v>
+        <v>2.7</v>
       </c>
       <c r="BC5">
-        <v>8.5</v>
+        <v>8.4</v>
       </c>
       <c r="BD5">
-        <v>5.3</v>
+        <v>5.1</v>
       </c>
       <c r="BE5">
-        <v>6.4</v>
+        <v>6.5</v>
       </c>
       <c r="BF5">
         <v>0.8</v>
@@ -2616,13 +2616,13 @@
         <v>0.09</v>
       </c>
       <c r="BK5">
-        <v>1.1639</v>
+        <v>1.1646</v>
       </c>
       <c r="BL5" t="s">
         <v>162</v>
       </c>
       <c r="BM5">
-        <v>1468</v>
+        <v>1449</v>
       </c>
       <c r="BN5" t="s">
         <v>61</v>
@@ -2631,25 +2631,25 @@
         <v>62</v>
       </c>
       <c r="BP5">
-        <v>79.5</v>
+        <v>79.40000000000001</v>
       </c>
       <c r="BQ5">
         <v>1.071</v>
       </c>
       <c r="BR5">
-        <v>81.40000000000001</v>
+        <v>81.09999999999999</v>
       </c>
       <c r="BS5">
-        <v>76.09999999999999</v>
+        <v>76</v>
       </c>
       <c r="BT5">
-        <v>58.8</v>
+        <v>58.6</v>
       </c>
       <c r="BU5">
-        <v>56.8</v>
+        <v>56.7</v>
       </c>
       <c r="BV5">
-        <v>57.6</v>
+        <v>58.4</v>
       </c>
       <c r="BW5">
         <v>10.6</v>
@@ -2658,7 +2658,7 @@
         <v>71</v>
       </c>
       <c r="BY5">
-        <v>10</v>
+        <v>11.3</v>
       </c>
       <c r="BZ5" t="s">
         <v>71</v>
@@ -2667,13 +2667,13 @@
         <v>82</v>
       </c>
       <c r="CB5">
-        <v>78.40000000000001</v>
+        <v>77.90000000000001</v>
       </c>
       <c r="CC5">
         <v>10</v>
       </c>
       <c r="CD5">
-        <v>8.699999999999999</v>
+        <v>8.5</v>
       </c>
     </row>
   </sheetData>
@@ -2774,19 +2774,19 @@
         <v>60</v>
       </c>
       <c r="E2">
-        <v>62.1</v>
+        <v>61.9</v>
       </c>
       <c r="F2" t="s">
         <v>67</v>
       </c>
       <c r="G2">
-        <v>88.2</v>
+        <v>87.2</v>
       </c>
       <c r="H2">
         <v>7</v>
       </c>
       <c r="I2">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="J2">
         <v>3.6</v>
@@ -2798,10 +2798,10 @@
         <v>69</v>
       </c>
       <c r="M2">
-        <v>85</v>
+        <v>84.8</v>
       </c>
       <c r="N2">
-        <v>1751</v>
+        <v>1738</v>
       </c>
       <c r="O2" t="s">
         <v>61</v>

</xml_diff>

<commit_message>
Update MLB weather 2026-07-14 04:32 PM PT
</commit_message>
<xml_diff>
--- a/mlb_weather_professional_v4_2026_07_14.xlsx
+++ b/mlb_weather_professional_v4_2026_07_14.xlsx
@@ -215,7 +215,7 @@
     <t>Clear</t>
   </si>
   <si>
-    <t>🟢 8.6 mph Out to RF</t>
+    <t>🟢 8.7 mph Out to RF</t>
   </si>
   <si>
     <t>SW</t>
@@ -239,7 +239,7 @@
     <t>LOW</t>
   </si>
   <si>
-    <t>2026-07-14 04:31:26 PM PDT</t>
+    <t>2026-07-14 04:32:21 PM PDT</t>
   </si>
   <si>
     <t>Period</t>
@@ -482,7 +482,7 @@
     <t>11:00 PM EDT</t>
   </si>
   <si>
-    <t>2026-07-14 23:31:26 UTC</t>
+    <t>2026-07-14 23:32:21 UTC</t>
   </si>
   <si>
     <t>2026-07-14T21:58:43+00:00</t>
@@ -1211,19 +1211,19 @@
         <v>64</v>
       </c>
       <c r="N2">
-        <v>9.199999999999999</v>
+        <v>9.4</v>
       </c>
       <c r="O2" t="s">
         <v>65</v>
       </c>
       <c r="P2">
-        <v>2.7</v>
+        <v>2.9</v>
       </c>
       <c r="Q2">
-        <v>7.3</v>
+        <v>7.5</v>
       </c>
       <c r="R2">
-        <v>8.6</v>
+        <v>8.699999999999999</v>
       </c>
       <c r="T2" t="s">
         <v>66</v>
@@ -1250,7 +1250,7 @@
         <v>3.6</v>
       </c>
       <c r="AB2">
-        <v>87.2</v>
+        <v>87.09999999999999</v>
       </c>
       <c r="AC2" t="s">
         <v>69</v>
@@ -1268,10 +1268,10 @@
         <v>0</v>
       </c>
       <c r="AH2">
-        <v>5</v>
+        <v>4.8</v>
       </c>
       <c r="AI2">
-        <v>0.5</v>
+        <v>0.6</v>
       </c>
       <c r="AJ2">
         <v>1.1552</v>
@@ -1295,13 +1295,13 @@
         <v>70</v>
       </c>
       <c r="AQ2">
-        <v>16.2</v>
+        <v>16.4</v>
       </c>
       <c r="AR2">
-        <v>0.38</v>
+        <v>0.45</v>
       </c>
       <c r="AS2">
-        <v>0.15</v>
+        <v>0.24</v>
       </c>
       <c r="AT2">
         <v>0</v>
@@ -1319,13 +1319,13 @@
         <v>71</v>
       </c>
       <c r="AY2">
-        <v>16.8</v>
+        <v>16.2</v>
       </c>
       <c r="AZ2" t="s">
         <v>72</v>
       </c>
       <c r="BA2">
-        <v>92.7</v>
+        <v>93.59999999999999</v>
       </c>
       <c r="BB2">
         <v>5</v>
@@ -1713,7 +1713,7 @@
         <v>154</v>
       </c>
       <c r="J2">
-        <v>92.7</v>
+        <v>93.59999999999999</v>
       </c>
       <c r="K2">
         <v>0.5</v>
@@ -1722,19 +1722,19 @@
         <v>5</v>
       </c>
       <c r="M2">
-        <v>1.41</v>
+        <v>1.4</v>
       </c>
       <c r="N2">
-        <v>0.54</v>
+        <v>0.57</v>
       </c>
       <c r="O2">
         <v>0</v>
       </c>
       <c r="P2">
-        <v>3</v>
+        <v>4.4</v>
       </c>
       <c r="Q2">
-        <v>0.4</v>
+        <v>0.6</v>
       </c>
       <c r="R2">
         <v>100</v>
@@ -1755,22 +1755,22 @@
         <v>1</v>
       </c>
       <c r="X2">
-        <v>0.9237</v>
+        <v>0.9261</v>
       </c>
       <c r="Y2">
-        <v>0.38</v>
+        <v>0.45</v>
       </c>
       <c r="Z2">
-        <v>0.15</v>
+        <v>0.24</v>
       </c>
       <c r="AA2">
         <v>7.3</v>
       </c>
       <c r="AB2">
-        <v>87.5</v>
+        <v>87.8</v>
       </c>
       <c r="AC2">
-        <v>80.3</v>
+        <v>80.90000000000001</v>
       </c>
       <c r="AD2">
         <v>0.98</v>
@@ -1791,7 +1791,7 @@
         <v>87.5</v>
       </c>
       <c r="AJ2">
-        <v>86.2</v>
+        <v>86</v>
       </c>
       <c r="AK2">
         <v>69.09999999999999</v>
@@ -1821,7 +1821,7 @@
         <v>1274</v>
       </c>
       <c r="AT2">
-        <v>9.199999999999999</v>
+        <v>9.4</v>
       </c>
       <c r="AU2">
         <v>21.8</v>
@@ -1830,31 +1830,31 @@
         <v>65</v>
       </c>
       <c r="AW2">
-        <v>226.1</v>
+        <v>224.6</v>
       </c>
       <c r="AX2">
-        <v>7.4</v>
+        <v>7.7</v>
       </c>
       <c r="AY2">
-        <v>3</v>
+        <v>3.3</v>
       </c>
       <c r="AZ2">
-        <v>9.199999999999999</v>
+        <v>9.4</v>
       </c>
       <c r="BA2">
-        <v>7.3</v>
+        <v>7.5</v>
       </c>
       <c r="BB2">
-        <v>2.7</v>
+        <v>2.9</v>
       </c>
       <c r="BC2">
-        <v>8.6</v>
+        <v>8.699999999999999</v>
       </c>
       <c r="BD2">
-        <v>5.3</v>
+        <v>5.2</v>
       </c>
       <c r="BE2">
-        <v>6.5</v>
+        <v>6.8</v>
       </c>
       <c r="BF2">
         <v>0.8</v>
@@ -1878,7 +1878,7 @@
         <v>161</v>
       </c>
       <c r="BM2">
-        <v>1914</v>
+        <v>1915</v>
       </c>
       <c r="BN2" t="s">
         <v>61</v>
@@ -1887,22 +1887,22 @@
         <v>62</v>
       </c>
       <c r="BP2">
-        <v>84.59999999999999</v>
+        <v>85.2</v>
       </c>
       <c r="BQ2">
-        <v>1.083</v>
+        <v>1.084</v>
       </c>
       <c r="BR2">
-        <v>86.5</v>
+        <v>86.90000000000001</v>
       </c>
       <c r="BS2">
-        <v>81.2</v>
+        <v>81.7</v>
       </c>
       <c r="BT2">
-        <v>60.2</v>
+        <v>60.3</v>
       </c>
       <c r="BU2">
-        <v>58.4</v>
+        <v>58.5</v>
       </c>
       <c r="BV2">
         <v>46.6</v>
@@ -1914,7 +1914,7 @@
         <v>71</v>
       </c>
       <c r="BY2">
-        <v>16.8</v>
+        <v>16.2</v>
       </c>
       <c r="BZ2" t="s">
         <v>71</v>
@@ -1929,7 +1929,7 @@
         <v>10</v>
       </c>
       <c r="CD2">
-        <v>8.9</v>
+        <v>9.199999999999999</v>
       </c>
     </row>
     <row r="3" spans="1:82">
@@ -1961,7 +1961,7 @@
         <v>154</v>
       </c>
       <c r="J3">
-        <v>92.7</v>
+        <v>93.59999999999999</v>
       </c>
       <c r="K3">
         <v>1.5</v>
@@ -1970,16 +1970,16 @@
         <v>5</v>
       </c>
       <c r="M3">
-        <v>1.89</v>
+        <v>1.88</v>
       </c>
       <c r="N3">
-        <v>1.09</v>
+        <v>1.1</v>
       </c>
       <c r="O3">
         <v>0</v>
       </c>
       <c r="P3">
-        <v>5.1</v>
+        <v>4.6</v>
       </c>
       <c r="Q3">
         <v>0.6</v>
@@ -2003,13 +2003,13 @@
         <v>1</v>
       </c>
       <c r="X3">
-        <v>0.7819</v>
+        <v>0.7839</v>
       </c>
       <c r="Y3">
-        <v>0.32</v>
+        <v>0.38</v>
       </c>
       <c r="Z3">
-        <v>0.13</v>
+        <v>0.2</v>
       </c>
       <c r="AA3">
         <v>10.8</v>
@@ -2018,7 +2018,7 @@
         <v>86.59999999999999</v>
       </c>
       <c r="AC3">
-        <v>77.40000000000001</v>
+        <v>77.3</v>
       </c>
       <c r="AD3">
         <v>0.98</v>
@@ -2039,7 +2039,7 @@
         <v>84.3</v>
       </c>
       <c r="AJ3">
-        <v>84.40000000000001</v>
+        <v>84.5</v>
       </c>
       <c r="AK3">
         <v>69.59999999999999</v>
@@ -2069,7 +2069,7 @@
         <v>1266</v>
       </c>
       <c r="AT3">
-        <v>8.9</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="AU3">
         <v>17.3</v>
@@ -2078,25 +2078,25 @@
         <v>65</v>
       </c>
       <c r="AW3">
-        <v>224.3</v>
+        <v>224.7</v>
       </c>
       <c r="AX3">
         <v>7.3</v>
       </c>
       <c r="AY3">
-        <v>3.2</v>
+        <v>3.1</v>
       </c>
       <c r="AZ3">
-        <v>8.9</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="BA3">
-        <v>7.2</v>
+        <v>7.1</v>
       </c>
       <c r="BB3">
-        <v>2.8</v>
+        <v>2.7</v>
       </c>
       <c r="BC3">
-        <v>8.300000000000001</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="BD3">
         <v>4.9</v>
@@ -2135,22 +2135,22 @@
         <v>62</v>
       </c>
       <c r="BP3">
-        <v>81.7</v>
+        <v>81.59999999999999</v>
       </c>
       <c r="BQ3">
         <v>1.076</v>
       </c>
       <c r="BR3">
-        <v>83.3</v>
+        <v>83.2</v>
       </c>
       <c r="BS3">
-        <v>78.40000000000001</v>
+        <v>78.3</v>
       </c>
       <c r="BT3">
         <v>59.3</v>
       </c>
       <c r="BU3">
-        <v>57.7</v>
+        <v>57.6</v>
       </c>
       <c r="BV3">
         <v>53.3</v>
@@ -2177,7 +2177,7 @@
         <v>10</v>
       </c>
       <c r="CD3">
-        <v>8.300000000000001</v>
+        <v>8.199999999999999</v>
       </c>
     </row>
     <row r="4" spans="1:82">
@@ -2209,7 +2209,7 @@
         <v>154</v>
       </c>
       <c r="J4">
-        <v>92.7</v>
+        <v>93.59999999999999</v>
       </c>
       <c r="K4">
         <v>2.5</v>
@@ -2218,16 +2218,16 @@
         <v>5</v>
       </c>
       <c r="M4">
-        <v>2.02</v>
+        <v>2</v>
       </c>
       <c r="N4">
-        <v>1.23</v>
+        <v>1.38</v>
       </c>
       <c r="O4">
         <v>0</v>
       </c>
       <c r="P4">
-        <v>6.8</v>
+        <v>4.8</v>
       </c>
       <c r="Q4">
         <v>0.5</v>
@@ -2251,22 +2251,22 @@
         <v>1</v>
       </c>
       <c r="X4">
-        <v>0.6619</v>
+        <v>0.6636</v>
       </c>
       <c r="Y4">
-        <v>0.27</v>
+        <v>0.32</v>
       </c>
       <c r="Z4">
-        <v>0.11</v>
+        <v>0.17</v>
       </c>
       <c r="AA4">
-        <v>11.8</v>
+        <v>12.2</v>
       </c>
       <c r="AB4">
-        <v>86.7</v>
+        <v>86.09999999999999</v>
       </c>
       <c r="AC4">
-        <v>76.7</v>
+        <v>75.90000000000001</v>
       </c>
       <c r="AD4">
         <v>0.98</v>
@@ -2287,10 +2287,10 @@
         <v>82.40000000000001</v>
       </c>
       <c r="AJ4">
-        <v>82.09999999999999</v>
+        <v>82.40000000000001</v>
       </c>
       <c r="AK4">
-        <v>68.90000000000001</v>
+        <v>69</v>
       </c>
       <c r="AL4">
         <v>65.7</v>
@@ -2317,7 +2317,7 @@
         <v>1148</v>
       </c>
       <c r="AT4">
-        <v>9</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="AU4">
         <v>17.4</v>
@@ -2326,31 +2326,31 @@
         <v>65</v>
       </c>
       <c r="AW4">
-        <v>224.2</v>
+        <v>226.4</v>
       </c>
       <c r="AX4">
-        <v>7.5</v>
+        <v>7.1</v>
       </c>
       <c r="AY4">
-        <v>3.2</v>
+        <v>2.8</v>
       </c>
       <c r="AZ4">
-        <v>9</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="BA4">
-        <v>7.3</v>
+        <v>7</v>
       </c>
       <c r="BB4">
-        <v>2.9</v>
+        <v>2.5</v>
       </c>
       <c r="BC4">
-        <v>8.4</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="BD4">
-        <v>5</v>
+        <v>5.1</v>
       </c>
       <c r="BE4">
-        <v>6.6</v>
+        <v>6.2</v>
       </c>
       <c r="BF4">
         <v>0.8</v>
@@ -2383,22 +2383,22 @@
         <v>62</v>
       </c>
       <c r="BP4">
-        <v>80.8</v>
+        <v>80.09999999999999</v>
       </c>
       <c r="BQ4">
-        <v>1.074</v>
+        <v>1.072</v>
       </c>
       <c r="BR4">
-        <v>82.5</v>
+        <v>81.8</v>
       </c>
       <c r="BS4">
-        <v>77.5</v>
+        <v>76.7</v>
       </c>
       <c r="BT4">
-        <v>59.1</v>
+        <v>58.9</v>
       </c>
       <c r="BU4">
-        <v>57.2</v>
+        <v>57.1</v>
       </c>
       <c r="BV4">
         <v>55.9</v>
@@ -2410,7 +2410,7 @@
         <v>71</v>
       </c>
       <c r="BY4">
-        <v>14.6</v>
+        <v>15.3</v>
       </c>
       <c r="BZ4" t="s">
         <v>71</v>
@@ -2425,7 +2425,7 @@
         <v>10</v>
       </c>
       <c r="CD4">
-        <v>8.6</v>
+        <v>8.199999999999999</v>
       </c>
     </row>
     <row r="5" spans="1:82">
@@ -2457,7 +2457,7 @@
         <v>154</v>
       </c>
       <c r="J5">
-        <v>92.7</v>
+        <v>93.59999999999999</v>
       </c>
       <c r="K5">
         <v>3.5</v>
@@ -2466,19 +2466,19 @@
         <v>5</v>
       </c>
       <c r="M5">
-        <v>2.05</v>
+        <v>2.04</v>
       </c>
       <c r="N5">
-        <v>1.29</v>
+        <v>1.37</v>
       </c>
       <c r="O5">
         <v>0</v>
       </c>
       <c r="P5">
-        <v>8.800000000000001</v>
+        <v>7.2</v>
       </c>
       <c r="Q5">
-        <v>0.5</v>
+        <v>0.3</v>
       </c>
       <c r="R5">
         <v>100</v>
@@ -2499,22 +2499,22 @@
         <v>1</v>
       </c>
       <c r="X5">
-        <v>0.5603</v>
+        <v>0.5617</v>
       </c>
       <c r="Y5">
-        <v>0.23</v>
+        <v>0.27</v>
       </c>
       <c r="Z5">
-        <v>0.09</v>
+        <v>0.14</v>
       </c>
       <c r="AA5">
-        <v>12</v>
+        <v>12.3</v>
       </c>
       <c r="AB5">
-        <v>88.40000000000001</v>
+        <v>88</v>
       </c>
       <c r="AC5">
-        <v>76</v>
+        <v>75.40000000000001</v>
       </c>
       <c r="AD5">
         <v>0.98</v>
@@ -2535,7 +2535,7 @@
         <v>80.3</v>
       </c>
       <c r="AJ5">
-        <v>81</v>
+        <v>81.2</v>
       </c>
       <c r="AK5">
         <v>68.90000000000001</v>
@@ -2565,7 +2565,7 @@
         <v>1063</v>
       </c>
       <c r="AT5">
-        <v>9</v>
+        <v>8.9</v>
       </c>
       <c r="AU5">
         <v>17.2</v>
@@ -2574,31 +2574,31 @@
         <v>65</v>
       </c>
       <c r="AW5">
-        <v>225.3</v>
+        <v>227</v>
       </c>
       <c r="AX5">
-        <v>7.4</v>
+        <v>7.1</v>
       </c>
       <c r="AY5">
-        <v>3</v>
+        <v>2.7</v>
       </c>
       <c r="AZ5">
-        <v>9</v>
+        <v>8.9</v>
       </c>
       <c r="BA5">
-        <v>7.2</v>
+        <v>6.9</v>
       </c>
       <c r="BB5">
-        <v>2.7</v>
+        <v>2.5</v>
       </c>
       <c r="BC5">
-        <v>8.4</v>
+        <v>8.300000000000001</v>
       </c>
       <c r="BD5">
-        <v>5.1</v>
+        <v>5.2</v>
       </c>
       <c r="BE5">
-        <v>6.5</v>
+        <v>6.2</v>
       </c>
       <c r="BF5">
         <v>0.8</v>
@@ -2631,22 +2631,22 @@
         <v>62</v>
       </c>
       <c r="BP5">
-        <v>79.40000000000001</v>
+        <v>78.8</v>
       </c>
       <c r="BQ5">
-        <v>1.071</v>
+        <v>1.069</v>
       </c>
       <c r="BR5">
-        <v>81.09999999999999</v>
+        <v>80.7</v>
       </c>
       <c r="BS5">
-        <v>76</v>
+        <v>75.40000000000001</v>
       </c>
       <c r="BT5">
         <v>58.6</v>
       </c>
       <c r="BU5">
-        <v>56.7</v>
+        <v>56.6</v>
       </c>
       <c r="BV5">
         <v>58.4</v>
@@ -2658,7 +2658,7 @@
         <v>71</v>
       </c>
       <c r="BY5">
-        <v>11.3</v>
+        <v>11.9</v>
       </c>
       <c r="BZ5" t="s">
         <v>71</v>
@@ -2673,7 +2673,7 @@
         <v>10</v>
       </c>
       <c r="CD5">
-        <v>8.5</v>
+        <v>8.300000000000001</v>
       </c>
     </row>
   </sheetData>
@@ -2780,7 +2780,7 @@
         <v>67</v>
       </c>
       <c r="G2">
-        <v>87.2</v>
+        <v>87.09999999999999</v>
       </c>
       <c r="H2">
         <v>7</v>

</xml_diff>

<commit_message>
Update MLB weather 2026-07-14 05:08 PM PT
</commit_message>
<xml_diff>
--- a/mlb_weather_professional_v4_2026_07_14.xlsx
+++ b/mlb_weather_professional_v4_2026_07_14.xlsx
@@ -13,7 +13,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Game Summary'!$A$1:$BB$2</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Hourly Detail'!$A$1:$CD$5</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Hourly Detail'!$A$1:$CG$5</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'HR Weather'!$A$1:$Q$2</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="410" uniqueCount="163">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="420" uniqueCount="166">
   <si>
     <t>Date</t>
   </si>
@@ -215,19 +215,22 @@
     <t>Clear</t>
   </si>
   <si>
-    <t>🟢 8.7 mph Out to RF</t>
+    <t>🟢 4.0 mph Out to CF</t>
   </si>
   <si>
     <t>SW</t>
   </si>
   <si>
-    <t>FORECAST MODEL</t>
+    <t>4 mph, Out To CF</t>
+  </si>
+  <si>
+    <t>MLB RECORDED GAME WEATHER</t>
   </si>
   <si>
     <t>B+</t>
   </si>
   <si>
-    <t>Density 79 | Wind 65 | Temp 63 | Altitude 62 | Confidence 87%</t>
+    <t>Density 80 | Wind 62 | Temp 64 | Altitude 62 | Confidence 92%</t>
   </si>
   <si>
     <t>🟢 Good</t>
@@ -239,7 +242,7 @@
     <t>LOW</t>
   </si>
   <si>
-    <t>2026-07-14 04:32:21 PM PDT</t>
+    <t>2026-07-14 05:08:12 PM PDT</t>
   </si>
   <si>
     <t>Period</t>
@@ -461,6 +464,9 @@
     <t>Model Wind MPH</t>
   </si>
   <si>
+    <t>Official First Pitch Wind</t>
+  </si>
+  <si>
     <t>First Pitch</t>
   </si>
   <si>
@@ -482,7 +488,7 @@
     <t>11:00 PM EDT</t>
   </si>
   <si>
-    <t>2026-07-14 23:32:21 UTC</t>
+    <t>2026-07-15 00:08:12 UTC</t>
   </si>
   <si>
     <t>2026-07-14T21:58:43+00:00</t>
@@ -510,6 +516,9 @@
   </si>
   <si>
     <t>NEUTRAL</t>
+  </si>
+  <si>
+    <t>ACTUAL / RECORDED</t>
   </si>
 </sst>
 </file>
@@ -973,7 +982,7 @@
     <col min="14" max="15" width="28.7109375" customWidth="1"/>
     <col min="16" max="18" width="32.7109375" customWidth="1"/>
     <col min="19" max="19" width="24.7109375" customWidth="1"/>
-    <col min="20" max="20" width="18.7109375" customWidth="1"/>
+    <col min="20" max="20" width="27.7109375" customWidth="1"/>
     <col min="21" max="21" width="29.7109375" customWidth="1"/>
     <col min="22" max="22" width="22.7109375" customWidth="1"/>
     <col min="23" max="23" width="19.7109375" customWidth="1"/>
@@ -1202,43 +1211,46 @@
         <v>63</v>
       </c>
       <c r="K2">
-        <v>87.5</v>
+        <v>88</v>
       </c>
       <c r="L2">
-        <v>56.3</v>
+        <v>57.7</v>
       </c>
       <c r="M2" t="s">
         <v>64</v>
       </c>
       <c r="N2">
-        <v>9.4</v>
+        <v>4</v>
       </c>
       <c r="O2" t="s">
         <v>65</v>
       </c>
       <c r="P2">
-        <v>2.9</v>
+        <v>3.3</v>
       </c>
       <c r="Q2">
-        <v>7.5</v>
+        <v>4</v>
       </c>
       <c r="R2">
-        <v>8.699999999999999</v>
+        <v>3.3</v>
+      </c>
+      <c r="S2" t="s">
+        <v>66</v>
       </c>
       <c r="T2" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="U2">
         <v>0</v>
       </c>
       <c r="V2">
-        <v>61.9</v>
+        <v>61.6</v>
       </c>
       <c r="W2" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="X2" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="Y2">
         <v>7</v>
@@ -1247,19 +1259,19 @@
         <v>5</v>
       </c>
       <c r="AA2">
-        <v>3.6</v>
+        <v>3.5</v>
       </c>
       <c r="AB2">
-        <v>87.09999999999999</v>
+        <v>92</v>
       </c>
       <c r="AC2" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="AD2">
-        <v>6.5</v>
+        <v>5.3</v>
       </c>
       <c r="AE2">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="AF2">
         <v>100</v>
@@ -1268,40 +1280,40 @@
         <v>0</v>
       </c>
       <c r="AH2">
-        <v>4.8</v>
+        <v>4.7</v>
       </c>
       <c r="AI2">
-        <v>0.6</v>
+        <v>0.5</v>
       </c>
       <c r="AJ2">
-        <v>1.1552</v>
+        <v>1.1547</v>
       </c>
       <c r="AK2">
-        <v>1738</v>
+        <v>1751</v>
       </c>
       <c r="AL2">
         <v>1012.2</v>
       </c>
       <c r="AM2">
-        <v>69.2</v>
+        <v>69.3</v>
       </c>
       <c r="AN2">
-        <v>84.8</v>
+        <v>85</v>
       </c>
       <c r="AO2">
-        <v>61.6</v>
+        <v>61.8</v>
       </c>
       <c r="AP2" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="AQ2">
-        <v>16.4</v>
+        <v>15.6</v>
       </c>
       <c r="AR2">
-        <v>0.45</v>
+        <v>0</v>
       </c>
       <c r="AS2">
-        <v>0.24</v>
+        <v>0</v>
       </c>
       <c r="AT2">
         <v>0</v>
@@ -1310,22 +1322,22 @@
         <v>0</v>
       </c>
       <c r="AV2" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="AW2">
         <v>12</v>
       </c>
       <c r="AX2" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="AY2">
-        <v>16.2</v>
+        <v>15.5</v>
       </c>
       <c r="AZ2" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="BA2">
-        <v>93.59999999999999</v>
+        <v>129.5</v>
       </c>
       <c r="BB2">
         <v>5</v>
@@ -1364,7 +1376,7 @@
   <sheetPr>
     <tabColor rgb="FF5B9BD5"/>
   </sheetPr>
-  <dimension ref="A1:CD5"/>
+  <dimension ref="A1:CG5"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="28.7109375" customWidth="1"/>
@@ -1434,9 +1446,12 @@
     <col min="79" max="79" width="12.7109375" customWidth="1"/>
     <col min="80" max="81" width="14.7109375" customWidth="1"/>
     <col min="82" max="82" width="16.7109375" customWidth="1"/>
+    <col min="83" max="83" width="27.7109375" customWidth="1"/>
+    <col min="84" max="84" width="24.7109375" customWidth="1"/>
+    <col min="85" max="85" width="27.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:82" ht="34" customHeight="1">
+    <row r="1" spans="1:85" ht="34" customHeight="1">
       <c r="A1" s="1" t="s">
         <v>3</v>
       </c>
@@ -1450,220 +1465,220 @@
         <v>6</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="H1" s="1" t="s">
         <v>51</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="J1" s="1" t="s">
         <v>52</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="L1" s="1" t="s">
         <v>53</v>
       </c>
       <c r="M1" s="1" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="N1" s="1" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="O1" s="1" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="P1" s="1" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="Q1" s="1" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="R1" s="1" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="S1" s="1" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="T1" s="1" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="U1" s="1" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="V1" s="1" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="W1" s="1" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="X1" s="1" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="Y1" s="1" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="Z1" s="1" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="AA1" s="1" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="AB1" s="1" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="AC1" s="1" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="AD1" s="1" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="AE1" s="1" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="AF1" s="1" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="AG1" s="1" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="AH1" s="1" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="AI1" s="1" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="AJ1" s="1" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="AK1" s="1" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="AL1" s="1" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="AM1" s="1" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="AN1" s="1" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="AO1" s="1" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="AP1" s="1" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="AQ1" s="1" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="AR1" s="1" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="AS1" s="1" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="AT1" s="1" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="AU1" s="1" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="AV1" s="1" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="AW1" s="1" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="AX1" s="1" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="AY1" s="1" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="AZ1" s="1" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="BA1" s="1" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="BB1" s="1" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="BC1" s="1" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="BD1" s="1" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="BE1" s="1" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="BF1" s="1" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="BG1" s="1" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="BH1" s="1" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="BI1" s="1" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="BJ1" s="1" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="BK1" s="1" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="BL1" s="1" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="BM1" s="1" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="BN1" s="1" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="BO1" s="1" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="BP1" s="1" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="BQ1" s="1" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="BR1" s="1" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="BS1" s="1" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="BT1" s="1" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="BU1" s="1" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="BV1" s="1" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="BW1" s="1" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="BX1" s="1" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="BY1" s="1" t="s">
         <v>50</v>
@@ -1672,19 +1687,28 @@
         <v>49</v>
       </c>
       <c r="CA1" s="1" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="CB1" s="1" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="CC1" s="1" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="CD1" s="1" t="s">
-        <v>145</v>
+        <v>146</v>
+      </c>
+      <c r="CE1" s="1" t="s">
+        <v>147</v>
+      </c>
+      <c r="CF1" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="CG1" s="1" t="s">
+        <v>19</v>
       </c>
     </row>
-    <row r="2" spans="1:82">
+    <row r="2" spans="1:85">
       <c r="A2" t="s">
         <v>57</v>
       </c>
@@ -1698,43 +1722,43 @@
         <v>60</v>
       </c>
       <c r="E2" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="F2" t="s">
         <v>59</v>
       </c>
       <c r="G2" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="H2" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="I2" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="J2">
-        <v>93.59999999999999</v>
+        <v>129.5</v>
       </c>
       <c r="K2">
-        <v>0.5</v>
+        <v>0</v>
       </c>
       <c r="L2">
         <v>5</v>
       </c>
       <c r="M2">
-        <v>1.4</v>
+        <v>1.5</v>
       </c>
       <c r="N2">
-        <v>0.57</v>
+        <v>0.54</v>
       </c>
       <c r="O2">
         <v>0</v>
       </c>
       <c r="P2">
-        <v>4.4</v>
+        <v>4.3</v>
       </c>
       <c r="Q2">
-        <v>0.6</v>
+        <v>0.5</v>
       </c>
       <c r="R2">
         <v>100</v>
@@ -1743,34 +1767,34 @@
         <v>0</v>
       </c>
       <c r="T2" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="U2" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="V2" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="W2">
         <v>1</v>
       </c>
       <c r="X2">
-        <v>0.9261</v>
+        <v>0</v>
       </c>
       <c r="Y2">
-        <v>0.45</v>
+        <v>0</v>
       </c>
       <c r="Z2">
-        <v>0.24</v>
+        <v>0</v>
       </c>
       <c r="AA2">
-        <v>7.3</v>
+        <v>0</v>
       </c>
       <c r="AB2">
-        <v>87.8</v>
+        <v>100</v>
       </c>
       <c r="AC2">
-        <v>80.90000000000001</v>
+        <v>79.09999999999999</v>
       </c>
       <c r="AD2">
         <v>0.98</v>
@@ -1788,22 +1812,22 @@
         <v>63</v>
       </c>
       <c r="AI2">
-        <v>87.5</v>
+        <v>88</v>
       </c>
       <c r="AJ2">
-        <v>86</v>
+        <v>86.90000000000001</v>
       </c>
       <c r="AK2">
-        <v>69.09999999999999</v>
+        <v>69.8</v>
       </c>
       <c r="AL2">
-        <v>56.3</v>
+        <v>57.7</v>
       </c>
       <c r="AM2">
-        <v>1012.3</v>
+        <v>1012.2</v>
       </c>
       <c r="AN2">
-        <v>1014.5</v>
+        <v>1014.4</v>
       </c>
       <c r="AO2">
         <v>0</v>
@@ -1818,43 +1842,43 @@
         <v>50.6</v>
       </c>
       <c r="AS2">
-        <v>1274</v>
+        <v>1308</v>
       </c>
       <c r="AT2">
-        <v>9.4</v>
+        <v>4</v>
       </c>
       <c r="AU2">
-        <v>21.8</v>
+        <v>21.7</v>
       </c>
       <c r="AV2" t="s">
         <v>65</v>
       </c>
       <c r="AW2">
-        <v>224.6</v>
+        <v>224.9</v>
       </c>
       <c r="AX2">
         <v>7.7</v>
       </c>
       <c r="AY2">
+        <v>3.2</v>
+      </c>
+      <c r="AZ2">
+        <v>9.300000000000001</v>
+      </c>
+      <c r="BA2">
+        <v>4</v>
+      </c>
+      <c r="BB2">
         <v>3.3</v>
       </c>
-      <c r="AZ2">
-        <v>9.4</v>
-      </c>
-      <c r="BA2">
-        <v>7.5</v>
-      </c>
-      <c r="BB2">
-        <v>2.9</v>
-      </c>
       <c r="BC2">
-        <v>8.699999999999999</v>
+        <v>3.3</v>
       </c>
       <c r="BD2">
-        <v>5.2</v>
+        <v>0</v>
       </c>
       <c r="BE2">
-        <v>6.8</v>
+        <v>3.7</v>
       </c>
       <c r="BF2">
         <v>0.8</v>
@@ -1872,13 +1896,13 @@
         <v>0.09</v>
       </c>
       <c r="BK2">
-        <v>1.1496</v>
+        <v>1.1482</v>
       </c>
       <c r="BL2" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="BM2">
-        <v>1915</v>
+        <v>1949</v>
       </c>
       <c r="BN2" t="s">
         <v>61</v>
@@ -1887,52 +1911,61 @@
         <v>62</v>
       </c>
       <c r="BP2">
-        <v>85.2</v>
+        <v>79.09999999999999</v>
       </c>
       <c r="BQ2">
-        <v>1.084</v>
+        <v>1.07</v>
       </c>
       <c r="BR2">
-        <v>86.90000000000001</v>
+        <v>76.90000000000001</v>
       </c>
       <c r="BS2">
-        <v>81.7</v>
+        <v>76.90000000000001</v>
       </c>
       <c r="BT2">
-        <v>60.3</v>
+        <v>56.2</v>
       </c>
       <c r="BU2">
-        <v>58.5</v>
+        <v>57.3</v>
       </c>
       <c r="BV2">
-        <v>46.6</v>
+        <v>45.5</v>
       </c>
       <c r="BW2">
         <v>12</v>
       </c>
       <c r="BX2" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="BY2">
-        <v>16.2</v>
+        <v>0</v>
       </c>
       <c r="BZ2" t="s">
-        <v>71</v>
+        <v>165</v>
       </c>
       <c r="CA2">
         <v>91</v>
       </c>
       <c r="CB2">
-        <v>83.8</v>
+        <v>83.7</v>
       </c>
       <c r="CC2">
         <v>10</v>
       </c>
       <c r="CD2">
-        <v>9.199999999999999</v>
+        <v>9.1</v>
+      </c>
+      <c r="CE2" t="s">
+        <v>64</v>
+      </c>
+      <c r="CF2" t="s">
+        <v>66</v>
+      </c>
+      <c r="CG2" t="s">
+        <v>67</v>
       </c>
     </row>
-    <row r="3" spans="1:82">
+    <row r="3" spans="1:85">
       <c r="A3" t="s">
         <v>57</v>
       </c>
@@ -1946,25 +1979,25 @@
         <v>60</v>
       </c>
       <c r="E3" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="F3" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="G3" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="H3" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="I3" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="J3">
-        <v>93.59999999999999</v>
+        <v>129.5</v>
       </c>
       <c r="K3">
-        <v>1.5</v>
+        <v>0.9</v>
       </c>
       <c r="L3">
         <v>5</v>
@@ -1973,13 +2006,13 @@
         <v>1.88</v>
       </c>
       <c r="N3">
-        <v>1.1</v>
+        <v>1.11</v>
       </c>
       <c r="O3">
         <v>0</v>
       </c>
       <c r="P3">
-        <v>4.6</v>
+        <v>4.4</v>
       </c>
       <c r="Q3">
         <v>0.6</v>
@@ -1991,25 +2024,25 @@
         <v>0</v>
       </c>
       <c r="T3" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="U3" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="V3" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="W3">
         <v>1</v>
       </c>
       <c r="X3">
-        <v>0.7839</v>
+        <v>0.866</v>
       </c>
       <c r="Y3">
-        <v>0.38</v>
+        <v>0.37</v>
       </c>
       <c r="Z3">
-        <v>0.2</v>
+        <v>0.17</v>
       </c>
       <c r="AA3">
         <v>10.8</v>
@@ -2048,10 +2081,10 @@
         <v>63</v>
       </c>
       <c r="AM3">
-        <v>1012</v>
+        <v>1012.3</v>
       </c>
       <c r="AN3">
-        <v>1014.3</v>
+        <v>1014.6</v>
       </c>
       <c r="AO3">
         <v>0</v>
@@ -2066,19 +2099,19 @@
         <v>42.4</v>
       </c>
       <c r="AS3">
-        <v>1266</v>
+        <v>1226</v>
       </c>
       <c r="AT3">
         <v>8.800000000000001</v>
       </c>
       <c r="AU3">
-        <v>17.3</v>
+        <v>17.4</v>
       </c>
       <c r="AV3" t="s">
         <v>65</v>
       </c>
       <c r="AW3">
-        <v>224.7</v>
+        <v>224.8</v>
       </c>
       <c r="AX3">
         <v>7.3</v>
@@ -2120,13 +2153,13 @@
         <v>0.09</v>
       </c>
       <c r="BK3">
-        <v>1.1559</v>
+        <v>1.1563</v>
       </c>
       <c r="BL3" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="BM3">
-        <v>1709</v>
+        <v>1698</v>
       </c>
       <c r="BN3" t="s">
         <v>61</v>
@@ -2135,16 +2168,16 @@
         <v>62</v>
       </c>
       <c r="BP3">
-        <v>81.59999999999999</v>
+        <v>81.5</v>
       </c>
       <c r="BQ3">
         <v>1.076</v>
       </c>
       <c r="BR3">
-        <v>83.2</v>
+        <v>83.09999999999999</v>
       </c>
       <c r="BS3">
-        <v>78.3</v>
+        <v>78.2</v>
       </c>
       <c r="BT3">
         <v>59.3</v>
@@ -2159,13 +2192,13 @@
         <v>12</v>
       </c>
       <c r="BX3" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="BY3">
         <v>15.5</v>
       </c>
       <c r="BZ3" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="CA3">
         <v>87</v>
@@ -2180,7 +2213,7 @@
         <v>8.199999999999999</v>
       </c>
     </row>
-    <row r="4" spans="1:82">
+    <row r="4" spans="1:85">
       <c r="A4" t="s">
         <v>57</v>
       </c>
@@ -2194,31 +2227,31 @@
         <v>60</v>
       </c>
       <c r="E4" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="F4" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="G4" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="H4" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="I4" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="J4">
-        <v>93.59999999999999</v>
+        <v>129.5</v>
       </c>
       <c r="K4">
-        <v>2.5</v>
+        <v>1.9</v>
       </c>
       <c r="L4">
         <v>5</v>
       </c>
       <c r="M4">
-        <v>2</v>
+        <v>2.01</v>
       </c>
       <c r="N4">
         <v>1.38</v>
@@ -2227,7 +2260,7 @@
         <v>0</v>
       </c>
       <c r="P4">
-        <v>4.8</v>
+        <v>4.7</v>
       </c>
       <c r="Q4">
         <v>0.5</v>
@@ -2239,25 +2272,25 @@
         <v>0</v>
       </c>
       <c r="T4" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="U4" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="V4" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="W4">
         <v>1</v>
       </c>
       <c r="X4">
-        <v>0.6636</v>
+        <v>0.7331</v>
       </c>
       <c r="Y4">
-        <v>0.32</v>
+        <v>0.31</v>
       </c>
       <c r="Z4">
-        <v>0.17</v>
+        <v>0.14</v>
       </c>
       <c r="AA4">
         <v>12.2</v>
@@ -2287,19 +2320,19 @@
         <v>82.40000000000001</v>
       </c>
       <c r="AJ4">
-        <v>82.40000000000001</v>
+        <v>82</v>
       </c>
       <c r="AK4">
-        <v>69</v>
+        <v>68.7</v>
       </c>
       <c r="AL4">
-        <v>65.7</v>
+        <v>65</v>
       </c>
       <c r="AM4">
-        <v>1012.3</v>
+        <v>1012</v>
       </c>
       <c r="AN4">
-        <v>1014.6</v>
+        <v>1014.3</v>
       </c>
       <c r="AO4">
         <v>0</v>
@@ -2314,7 +2347,7 @@
         <v>40.6</v>
       </c>
       <c r="AS4">
-        <v>1148</v>
+        <v>889</v>
       </c>
       <c r="AT4">
         <v>8.800000000000001</v>
@@ -2326,7 +2359,7 @@
         <v>65</v>
       </c>
       <c r="AW4">
-        <v>226.4</v>
+        <v>226.5</v>
       </c>
       <c r="AX4">
         <v>7.1</v>
@@ -2368,13 +2401,13 @@
         <v>0.09</v>
       </c>
       <c r="BK4">
-        <v>1.1606</v>
+        <v>1.1604</v>
       </c>
       <c r="BL4" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="BM4">
-        <v>1573</v>
+        <v>1583</v>
       </c>
       <c r="BN4" t="s">
         <v>61</v>
@@ -2389,7 +2422,7 @@
         <v>1.072</v>
       </c>
       <c r="BR4">
-        <v>81.8</v>
+        <v>81.90000000000001</v>
       </c>
       <c r="BS4">
         <v>76.7</v>
@@ -2398,22 +2431,22 @@
         <v>58.9</v>
       </c>
       <c r="BU4">
-        <v>57.1</v>
+        <v>57</v>
       </c>
       <c r="BV4">
-        <v>55.9</v>
+        <v>56.1</v>
       </c>
       <c r="BW4">
-        <v>11.5</v>
+        <v>8.9</v>
       </c>
       <c r="BX4" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="BY4">
         <v>15.3</v>
       </c>
       <c r="BZ4" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="CA4">
         <v>85</v>
@@ -2428,7 +2461,7 @@
         <v>8.199999999999999</v>
       </c>
     </row>
-    <row r="5" spans="1:82">
+    <row r="5" spans="1:85">
       <c r="A5" t="s">
         <v>57</v>
       </c>
@@ -2442,25 +2475,25 @@
         <v>60</v>
       </c>
       <c r="E5" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="F5" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="G5" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="H5" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="I5" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="J5">
-        <v>93.59999999999999</v>
+        <v>129.5</v>
       </c>
       <c r="K5">
-        <v>3.5</v>
+        <v>2.9</v>
       </c>
       <c r="L5">
         <v>5</v>
@@ -2475,7 +2508,7 @@
         <v>0</v>
       </c>
       <c r="P5">
-        <v>7.2</v>
+        <v>7.1</v>
       </c>
       <c r="Q5">
         <v>0.3</v>
@@ -2487,25 +2520,25 @@
         <v>0</v>
       </c>
       <c r="T5" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="U5" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="V5" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="W5">
         <v>1</v>
       </c>
       <c r="X5">
-        <v>0.5617</v>
+        <v>0.6205000000000001</v>
       </c>
       <c r="Y5">
-        <v>0.27</v>
+        <v>0.26</v>
       </c>
       <c r="Z5">
-        <v>0.14</v>
+        <v>0.12</v>
       </c>
       <c r="AA5">
         <v>12.3</v>
@@ -2514,7 +2547,7 @@
         <v>88</v>
       </c>
       <c r="AC5">
-        <v>75.40000000000001</v>
+        <v>75.3</v>
       </c>
       <c r="AD5">
         <v>0.98</v>
@@ -2535,22 +2568,22 @@
         <v>80.3</v>
       </c>
       <c r="AJ5">
-        <v>81.2</v>
+        <v>80</v>
       </c>
       <c r="AK5">
-        <v>68.90000000000001</v>
+        <v>68</v>
       </c>
       <c r="AL5">
-        <v>69.90000000000001</v>
+        <v>67.90000000000001</v>
       </c>
       <c r="AM5">
-        <v>1012.1</v>
+        <v>1012</v>
       </c>
       <c r="AN5">
         <v>1014.3</v>
       </c>
       <c r="AO5">
-        <v>1.1</v>
+        <v>0</v>
       </c>
       <c r="AP5">
         <v>0</v>
@@ -2562,7 +2595,7 @@
         <v>40.8</v>
       </c>
       <c r="AS5">
-        <v>1063</v>
+        <v>591</v>
       </c>
       <c r="AT5">
         <v>8.9</v>
@@ -2574,7 +2607,7 @@
         <v>65</v>
       </c>
       <c r="AW5">
-        <v>227</v>
+        <v>227.1</v>
       </c>
       <c r="AX5">
         <v>7.1</v>
@@ -2589,7 +2622,7 @@
         <v>6.9</v>
       </c>
       <c r="BB5">
-        <v>2.5</v>
+        <v>2.4</v>
       </c>
       <c r="BC5">
         <v>8.300000000000001</v>
@@ -2616,13 +2649,13 @@
         <v>0.09</v>
       </c>
       <c r="BK5">
-        <v>1.1646</v>
+        <v>1.1649</v>
       </c>
       <c r="BL5" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="BM5">
-        <v>1449</v>
+        <v>1451</v>
       </c>
       <c r="BN5" t="s">
         <v>61</v>
@@ -2637,7 +2670,7 @@
         <v>1.069</v>
       </c>
       <c r="BR5">
-        <v>80.7</v>
+        <v>80.59999999999999</v>
       </c>
       <c r="BS5">
         <v>75.40000000000001</v>
@@ -2646,22 +2679,22 @@
         <v>58.6</v>
       </c>
       <c r="BU5">
-        <v>56.6</v>
+        <v>56.5</v>
       </c>
       <c r="BV5">
-        <v>58.4</v>
+        <v>59.2</v>
       </c>
       <c r="BW5">
-        <v>10.6</v>
+        <v>5.9</v>
       </c>
       <c r="BX5" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="BY5">
-        <v>11.9</v>
+        <v>11.8</v>
       </c>
       <c r="BZ5" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="CA5">
         <v>82</v>
@@ -2677,7 +2710,7 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:CD5"/>
+  <autoFilter ref="A1:CG5"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
@@ -2774,13 +2807,13 @@
         <v>60</v>
       </c>
       <c r="E2">
-        <v>61.9</v>
+        <v>61.6</v>
       </c>
       <c r="F2" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="G2">
-        <v>87.09999999999999</v>
+        <v>92</v>
       </c>
       <c r="H2">
         <v>7</v>
@@ -2789,25 +2822,25 @@
         <v>5</v>
       </c>
       <c r="J2">
-        <v>3.6</v>
+        <v>3.5</v>
       </c>
       <c r="K2">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="L2" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="M2">
-        <v>84.8</v>
+        <v>85</v>
       </c>
       <c r="N2">
-        <v>1738</v>
+        <v>1751</v>
       </c>
       <c r="O2" t="s">
         <v>61</v>
       </c>
       <c r="P2" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="Q2">
         <v>5</v>

</xml_diff>

<commit_message>
Update MLB weather 2026-07-14 06:01 PM PT
</commit_message>
<xml_diff>
--- a/mlb_weather_professional_v4_2026_07_14.xlsx
+++ b/mlb_weather_professional_v4_2026_07_14.xlsx
@@ -230,7 +230,7 @@
     <t>B+</t>
   </si>
   <si>
-    <t>Density 80 | Wind 62 | Temp 64 | Altitude 62 | Confidence 92%</t>
+    <t>Density 80 | Wind 62 | Temp 64 | Altitude 62 | Confidence 93%</t>
   </si>
   <si>
     <t>🟢 Good</t>
@@ -242,7 +242,7 @@
     <t>LOW</t>
   </si>
   <si>
-    <t>2026-07-14 05:08:12 PM PDT</t>
+    <t>2026-07-14 06:01:45 PM PDT</t>
   </si>
   <si>
     <t>Period</t>
@@ -488,7 +488,7 @@
     <t>11:00 PM EDT</t>
   </si>
   <si>
-    <t>2026-07-15 00:08:12 UTC</t>
+    <t>2026-07-15 01:01:45 UTC</t>
   </si>
   <si>
     <t>2026-07-14T21:58:43+00:00</t>
@@ -1214,7 +1214,7 @@
         <v>88</v>
       </c>
       <c r="L2">
-        <v>57.7</v>
+        <v>59.7</v>
       </c>
       <c r="M2" t="s">
         <v>64</v>
@@ -1244,7 +1244,7 @@
         <v>0</v>
       </c>
       <c r="V2">
-        <v>61.6</v>
+        <v>61.7</v>
       </c>
       <c r="W2" t="s">
         <v>68</v>
@@ -1262,13 +1262,13 @@
         <v>3.5</v>
       </c>
       <c r="AB2">
-        <v>92</v>
+        <v>93.09999999999999</v>
       </c>
       <c r="AC2" t="s">
         <v>70</v>
       </c>
       <c r="AD2">
-        <v>5.3</v>
+        <v>5.2</v>
       </c>
       <c r="AE2">
         <v>4</v>
@@ -1280,34 +1280,34 @@
         <v>0</v>
       </c>
       <c r="AH2">
-        <v>4.7</v>
+        <v>4</v>
       </c>
       <c r="AI2">
-        <v>0.5</v>
+        <v>0.6</v>
       </c>
       <c r="AJ2">
-        <v>1.1547</v>
+        <v>1.1538</v>
       </c>
       <c r="AK2">
-        <v>1751</v>
+        <v>1771</v>
       </c>
       <c r="AL2">
-        <v>1012.2</v>
+        <v>1012</v>
       </c>
       <c r="AM2">
-        <v>69.3</v>
+        <v>70</v>
       </c>
       <c r="AN2">
-        <v>85</v>
+        <v>85.2</v>
       </c>
       <c r="AO2">
-        <v>61.8</v>
+        <v>63.4</v>
       </c>
       <c r="AP2" t="s">
         <v>71</v>
       </c>
       <c r="AQ2">
-        <v>15.6</v>
+        <v>16.3</v>
       </c>
       <c r="AR2">
         <v>0</v>
@@ -1331,13 +1331,13 @@
         <v>72</v>
       </c>
       <c r="AY2">
-        <v>15.5</v>
+        <v>14.6</v>
       </c>
       <c r="AZ2" t="s">
         <v>73</v>
       </c>
       <c r="BA2">
-        <v>129.5</v>
+        <v>183</v>
       </c>
       <c r="BB2">
         <v>5</v>
@@ -1737,7 +1737,7 @@
         <v>156</v>
       </c>
       <c r="J2">
-        <v>129.5</v>
+        <v>183</v>
       </c>
       <c r="K2">
         <v>0</v>
@@ -1746,16 +1746,16 @@
         <v>5</v>
       </c>
       <c r="M2">
-        <v>1.5</v>
+        <v>1.2</v>
       </c>
       <c r="N2">
-        <v>0.54</v>
+        <v>0.5600000000000001</v>
       </c>
       <c r="O2">
         <v>0</v>
       </c>
       <c r="P2">
-        <v>4.3</v>
+        <v>3.8</v>
       </c>
       <c r="Q2">
         <v>0.5</v>
@@ -1794,7 +1794,7 @@
         <v>100</v>
       </c>
       <c r="AC2">
-        <v>79.09999999999999</v>
+        <v>79.2</v>
       </c>
       <c r="AD2">
         <v>0.98</v>
@@ -1815,19 +1815,19 @@
         <v>88</v>
       </c>
       <c r="AJ2">
-        <v>86.90000000000001</v>
+        <v>88.09999999999999</v>
       </c>
       <c r="AK2">
-        <v>69.8</v>
+        <v>69.90000000000001</v>
       </c>
       <c r="AL2">
-        <v>57.7</v>
+        <v>59.7</v>
       </c>
       <c r="AM2">
-        <v>1012.2</v>
+        <v>1011.9</v>
       </c>
       <c r="AN2">
-        <v>1014.4</v>
+        <v>1014.1</v>
       </c>
       <c r="AO2">
         <v>0</v>
@@ -1839,22 +1839,22 @@
         <v>0</v>
       </c>
       <c r="AR2">
-        <v>50.6</v>
+        <v>49.3</v>
       </c>
       <c r="AS2">
-        <v>1308</v>
+        <v>1482</v>
       </c>
       <c r="AT2">
         <v>4</v>
       </c>
       <c r="AU2">
-        <v>21.7</v>
+        <v>21.6</v>
       </c>
       <c r="AV2" t="s">
         <v>65</v>
       </c>
       <c r="AW2">
-        <v>224.9</v>
+        <v>225.2</v>
       </c>
       <c r="AX2">
         <v>7.7</v>
@@ -1863,7 +1863,7 @@
         <v>3.2</v>
       </c>
       <c r="AZ2">
-        <v>9.300000000000001</v>
+        <v>9.4</v>
       </c>
       <c r="BA2">
         <v>4</v>
@@ -1896,13 +1896,13 @@
         <v>0.09</v>
       </c>
       <c r="BK2">
-        <v>1.1482</v>
+        <v>1.1478</v>
       </c>
       <c r="BL2" t="s">
         <v>163</v>
       </c>
       <c r="BM2">
-        <v>1949</v>
+        <v>1960</v>
       </c>
       <c r="BN2" t="s">
         <v>61</v>
@@ -1911,7 +1911,7 @@
         <v>62</v>
       </c>
       <c r="BP2">
-        <v>79.09999999999999</v>
+        <v>79.2</v>
       </c>
       <c r="BQ2">
         <v>1.07</v>
@@ -1944,16 +1944,16 @@
         <v>165</v>
       </c>
       <c r="CA2">
-        <v>91</v>
+        <v>87</v>
       </c>
       <c r="CB2">
-        <v>83.7</v>
+        <v>84</v>
       </c>
       <c r="CC2">
         <v>10</v>
       </c>
       <c r="CD2">
-        <v>9.1</v>
+        <v>9.199999999999999</v>
       </c>
       <c r="CE2" t="s">
         <v>64</v>
@@ -1994,19 +1994,19 @@
         <v>156</v>
       </c>
       <c r="J3">
-        <v>129.5</v>
+        <v>183</v>
       </c>
       <c r="K3">
-        <v>0.9</v>
+        <v>0</v>
       </c>
       <c r="L3">
         <v>5</v>
       </c>
       <c r="M3">
-        <v>1.88</v>
+        <v>1.72</v>
       </c>
       <c r="N3">
-        <v>1.11</v>
+        <v>1.07</v>
       </c>
       <c r="O3">
         <v>0</v>
@@ -2015,7 +2015,7 @@
         <v>4.4</v>
       </c>
       <c r="Q3">
-        <v>0.6</v>
+        <v>0.7</v>
       </c>
       <c r="R3">
         <v>100</v>
@@ -2036,22 +2036,22 @@
         <v>1</v>
       </c>
       <c r="X3">
-        <v>0.866</v>
+        <v>0</v>
       </c>
       <c r="Y3">
-        <v>0.37</v>
+        <v>0</v>
       </c>
       <c r="Z3">
-        <v>0.17</v>
+        <v>0</v>
       </c>
       <c r="AA3">
-        <v>10.8</v>
+        <v>10.1</v>
       </c>
       <c r="AB3">
-        <v>86.59999999999999</v>
+        <v>87.5</v>
       </c>
       <c r="AC3">
-        <v>77.3</v>
+        <v>77.90000000000001</v>
       </c>
       <c r="AD3">
         <v>0.98</v>
@@ -2069,22 +2069,22 @@
         <v>63</v>
       </c>
       <c r="AI3">
-        <v>84.3</v>
+        <v>84.40000000000001</v>
       </c>
       <c r="AJ3">
-        <v>84.5</v>
+        <v>86</v>
       </c>
       <c r="AK3">
-        <v>69.59999999999999</v>
+        <v>70.40000000000001</v>
       </c>
       <c r="AL3">
-        <v>63</v>
+        <v>64.3</v>
       </c>
       <c r="AM3">
-        <v>1012.3</v>
+        <v>1012</v>
       </c>
       <c r="AN3">
-        <v>1014.6</v>
+        <v>1014.2</v>
       </c>
       <c r="AO3">
         <v>0</v>
@@ -2096,22 +2096,22 @@
         <v>0</v>
       </c>
       <c r="AR3">
-        <v>42.4</v>
+        <v>37.7</v>
       </c>
       <c r="AS3">
-        <v>1226</v>
+        <v>1614</v>
       </c>
       <c r="AT3">
-        <v>8.800000000000001</v>
+        <v>9</v>
       </c>
       <c r="AU3">
-        <v>17.4</v>
+        <v>17.7</v>
       </c>
       <c r="AV3" t="s">
         <v>65</v>
       </c>
       <c r="AW3">
-        <v>224.8</v>
+        <v>224.9</v>
       </c>
       <c r="AX3">
         <v>7.3</v>
@@ -2120,22 +2120,22 @@
         <v>3.1</v>
       </c>
       <c r="AZ3">
-        <v>8.800000000000001</v>
+        <v>9</v>
       </c>
       <c r="BA3">
-        <v>7.1</v>
+        <v>7.2</v>
       </c>
       <c r="BB3">
-        <v>2.7</v>
+        <v>2.8</v>
       </c>
       <c r="BC3">
-        <v>8.199999999999999</v>
+        <v>8.300000000000001</v>
       </c>
       <c r="BD3">
-        <v>4.9</v>
+        <v>5</v>
       </c>
       <c r="BE3">
-        <v>6.4</v>
+        <v>6.5</v>
       </c>
       <c r="BF3">
         <v>0.8</v>
@@ -2153,13 +2153,13 @@
         <v>0.09</v>
       </c>
       <c r="BK3">
-        <v>1.1563</v>
+        <v>1.1553</v>
       </c>
       <c r="BL3" t="s">
         <v>163</v>
       </c>
       <c r="BM3">
-        <v>1698</v>
+        <v>1720</v>
       </c>
       <c r="BN3" t="s">
         <v>61</v>
@@ -2168,25 +2168,25 @@
         <v>62</v>
       </c>
       <c r="BP3">
-        <v>81.5</v>
+        <v>81.90000000000001</v>
       </c>
       <c r="BQ3">
-        <v>1.076</v>
+        <v>1.077</v>
       </c>
       <c r="BR3">
-        <v>83.09999999999999</v>
+        <v>83.59999999999999</v>
       </c>
       <c r="BS3">
-        <v>78.2</v>
+        <v>78.59999999999999</v>
       </c>
       <c r="BT3">
-        <v>59.3</v>
+        <v>59.4</v>
       </c>
       <c r="BU3">
-        <v>57.6</v>
+        <v>57.8</v>
       </c>
       <c r="BV3">
-        <v>53.3</v>
+        <v>52.2</v>
       </c>
       <c r="BW3">
         <v>12</v>
@@ -2195,7 +2195,7 @@
         <v>72</v>
       </c>
       <c r="BY3">
-        <v>15.5</v>
+        <v>14.6</v>
       </c>
       <c r="BZ3" t="s">
         <v>72</v>
@@ -2204,13 +2204,13 @@
         <v>87</v>
       </c>
       <c r="CB3">
-        <v>81.09999999999999</v>
+        <v>81.3</v>
       </c>
       <c r="CC3">
         <v>10</v>
       </c>
       <c r="CD3">
-        <v>8.199999999999999</v>
+        <v>8.4</v>
       </c>
     </row>
     <row r="4" spans="1:85">
@@ -2242,28 +2242,28 @@
         <v>156</v>
       </c>
       <c r="J4">
-        <v>129.5</v>
+        <v>183</v>
       </c>
       <c r="K4">
-        <v>1.9</v>
+        <v>1</v>
       </c>
       <c r="L4">
         <v>5</v>
       </c>
       <c r="M4">
-        <v>2.01</v>
+        <v>1.37</v>
       </c>
       <c r="N4">
-        <v>1.38</v>
+        <v>1.3</v>
       </c>
       <c r="O4">
         <v>0</v>
       </c>
       <c r="P4">
-        <v>4.7</v>
+        <v>3.3</v>
       </c>
       <c r="Q4">
-        <v>0.5</v>
+        <v>0.6</v>
       </c>
       <c r="R4">
         <v>100</v>
@@ -2284,22 +2284,22 @@
         <v>1</v>
       </c>
       <c r="X4">
-        <v>0.7331</v>
+        <v>0.8506</v>
       </c>
       <c r="Y4">
-        <v>0.31</v>
+        <v>0.02</v>
       </c>
       <c r="Z4">
-        <v>0.14</v>
+        <v>0.01</v>
       </c>
       <c r="AA4">
-        <v>12.2</v>
+        <v>9.4</v>
       </c>
       <c r="AB4">
-        <v>86.09999999999999</v>
+        <v>88.5</v>
       </c>
       <c r="AC4">
-        <v>75.90000000000001</v>
+        <v>76.5</v>
       </c>
       <c r="AD4">
         <v>0.98</v>
@@ -2317,16 +2317,16 @@
         <v>63</v>
       </c>
       <c r="AI4">
-        <v>82.40000000000001</v>
+        <v>82.8</v>
       </c>
       <c r="AJ4">
-        <v>82</v>
+        <v>84.8</v>
       </c>
       <c r="AK4">
-        <v>68.7</v>
+        <v>69.7</v>
       </c>
       <c r="AL4">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="AM4">
         <v>1012</v>
@@ -2344,46 +2344,46 @@
         <v>0</v>
       </c>
       <c r="AR4">
-        <v>40.6</v>
+        <v>37.1</v>
       </c>
       <c r="AS4">
-        <v>889</v>
+        <v>1407</v>
       </c>
       <c r="AT4">
-        <v>8.800000000000001</v>
+        <v>8.9</v>
       </c>
       <c r="AU4">
-        <v>17.4</v>
+        <v>17.1</v>
       </c>
       <c r="AV4" t="s">
         <v>65</v>
       </c>
       <c r="AW4">
-        <v>226.5</v>
+        <v>229.9</v>
       </c>
       <c r="AX4">
-        <v>7.1</v>
+        <v>6.9</v>
       </c>
       <c r="AY4">
-        <v>2.8</v>
+        <v>2.3</v>
       </c>
       <c r="AZ4">
-        <v>8.800000000000001</v>
+        <v>8.9</v>
       </c>
       <c r="BA4">
-        <v>7</v>
+        <v>6.7</v>
       </c>
       <c r="BB4">
-        <v>2.5</v>
+        <v>2.1</v>
       </c>
       <c r="BC4">
-        <v>8.199999999999999</v>
+        <v>8.300000000000001</v>
       </c>
       <c r="BD4">
-        <v>5.1</v>
+        <v>5.6</v>
       </c>
       <c r="BE4">
-        <v>6.2</v>
+        <v>6</v>
       </c>
       <c r="BF4">
         <v>0.8</v>
@@ -2401,13 +2401,13 @@
         <v>0.09</v>
       </c>
       <c r="BK4">
-        <v>1.1604</v>
+        <v>1.159</v>
       </c>
       <c r="BL4" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="BM4">
-        <v>1583</v>
+        <v>1613</v>
       </c>
       <c r="BN4" t="s">
         <v>61</v>
@@ -2416,7 +2416,7 @@
         <v>62</v>
       </c>
       <c r="BP4">
-        <v>80.09999999999999</v>
+        <v>79.90000000000001</v>
       </c>
       <c r="BQ4">
         <v>1.072</v>
@@ -2425,25 +2425,25 @@
         <v>81.90000000000001</v>
       </c>
       <c r="BS4">
-        <v>76.7</v>
+        <v>76.3</v>
       </c>
       <c r="BT4">
-        <v>58.9</v>
+        <v>59.1</v>
       </c>
       <c r="BU4">
-        <v>57</v>
+        <v>57.2</v>
       </c>
       <c r="BV4">
-        <v>56.1</v>
+        <v>55</v>
       </c>
       <c r="BW4">
-        <v>8.9</v>
+        <v>12</v>
       </c>
       <c r="BX4" t="s">
         <v>72</v>
       </c>
       <c r="BY4">
-        <v>15.3</v>
+        <v>13.2</v>
       </c>
       <c r="BZ4" t="s">
         <v>72</v>
@@ -2452,13 +2452,13 @@
         <v>85</v>
       </c>
       <c r="CB4">
-        <v>79.2</v>
+        <v>80</v>
       </c>
       <c r="CC4">
         <v>10</v>
       </c>
       <c r="CD4">
-        <v>8.199999999999999</v>
+        <v>8.4</v>
       </c>
     </row>
     <row r="5" spans="1:85">
@@ -2490,28 +2490,28 @@
         <v>156</v>
       </c>
       <c r="J5">
-        <v>129.5</v>
+        <v>183</v>
       </c>
       <c r="K5">
-        <v>2.9</v>
+        <v>2</v>
       </c>
       <c r="L5">
         <v>5</v>
       </c>
       <c r="M5">
-        <v>2.04</v>
+        <v>1.1</v>
       </c>
       <c r="N5">
-        <v>1.37</v>
+        <v>1.39</v>
       </c>
       <c r="O5">
         <v>0</v>
       </c>
       <c r="P5">
-        <v>7.1</v>
+        <v>5</v>
       </c>
       <c r="Q5">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
       <c r="R5">
         <v>100</v>
@@ -2532,22 +2532,22 @@
         <v>1</v>
       </c>
       <c r="X5">
-        <v>0.6205000000000001</v>
+        <v>0.72</v>
       </c>
       <c r="Y5">
-        <v>0.26</v>
+        <v>0.02</v>
       </c>
       <c r="Z5">
-        <v>0.12</v>
+        <v>0.01</v>
       </c>
       <c r="AA5">
-        <v>12.3</v>
+        <v>8.5</v>
       </c>
       <c r="AB5">
-        <v>88</v>
+        <v>91</v>
       </c>
       <c r="AC5">
-        <v>75.3</v>
+        <v>75.90000000000001</v>
       </c>
       <c r="AD5">
         <v>0.98</v>
@@ -2565,22 +2565,22 @@
         <v>63</v>
       </c>
       <c r="AI5">
-        <v>80.3</v>
+        <v>81</v>
       </c>
       <c r="AJ5">
-        <v>80</v>
+        <v>84.5</v>
       </c>
       <c r="AK5">
-        <v>68</v>
+        <v>69.7</v>
       </c>
       <c r="AL5">
-        <v>67.90000000000001</v>
+        <v>69.90000000000001</v>
       </c>
       <c r="AM5">
-        <v>1012</v>
+        <v>1012.3</v>
       </c>
       <c r="AN5">
-        <v>1014.3</v>
+        <v>1014.6</v>
       </c>
       <c r="AO5">
         <v>0</v>
@@ -2592,46 +2592,46 @@
         <v>0</v>
       </c>
       <c r="AR5">
-        <v>40.8</v>
+        <v>35.1</v>
       </c>
       <c r="AS5">
-        <v>591</v>
+        <v>1344</v>
       </c>
       <c r="AT5">
         <v>8.9</v>
       </c>
       <c r="AU5">
-        <v>17.2</v>
+        <v>16.7</v>
       </c>
       <c r="AV5" t="s">
         <v>65</v>
       </c>
       <c r="AW5">
-        <v>227.1</v>
+        <v>230.3</v>
       </c>
       <c r="AX5">
-        <v>7.1</v>
+        <v>6.8</v>
       </c>
       <c r="AY5">
-        <v>2.7</v>
+        <v>2.3</v>
       </c>
       <c r="AZ5">
-        <v>8.9</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="BA5">
-        <v>6.9</v>
+        <v>6.6</v>
       </c>
       <c r="BB5">
-        <v>2.4</v>
+        <v>2</v>
       </c>
       <c r="BC5">
-        <v>8.300000000000001</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="BD5">
-        <v>5.2</v>
+        <v>5.6</v>
       </c>
       <c r="BE5">
-        <v>6.2</v>
+        <v>5.9</v>
       </c>
       <c r="BF5">
         <v>0.8</v>
@@ -2649,13 +2649,13 @@
         <v>0.09</v>
       </c>
       <c r="BK5">
-        <v>1.1649</v>
+        <v>1.1631</v>
       </c>
       <c r="BL5" t="s">
         <v>164</v>
       </c>
       <c r="BM5">
-        <v>1451</v>
+        <v>1488</v>
       </c>
       <c r="BN5" t="s">
         <v>61</v>
@@ -2664,34 +2664,34 @@
         <v>62</v>
       </c>
       <c r="BP5">
-        <v>78.8</v>
+        <v>78.5</v>
       </c>
       <c r="BQ5">
-        <v>1.069</v>
+        <v>1.068</v>
       </c>
       <c r="BR5">
         <v>80.59999999999999</v>
       </c>
       <c r="BS5">
-        <v>75.40000000000001</v>
+        <v>75</v>
       </c>
       <c r="BT5">
-        <v>58.6</v>
+        <v>58.7</v>
       </c>
       <c r="BU5">
-        <v>56.5</v>
+        <v>56.7</v>
       </c>
       <c r="BV5">
-        <v>59.2</v>
+        <v>57.2</v>
       </c>
       <c r="BW5">
-        <v>5.9</v>
+        <v>12</v>
       </c>
       <c r="BX5" t="s">
         <v>72</v>
       </c>
       <c r="BY5">
-        <v>11.8</v>
+        <v>9.4</v>
       </c>
       <c r="BZ5" t="s">
         <v>72</v>
@@ -2700,7 +2700,7 @@
         <v>82</v>
       </c>
       <c r="CB5">
-        <v>77.90000000000001</v>
+        <v>79.09999999999999</v>
       </c>
       <c r="CC5">
         <v>10</v>
@@ -2807,13 +2807,13 @@
         <v>60</v>
       </c>
       <c r="E2">
-        <v>61.6</v>
+        <v>61.7</v>
       </c>
       <c r="F2" t="s">
         <v>68</v>
       </c>
       <c r="G2">
-        <v>92</v>
+        <v>93.09999999999999</v>
       </c>
       <c r="H2">
         <v>7</v>
@@ -2831,10 +2831,10 @@
         <v>70</v>
       </c>
       <c r="M2">
-        <v>85</v>
+        <v>85.2</v>
       </c>
       <c r="N2">
-        <v>1751</v>
+        <v>1771</v>
       </c>
       <c r="O2" t="s">
         <v>61</v>

</xml_diff>

<commit_message>
Update MLB weather 2026-07-14 06:07 PM PT
</commit_message>
<xml_diff>
--- a/mlb_weather_professional_v4_2026_07_14.xlsx
+++ b/mlb_weather_professional_v4_2026_07_14.xlsx
@@ -12,8 +12,8 @@
     <sheet name="HR Weather" sheetId="3" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Game Summary'!$A$1:$BB$2</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Hourly Detail'!$A$1:$CG$5</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Game Summary'!$A$1:$AZ$2</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Hourly Detail'!$A$1:$CA$5</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'HR Weather'!$A$1:$Q$2</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="420" uniqueCount="166">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="400" uniqueCount="158">
   <si>
     <t>Date</t>
   </si>
@@ -152,12 +152,6 @@
     <t>Carry Score Change Since Last Run</t>
   </si>
   <si>
-    <t>Current Temp Bias F</t>
-  </si>
-  <si>
-    <t>Current Wind Bias MPH</t>
-  </si>
-  <si>
     <t>Park Learned Calibration Points</t>
   </si>
   <si>
@@ -215,22 +209,19 @@
     <t>Clear</t>
   </si>
   <si>
-    <t>🟢 4.0 mph Out to CF</t>
+    <t>🟢 8.7 mph Out to RF</t>
   </si>
   <si>
     <t>SW</t>
   </si>
   <si>
-    <t>4 mph, Out To CF</t>
-  </si>
-  <si>
-    <t>MLB RECORDED GAME WEATHER</t>
+    <t>FORECAST MODEL</t>
   </si>
   <si>
     <t>B+</t>
   </si>
   <si>
-    <t>Density 80 | Wind 62 | Temp 64 | Altitude 62 | Confidence 93%</t>
+    <t>Density 79 | Wind 64 | Temp 63 | Altitude 62 | Confidence 90%</t>
   </si>
   <si>
     <t>🟢 Good</t>
@@ -242,7 +233,7 @@
     <t>LOW</t>
   </si>
   <si>
-    <t>2026-07-14 06:01:45 PM PDT</t>
+    <t>2026-07-14 06:07:02 PM PDT</t>
   </si>
   <si>
     <t>Period</t>
@@ -293,15 +284,6 @@
     <t>Interpolation Fraction</t>
   </si>
   <si>
-    <t>Observation Bias Weight</t>
-  </si>
-  <si>
-    <t>Temperature Bias Applied F</t>
-  </si>
-  <si>
-    <t>Wind Bias Applied MPH</t>
-  </si>
-  <si>
     <t>Ensemble Disagreement Score</t>
   </si>
   <si>
@@ -464,9 +446,6 @@
     <t>Model Wind MPH</t>
   </si>
   <si>
-    <t>Official First Pitch Wind</t>
-  </si>
-  <si>
     <t>First Pitch</t>
   </si>
   <si>
@@ -488,7 +467,7 @@
     <t>11:00 PM EDT</t>
   </si>
   <si>
-    <t>2026-07-15 01:01:45 UTC</t>
+    <t>2026-07-15 01:07:02 UTC</t>
   </si>
   <si>
     <t>2026-07-14T21:58:43+00:00</t>
@@ -516,9 +495,6 @@
   </si>
   <si>
     <t>NEUTRAL</t>
-  </si>
-  <si>
-    <t>ACTUAL / RECORDED</t>
   </si>
 </sst>
 </file>
@@ -964,7 +940,7 @@
   <sheetPr>
     <tabColor rgb="FF70AD47"/>
   </sheetPr>
-  <dimension ref="A1:BB2"/>
+  <dimension ref="A1:AZ2"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="12.7109375" customWidth="1"/>
@@ -982,7 +958,7 @@
     <col min="14" max="15" width="28.7109375" customWidth="1"/>
     <col min="16" max="18" width="32.7109375" customWidth="1"/>
     <col min="19" max="19" width="24.7109375" customWidth="1"/>
-    <col min="20" max="20" width="27.7109375" customWidth="1"/>
+    <col min="20" max="20" width="18.7109375" customWidth="1"/>
     <col min="21" max="21" width="29.7109375" customWidth="1"/>
     <col min="22" max="22" width="22.7109375" customWidth="1"/>
     <col min="23" max="23" width="19.7109375" customWidth="1"/>
@@ -1004,18 +980,16 @@
     <col min="41" max="41" width="15.7109375" customWidth="1"/>
     <col min="42" max="42" width="19.7109375" customWidth="1"/>
     <col min="43" max="43" width="34.7109375" customWidth="1"/>
-    <col min="44" max="44" width="21.7109375" customWidth="1"/>
-    <col min="45" max="45" width="23.7109375" customWidth="1"/>
-    <col min="46" max="46" width="33.7109375" customWidth="1"/>
-    <col min="47" max="47" width="32.7109375" customWidth="1"/>
-    <col min="48" max="48" width="16.7109375" customWidth="1"/>
-    <col min="49" max="50" width="22.7109375" customWidth="1"/>
-    <col min="51" max="52" width="28.7109375" customWidth="1"/>
-    <col min="53" max="53" width="22.7109375" customWidth="1"/>
-    <col min="54" max="54" width="18.7109375" customWidth="1"/>
+    <col min="44" max="44" width="33.7109375" customWidth="1"/>
+    <col min="45" max="45" width="32.7109375" customWidth="1"/>
+    <col min="46" max="46" width="16.7109375" customWidth="1"/>
+    <col min="47" max="48" width="22.7109375" customWidth="1"/>
+    <col min="49" max="50" width="28.7109375" customWidth="1"/>
+    <col min="51" max="51" width="22.7109375" customWidth="1"/>
+    <col min="52" max="52" width="18.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:54" ht="34" customHeight="1">
+    <row r="1" spans="1:52" ht="34" customHeight="1">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1172,106 +1146,97 @@
       <c r="AZ1" s="1" t="s">
         <v>51</v>
       </c>
-      <c r="BA1" s="1" t="s">
+    </row>
+    <row r="2" spans="1:52">
+      <c r="A2" t="s">
         <v>52</v>
       </c>
-      <c r="BB1" s="1" t="s">
+      <c r="B2" t="s">
         <v>53</v>
       </c>
-    </row>
-    <row r="2" spans="1:54">
-      <c r="A2" t="s">
+      <c r="C2" t="s">
         <v>54</v>
       </c>
-      <c r="B2" t="s">
+      <c r="D2" t="s">
         <v>55</v>
       </c>
-      <c r="C2" t="s">
+      <c r="E2" t="s">
         <v>56</v>
       </c>
-      <c r="D2" t="s">
+      <c r="F2" t="s">
         <v>57</v>
       </c>
-      <c r="E2" t="s">
+      <c r="G2" t="s">
         <v>58</v>
       </c>
-      <c r="F2" t="s">
+      <c r="H2" t="s">
         <v>59</v>
       </c>
-      <c r="G2" t="s">
+      <c r="I2" t="s">
         <v>60</v>
       </c>
-      <c r="H2" t="s">
+      <c r="J2" t="s">
         <v>61</v>
       </c>
-      <c r="I2" t="s">
+      <c r="K2">
+        <v>85.8</v>
+      </c>
+      <c r="L2">
+        <v>60.4</v>
+      </c>
+      <c r="M2" t="s">
         <v>62</v>
       </c>
-      <c r="J2" t="s">
+      <c r="N2">
+        <v>9.4</v>
+      </c>
+      <c r="O2" t="s">
         <v>63</v>
       </c>
-      <c r="K2">
-        <v>88</v>
-      </c>
-      <c r="L2">
-        <v>59.7</v>
-      </c>
-      <c r="M2" t="s">
+      <c r="P2">
+        <v>2.8</v>
+      </c>
+      <c r="Q2">
+        <v>7.5</v>
+      </c>
+      <c r="R2">
+        <v>8.699999999999999</v>
+      </c>
+      <c r="T2" t="s">
         <v>64</v>
-      </c>
-      <c r="N2">
-        <v>4</v>
-      </c>
-      <c r="O2" t="s">
-        <v>65</v>
-      </c>
-      <c r="P2">
-        <v>3.3</v>
-      </c>
-      <c r="Q2">
-        <v>4</v>
-      </c>
-      <c r="R2">
-        <v>3.3</v>
-      </c>
-      <c r="S2" t="s">
-        <v>66</v>
-      </c>
-      <c r="T2" t="s">
-        <v>67</v>
       </c>
       <c r="U2">
         <v>0</v>
       </c>
       <c r="V2">
-        <v>61.7</v>
+        <v>62.7</v>
       </c>
       <c r="W2" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="X2" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="Y2">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="Z2">
+        <v>6</v>
+      </c>
+      <c r="AA2">
+        <v>3.8</v>
+      </c>
+      <c r="AB2">
+        <v>90.5</v>
+      </c>
+      <c r="AC2" t="s">
+        <v>67</v>
+      </c>
+      <c r="AD2">
+        <v>6.4</v>
+      </c>
+      <c r="AE2">
         <v>5</v>
-      </c>
-      <c r="AA2">
-        <v>3.5</v>
-      </c>
-      <c r="AB2">
-        <v>93.09999999999999</v>
-      </c>
-      <c r="AC2" t="s">
-        <v>70</v>
-      </c>
-      <c r="AD2">
-        <v>5.2</v>
-      </c>
-      <c r="AE2">
-        <v>4</v>
       </c>
       <c r="AF2">
         <v>100</v>
@@ -1280,34 +1245,34 @@
         <v>0</v>
       </c>
       <c r="AH2">
-        <v>4</v>
+        <v>4.8</v>
       </c>
       <c r="AI2">
-        <v>0.6</v>
+        <v>0.4</v>
       </c>
       <c r="AJ2">
-        <v>1.1538</v>
+        <v>1.1557</v>
       </c>
       <c r="AK2">
-        <v>1771</v>
+        <v>1710</v>
       </c>
       <c r="AL2">
         <v>1012</v>
       </c>
       <c r="AM2">
-        <v>70</v>
+        <v>70.2</v>
       </c>
       <c r="AN2">
-        <v>85.2</v>
+        <v>84.2</v>
       </c>
       <c r="AO2">
-        <v>63.4</v>
+        <v>64.09999999999999</v>
       </c>
       <c r="AP2" t="s">
-        <v>71</v>
+        <v>68</v>
       </c>
       <c r="AQ2">
-        <v>16.3</v>
+        <v>17.2</v>
       </c>
       <c r="AR2">
         <v>0</v>
@@ -1315,36 +1280,30 @@
       <c r="AS2">
         <v>0</v>
       </c>
-      <c r="AT2">
-        <v>0</v>
+      <c r="AT2" t="s">
+        <v>69</v>
       </c>
       <c r="AU2">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="AV2" t="s">
-        <v>72</v>
+        <v>69</v>
       </c>
       <c r="AW2">
-        <v>12</v>
+        <v>15.1</v>
       </c>
       <c r="AX2" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="AY2">
-        <v>14.6</v>
-      </c>
-      <c r="AZ2" t="s">
-        <v>73</v>
-      </c>
-      <c r="BA2">
-        <v>183</v>
-      </c>
-      <c r="BB2">
+        <v>188.3</v>
+      </c>
+      <c r="AZ2">
         <v>5</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:BB2"/>
+  <autoFilter ref="A1:AZ2"/>
   <conditionalFormatting sqref="B2">
     <cfRule type="expression" dxfId="0" priority="1">
       <formula>OR(ISNUMBER(SEARCH("Elite",$AC2)),ISNUMBER(SEARCH("Excellent",$AC2)),ISNUMBER(SEARCH("Very Good",$AC2)),ISNUMBER(SEARCH("Good",$AC2)))</formula>
@@ -1376,7 +1335,7 @@
   <sheetPr>
     <tabColor rgb="FF5B9BD5"/>
   </sheetPr>
-  <dimension ref="A1:CG5"/>
+  <dimension ref="A1:CA5"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="28.7109375" customWidth="1"/>
@@ -1397,61 +1356,55 @@
     <col min="18" max="19" width="28.7109375" customWidth="1"/>
     <col min="20" max="22" width="26.7109375" customWidth="1"/>
     <col min="23" max="23" width="24.7109375" customWidth="1"/>
-    <col min="24" max="24" width="25.7109375" customWidth="1"/>
-    <col min="25" max="25" width="28.7109375" customWidth="1"/>
-    <col min="26" max="26" width="23.7109375" customWidth="1"/>
-    <col min="27" max="27" width="28.7109375" customWidth="1"/>
-    <col min="28" max="28" width="22.7109375" customWidth="1"/>
-    <col min="29" max="29" width="28.7109375" customWidth="1"/>
-    <col min="30" max="30" width="20.7109375" customWidth="1"/>
-    <col min="31" max="31" width="27.7109375" customWidth="1"/>
-    <col min="32" max="32" width="17.7109375" customWidth="1"/>
-    <col min="33" max="33" width="25.7109375" customWidth="1"/>
-    <col min="34" max="34" width="12.7109375" customWidth="1"/>
+    <col min="24" max="24" width="28.7109375" customWidth="1"/>
+    <col min="25" max="25" width="22.7109375" customWidth="1"/>
+    <col min="26" max="26" width="28.7109375" customWidth="1"/>
+    <col min="27" max="27" width="20.7109375" customWidth="1"/>
+    <col min="28" max="28" width="27.7109375" customWidth="1"/>
+    <col min="29" max="29" width="17.7109375" customWidth="1"/>
+    <col min="30" max="30" width="25.7109375" customWidth="1"/>
+    <col min="31" max="31" width="12.7109375" customWidth="1"/>
+    <col min="32" max="32" width="10.7109375" customWidth="1"/>
+    <col min="33" max="33" width="14.7109375" customWidth="1"/>
+    <col min="34" max="34" width="13.7109375" customWidth="1"/>
     <col min="35" max="35" width="10.7109375" customWidth="1"/>
-    <col min="36" max="36" width="14.7109375" customWidth="1"/>
-    <col min="37" max="37" width="13.7109375" customWidth="1"/>
-    <col min="38" max="38" width="10.7109375" customWidth="1"/>
-    <col min="39" max="39" width="22.7109375" customWidth="1"/>
-    <col min="40" max="40" width="24.7109375" customWidth="1"/>
-    <col min="41" max="41" width="15.7109375" customWidth="1"/>
-    <col min="42" max="42" width="10.7109375" customWidth="1"/>
-    <col min="43" max="43" width="15.7109375" customWidth="1"/>
-    <col min="44" max="44" width="18.7109375" customWidth="1"/>
+    <col min="36" max="36" width="22.7109375" customWidth="1"/>
+    <col min="37" max="37" width="24.7109375" customWidth="1"/>
+    <col min="38" max="38" width="15.7109375" customWidth="1"/>
+    <col min="39" max="39" width="10.7109375" customWidth="1"/>
+    <col min="40" max="40" width="15.7109375" customWidth="1"/>
+    <col min="41" max="41" width="18.7109375" customWidth="1"/>
+    <col min="42" max="42" width="11.7109375" customWidth="1"/>
+    <col min="43" max="43" width="10.7109375" customWidth="1"/>
+    <col min="44" max="44" width="15.7109375" customWidth="1"/>
     <col min="45" max="45" width="11.7109375" customWidth="1"/>
-    <col min="46" max="46" width="10.7109375" customWidth="1"/>
-    <col min="47" max="47" width="15.7109375" customWidth="1"/>
-    <col min="48" max="48" width="11.7109375" customWidth="1"/>
-    <col min="49" max="49" width="19.7109375" customWidth="1"/>
-    <col min="50" max="52" width="24.7109375" customWidth="1"/>
-    <col min="53" max="55" width="20.7109375" customWidth="1"/>
-    <col min="56" max="56" width="15.7109375" customWidth="1"/>
-    <col min="57" max="57" width="27.7109375" customWidth="1"/>
-    <col min="58" max="58" width="28.7109375" customWidth="1"/>
-    <col min="59" max="61" width="22.7109375" customWidth="1"/>
-    <col min="62" max="64" width="19.7109375" customWidth="1"/>
-    <col min="65" max="65" width="21.7109375" customWidth="1"/>
-    <col min="66" max="66" width="13.7109375" customWidth="1"/>
-    <col min="67" max="67" width="15.7109375" customWidth="1"/>
-    <col min="68" max="68" width="16.7109375" customWidth="1"/>
-    <col min="69" max="69" width="18.7109375" customWidth="1"/>
-    <col min="70" max="71" width="17.7109375" customWidth="1"/>
-    <col min="72" max="72" width="11.7109375" customWidth="1"/>
-    <col min="73" max="73" width="23.7109375" customWidth="1"/>
-    <col min="74" max="74" width="24.7109375" customWidth="1"/>
-    <col min="75" max="75" width="18.7109375" customWidth="1"/>
+    <col min="46" max="46" width="19.7109375" customWidth="1"/>
+    <col min="47" max="49" width="24.7109375" customWidth="1"/>
+    <col min="50" max="52" width="20.7109375" customWidth="1"/>
+    <col min="53" max="53" width="15.7109375" customWidth="1"/>
+    <col min="54" max="54" width="27.7109375" customWidth="1"/>
+    <col min="55" max="55" width="28.7109375" customWidth="1"/>
+    <col min="56" max="58" width="22.7109375" customWidth="1"/>
+    <col min="59" max="61" width="19.7109375" customWidth="1"/>
+    <col min="62" max="62" width="21.7109375" customWidth="1"/>
+    <col min="63" max="63" width="13.7109375" customWidth="1"/>
+    <col min="64" max="64" width="15.7109375" customWidth="1"/>
+    <col min="65" max="65" width="16.7109375" customWidth="1"/>
+    <col min="66" max="66" width="18.7109375" customWidth="1"/>
+    <col min="67" max="68" width="17.7109375" customWidth="1"/>
+    <col min="69" max="69" width="11.7109375" customWidth="1"/>
+    <col min="70" max="70" width="23.7109375" customWidth="1"/>
+    <col min="71" max="71" width="24.7109375" customWidth="1"/>
+    <col min="72" max="72" width="18.7109375" customWidth="1"/>
+    <col min="73" max="73" width="12.7109375" customWidth="1"/>
+    <col min="74" max="74" width="28.7109375" customWidth="1"/>
+    <col min="75" max="75" width="22.7109375" customWidth="1"/>
     <col min="76" max="76" width="12.7109375" customWidth="1"/>
-    <col min="77" max="77" width="28.7109375" customWidth="1"/>
-    <col min="78" max="78" width="22.7109375" customWidth="1"/>
-    <col min="79" max="79" width="12.7109375" customWidth="1"/>
-    <col min="80" max="81" width="14.7109375" customWidth="1"/>
-    <col min="82" max="82" width="16.7109375" customWidth="1"/>
-    <col min="83" max="83" width="27.7109375" customWidth="1"/>
-    <col min="84" max="84" width="24.7109375" customWidth="1"/>
-    <col min="85" max="85" width="27.7109375" customWidth="1"/>
+    <col min="77" max="78" width="14.7109375" customWidth="1"/>
+    <col min="79" max="79" width="16.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:85" ht="34" customHeight="1">
+    <row r="1" spans="1:79" ht="34" customHeight="1">
       <c r="A1" s="1" t="s">
         <v>3</v>
       </c>
@@ -1465,279 +1418,261 @@
         <v>6</v>
       </c>
       <c r="E1" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="I1" s="1" t="s">
         <v>74</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="J1" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="K1" s="1" t="s">
         <v>75</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="L1" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="M1" s="1" t="s">
         <v>76</v>
       </c>
-      <c r="H1" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="I1" s="1" t="s">
+      <c r="N1" s="1" t="s">
         <v>77</v>
       </c>
-      <c r="J1" s="1" t="s">
-        <v>52</v>
-      </c>
-      <c r="K1" s="1" t="s">
+      <c r="O1" s="1" t="s">
         <v>78</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="P1" s="1" t="s">
+        <v>79</v>
+      </c>
+      <c r="Q1" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="R1" s="1" t="s">
+        <v>81</v>
+      </c>
+      <c r="S1" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="T1" s="1" t="s">
+        <v>83</v>
+      </c>
+      <c r="U1" s="1" t="s">
+        <v>84</v>
+      </c>
+      <c r="V1" s="1" t="s">
+        <v>85</v>
+      </c>
+      <c r="W1" s="1" t="s">
+        <v>86</v>
+      </c>
+      <c r="X1" s="1" t="s">
+        <v>87</v>
+      </c>
+      <c r="Y1" s="1" t="s">
+        <v>88</v>
+      </c>
+      <c r="Z1" s="1" t="s">
+        <v>89</v>
+      </c>
+      <c r="AA1" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="AB1" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="AC1" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="AD1" s="1" t="s">
+        <v>93</v>
+      </c>
+      <c r="AE1" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="AF1" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="AG1" s="1" t="s">
+        <v>96</v>
+      </c>
+      <c r="AH1" s="1" t="s">
+        <v>97</v>
+      </c>
+      <c r="AI1" s="1" t="s">
+        <v>98</v>
+      </c>
+      <c r="AJ1" s="1" t="s">
+        <v>99</v>
+      </c>
+      <c r="AK1" s="1" t="s">
+        <v>100</v>
+      </c>
+      <c r="AL1" s="1" t="s">
+        <v>101</v>
+      </c>
+      <c r="AM1" s="1" t="s">
+        <v>102</v>
+      </c>
+      <c r="AN1" s="1" t="s">
+        <v>103</v>
+      </c>
+      <c r="AO1" s="1" t="s">
+        <v>104</v>
+      </c>
+      <c r="AP1" s="1" t="s">
+        <v>105</v>
+      </c>
+      <c r="AQ1" s="1" t="s">
+        <v>106</v>
+      </c>
+      <c r="AR1" s="1" t="s">
+        <v>107</v>
+      </c>
+      <c r="AS1" s="1" t="s">
+        <v>108</v>
+      </c>
+      <c r="AT1" s="1" t="s">
+        <v>109</v>
+      </c>
+      <c r="AU1" s="1" t="s">
+        <v>110</v>
+      </c>
+      <c r="AV1" s="1" t="s">
+        <v>111</v>
+      </c>
+      <c r="AW1" s="1" t="s">
+        <v>112</v>
+      </c>
+      <c r="AX1" s="1" t="s">
+        <v>113</v>
+      </c>
+      <c r="AY1" s="1" t="s">
+        <v>114</v>
+      </c>
+      <c r="AZ1" s="1" t="s">
+        <v>115</v>
+      </c>
+      <c r="BA1" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="BB1" s="1" t="s">
+        <v>117</v>
+      </c>
+      <c r="BC1" s="1" t="s">
+        <v>118</v>
+      </c>
+      <c r="BD1" s="1" t="s">
+        <v>119</v>
+      </c>
+      <c r="BE1" s="1" t="s">
+        <v>120</v>
+      </c>
+      <c r="BF1" s="1" t="s">
+        <v>121</v>
+      </c>
+      <c r="BG1" s="1" t="s">
+        <v>122</v>
+      </c>
+      <c r="BH1" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="BI1" s="1" t="s">
+        <v>124</v>
+      </c>
+      <c r="BJ1" s="1" t="s">
+        <v>125</v>
+      </c>
+      <c r="BK1" s="1" t="s">
+        <v>126</v>
+      </c>
+      <c r="BL1" s="1" t="s">
+        <v>127</v>
+      </c>
+      <c r="BM1" s="1" t="s">
+        <v>128</v>
+      </c>
+      <c r="BN1" s="1" t="s">
+        <v>129</v>
+      </c>
+      <c r="BO1" s="1" t="s">
+        <v>130</v>
+      </c>
+      <c r="BP1" s="1" t="s">
+        <v>131</v>
+      </c>
+      <c r="BQ1" s="1" t="s">
+        <v>132</v>
+      </c>
+      <c r="BR1" s="1" t="s">
+        <v>133</v>
+      </c>
+      <c r="BS1" s="1" t="s">
+        <v>134</v>
+      </c>
+      <c r="BT1" s="1" t="s">
+        <v>135</v>
+      </c>
+      <c r="BU1" s="1" t="s">
+        <v>136</v>
+      </c>
+      <c r="BV1" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="BW1" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="BX1" s="1" t="s">
+        <v>137</v>
+      </c>
+      <c r="BY1" s="1" t="s">
+        <v>138</v>
+      </c>
+      <c r="BZ1" s="1" t="s">
+        <v>139</v>
+      </c>
+      <c r="CA1" s="1" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="2" spans="1:79">
+      <c r="A2" t="s">
+        <v>55</v>
+      </c>
+      <c r="B2" t="s">
         <v>53</v>
       </c>
-      <c r="M1" s="1" t="s">
-        <v>79</v>
-      </c>
-      <c r="N1" s="1" t="s">
-        <v>80</v>
-      </c>
-      <c r="O1" s="1" t="s">
-        <v>81</v>
-      </c>
-      <c r="P1" s="1" t="s">
-        <v>82</v>
-      </c>
-      <c r="Q1" s="1" t="s">
-        <v>83</v>
-      </c>
-      <c r="R1" s="1" t="s">
-        <v>84</v>
-      </c>
-      <c r="S1" s="1" t="s">
-        <v>85</v>
-      </c>
-      <c r="T1" s="1" t="s">
-        <v>86</v>
-      </c>
-      <c r="U1" s="1" t="s">
-        <v>87</v>
-      </c>
-      <c r="V1" s="1" t="s">
-        <v>88</v>
-      </c>
-      <c r="W1" s="1" t="s">
-        <v>89</v>
-      </c>
-      <c r="X1" s="1" t="s">
-        <v>90</v>
-      </c>
-      <c r="Y1" s="1" t="s">
-        <v>91</v>
-      </c>
-      <c r="Z1" s="1" t="s">
-        <v>92</v>
-      </c>
-      <c r="AA1" s="1" t="s">
-        <v>93</v>
-      </c>
-      <c r="AB1" s="1" t="s">
-        <v>94</v>
-      </c>
-      <c r="AC1" s="1" t="s">
-        <v>95</v>
-      </c>
-      <c r="AD1" s="1" t="s">
-        <v>96</v>
-      </c>
-      <c r="AE1" s="1" t="s">
-        <v>97</v>
-      </c>
-      <c r="AF1" s="1" t="s">
-        <v>98</v>
-      </c>
-      <c r="AG1" s="1" t="s">
-        <v>99</v>
-      </c>
-      <c r="AH1" s="1" t="s">
-        <v>100</v>
-      </c>
-      <c r="AI1" s="1" t="s">
-        <v>101</v>
-      </c>
-      <c r="AJ1" s="1" t="s">
-        <v>102</v>
-      </c>
-      <c r="AK1" s="1" t="s">
-        <v>103</v>
-      </c>
-      <c r="AL1" s="1" t="s">
-        <v>104</v>
-      </c>
-      <c r="AM1" s="1" t="s">
-        <v>105</v>
-      </c>
-      <c r="AN1" s="1" t="s">
-        <v>106</v>
-      </c>
-      <c r="AO1" s="1" t="s">
-        <v>107</v>
-      </c>
-      <c r="AP1" s="1" t="s">
-        <v>108</v>
-      </c>
-      <c r="AQ1" s="1" t="s">
-        <v>109</v>
-      </c>
-      <c r="AR1" s="1" t="s">
-        <v>110</v>
-      </c>
-      <c r="AS1" s="1" t="s">
-        <v>111</v>
-      </c>
-      <c r="AT1" s="1" t="s">
-        <v>112</v>
-      </c>
-      <c r="AU1" s="1" t="s">
-        <v>113</v>
-      </c>
-      <c r="AV1" s="1" t="s">
-        <v>114</v>
-      </c>
-      <c r="AW1" s="1" t="s">
-        <v>115</v>
-      </c>
-      <c r="AX1" s="1" t="s">
-        <v>116</v>
-      </c>
-      <c r="AY1" s="1" t="s">
-        <v>117</v>
-      </c>
-      <c r="AZ1" s="1" t="s">
-        <v>118</v>
-      </c>
-      <c r="BA1" s="1" t="s">
-        <v>119</v>
-      </c>
-      <c r="BB1" s="1" t="s">
-        <v>120</v>
-      </c>
-      <c r="BC1" s="1" t="s">
-        <v>121</v>
-      </c>
-      <c r="BD1" s="1" t="s">
-        <v>122</v>
-      </c>
-      <c r="BE1" s="1" t="s">
-        <v>123</v>
-      </c>
-      <c r="BF1" s="1" t="s">
-        <v>124</v>
-      </c>
-      <c r="BG1" s="1" t="s">
-        <v>125</v>
-      </c>
-      <c r="BH1" s="1" t="s">
-        <v>126</v>
-      </c>
-      <c r="BI1" s="1" t="s">
-        <v>127</v>
-      </c>
-      <c r="BJ1" s="1" t="s">
-        <v>128</v>
-      </c>
-      <c r="BK1" s="1" t="s">
-        <v>129</v>
-      </c>
-      <c r="BL1" s="1" t="s">
-        <v>130</v>
-      </c>
-      <c r="BM1" s="1" t="s">
-        <v>131</v>
-      </c>
-      <c r="BN1" s="1" t="s">
-        <v>132</v>
-      </c>
-      <c r="BO1" s="1" t="s">
-        <v>133</v>
-      </c>
-      <c r="BP1" s="1" t="s">
-        <v>134</v>
-      </c>
-      <c r="BQ1" s="1" t="s">
-        <v>135</v>
-      </c>
-      <c r="BR1" s="1" t="s">
-        <v>136</v>
-      </c>
-      <c r="BS1" s="1" t="s">
-        <v>137</v>
-      </c>
-      <c r="BT1" s="1" t="s">
-        <v>138</v>
-      </c>
-      <c r="BU1" s="1" t="s">
-        <v>139</v>
-      </c>
-      <c r="BV1" s="1" t="s">
-        <v>140</v>
-      </c>
-      <c r="BW1" s="1" t="s">
+      <c r="C2" t="s">
+        <v>54</v>
+      </c>
+      <c r="D2" t="s">
+        <v>58</v>
+      </c>
+      <c r="E2" t="s">
         <v>141</v>
       </c>
-      <c r="BX1" s="1" t="s">
-        <v>142</v>
-      </c>
-      <c r="BY1" s="1" t="s">
-        <v>50</v>
-      </c>
-      <c r="BZ1" s="1" t="s">
-        <v>49</v>
-      </c>
-      <c r="CA1" s="1" t="s">
-        <v>143</v>
-      </c>
-      <c r="CB1" s="1" t="s">
-        <v>144</v>
-      </c>
-      <c r="CC1" s="1" t="s">
-        <v>145</v>
-      </c>
-      <c r="CD1" s="1" t="s">
-        <v>146</v>
-      </c>
-      <c r="CE1" s="1" t="s">
-        <v>147</v>
-      </c>
-      <c r="CF1" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="CG1" s="1" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="2" spans="1:85">
-      <c r="A2" t="s">
+      <c r="F2" t="s">
         <v>57</v>
       </c>
-      <c r="B2" t="s">
-        <v>55</v>
-      </c>
-      <c r="C2" t="s">
-        <v>56</v>
-      </c>
-      <c r="D2" t="s">
-        <v>60</v>
-      </c>
-      <c r="E2" t="s">
+      <c r="G2" t="s">
         <v>148</v>
       </c>
-      <c r="F2" t="s">
-        <v>59</v>
-      </c>
-      <c r="G2" t="s">
-        <v>155</v>
-      </c>
       <c r="H2" t="s">
-        <v>73</v>
+        <v>70</v>
       </c>
       <c r="I2" t="s">
-        <v>156</v>
+        <v>149</v>
       </c>
       <c r="J2">
-        <v>183</v>
+        <v>188.3</v>
       </c>
       <c r="K2">
         <v>0</v>
@@ -1746,7 +1681,7 @@
         <v>5</v>
       </c>
       <c r="M2">
-        <v>1.2</v>
+        <v>0.99</v>
       </c>
       <c r="N2">
         <v>0.5600000000000001</v>
@@ -1755,7 +1690,7 @@
         <v>0</v>
       </c>
       <c r="P2">
-        <v>3.8</v>
+        <v>4.4</v>
       </c>
       <c r="Q2">
         <v>0.5</v>
@@ -1767,234 +1702,216 @@
         <v>0</v>
       </c>
       <c r="T2" t="s">
-        <v>157</v>
+        <v>150</v>
       </c>
       <c r="U2" t="s">
-        <v>158</v>
+        <v>151</v>
       </c>
       <c r="V2" t="s">
-        <v>159</v>
+        <v>152</v>
       </c>
       <c r="W2">
         <v>1</v>
       </c>
       <c r="X2">
+        <v>5.7</v>
+      </c>
+      <c r="Y2">
+        <v>93</v>
+      </c>
+      <c r="Z2">
+        <v>81.7</v>
+      </c>
+      <c r="AA2">
+        <v>0.98</v>
+      </c>
+      <c r="AB2">
+        <v>0.7</v>
+      </c>
+      <c r="AC2">
+        <v>1.6</v>
+      </c>
+      <c r="AD2">
+        <v>1.6</v>
+      </c>
+      <c r="AE2" t="s">
+        <v>61</v>
+      </c>
+      <c r="AF2">
+        <v>85.8</v>
+      </c>
+      <c r="AG2">
+        <v>88.09999999999999</v>
+      </c>
+      <c r="AH2">
+        <v>70.09999999999999</v>
+      </c>
+      <c r="AI2">
+        <v>60.4</v>
+      </c>
+      <c r="AJ2">
+        <v>1011.9</v>
+      </c>
+      <c r="AK2">
+        <v>1014.1</v>
+      </c>
+      <c r="AL2">
         <v>0</v>
       </c>
-      <c r="Y2">
+      <c r="AM2">
         <v>0</v>
       </c>
-      <c r="Z2">
+      <c r="AN2">
         <v>0</v>
       </c>
-      <c r="AA2">
-        <v>0</v>
-      </c>
-      <c r="AB2">
-        <v>100</v>
-      </c>
-      <c r="AC2">
-        <v>79.2</v>
-      </c>
-      <c r="AD2">
+      <c r="AO2">
+        <v>49.3</v>
+      </c>
+      <c r="AP2">
+        <v>1542</v>
+      </c>
+      <c r="AQ2">
+        <v>9.4</v>
+      </c>
+      <c r="AR2">
+        <v>21.4</v>
+      </c>
+      <c r="AS2" t="s">
+        <v>63</v>
+      </c>
+      <c r="AT2">
+        <v>225.5</v>
+      </c>
+      <c r="AU2">
+        <v>7.6</v>
+      </c>
+      <c r="AV2">
+        <v>3.1</v>
+      </c>
+      <c r="AW2">
+        <v>9.4</v>
+      </c>
+      <c r="AX2">
+        <v>7.5</v>
+      </c>
+      <c r="AY2">
+        <v>2.8</v>
+      </c>
+      <c r="AZ2">
+        <v>8.699999999999999</v>
+      </c>
+      <c r="BA2">
+        <v>5.3</v>
+      </c>
+      <c r="BB2">
+        <v>6.7</v>
+      </c>
+      <c r="BC2">
+        <v>0.8</v>
+      </c>
+      <c r="BD2">
+        <v>0.9399999999999999</v>
+      </c>
+      <c r="BE2">
+        <v>1.03</v>
+      </c>
+      <c r="BF2">
         <v>0.98</v>
       </c>
-      <c r="AE2">
-        <v>0.7</v>
-      </c>
-      <c r="AF2">
-        <v>1.6</v>
-      </c>
-      <c r="AG2">
-        <v>1.6</v>
-      </c>
-      <c r="AH2" t="s">
-        <v>63</v>
-      </c>
-      <c r="AI2">
-        <v>88</v>
-      </c>
-      <c r="AJ2">
-        <v>88.09999999999999</v>
-      </c>
-      <c r="AK2">
-        <v>69.90000000000001</v>
-      </c>
-      <c r="AL2">
-        <v>59.7</v>
-      </c>
-      <c r="AM2">
-        <v>1011.9</v>
-      </c>
-      <c r="AN2">
-        <v>1014.1</v>
-      </c>
-      <c r="AO2">
-        <v>0</v>
-      </c>
-      <c r="AP2">
-        <v>0</v>
-      </c>
-      <c r="AQ2">
-        <v>0</v>
-      </c>
-      <c r="AR2">
-        <v>49.3</v>
-      </c>
-      <c r="AS2">
-        <v>1482</v>
-      </c>
-      <c r="AT2">
-        <v>4</v>
-      </c>
-      <c r="AU2">
-        <v>21.6</v>
-      </c>
-      <c r="AV2" t="s">
-        <v>65</v>
-      </c>
-      <c r="AW2">
-        <v>225.2</v>
-      </c>
-      <c r="AX2">
-        <v>7.7</v>
-      </c>
-      <c r="AY2">
-        <v>3.2</v>
-      </c>
-      <c r="AZ2">
-        <v>9.4</v>
-      </c>
-      <c r="BA2">
-        <v>4</v>
-      </c>
-      <c r="BB2">
-        <v>3.3</v>
-      </c>
-      <c r="BC2">
-        <v>3.3</v>
-      </c>
-      <c r="BD2">
-        <v>0</v>
-      </c>
-      <c r="BE2">
-        <v>3.7</v>
-      </c>
-      <c r="BF2">
-        <v>0.8</v>
-      </c>
       <c r="BG2">
-        <v>0.9399999999999999</v>
+        <v>0.09</v>
       </c>
       <c r="BH2">
-        <v>1.03</v>
-      </c>
-      <c r="BI2">
-        <v>0.98</v>
+        <v>1.1523</v>
+      </c>
+      <c r="BI2" t="s">
+        <v>156</v>
       </c>
       <c r="BJ2">
-        <v>0.09</v>
-      </c>
-      <c r="BK2">
-        <v>1.1478</v>
+        <v>1817</v>
+      </c>
+      <c r="BK2" t="s">
+        <v>59</v>
       </c>
       <c r="BL2" t="s">
-        <v>163</v>
+        <v>60</v>
       </c>
       <c r="BM2">
-        <v>1960</v>
-      </c>
-      <c r="BN2" t="s">
-        <v>61</v>
-      </c>
-      <c r="BO2" t="s">
-        <v>62</v>
+        <v>84.09999999999999</v>
+      </c>
+      <c r="BN2">
+        <v>1.082</v>
+      </c>
+      <c r="BO2">
+        <v>85.90000000000001</v>
       </c>
       <c r="BP2">
-        <v>79.2</v>
+        <v>80.59999999999999</v>
       </c>
       <c r="BQ2">
-        <v>1.07</v>
+        <v>60</v>
       </c>
       <c r="BR2">
-        <v>76.90000000000001</v>
+        <v>58.2</v>
       </c>
       <c r="BS2">
-        <v>76.90000000000001</v>
+        <v>47.9</v>
       </c>
       <c r="BT2">
-        <v>56.2</v>
-      </c>
-      <c r="BU2">
-        <v>57.3</v>
+        <v>12</v>
+      </c>
+      <c r="BU2" t="s">
+        <v>69</v>
       </c>
       <c r="BV2">
-        <v>45.5</v>
-      </c>
-      <c r="BW2">
-        <v>12</v>
-      </c>
-      <c r="BX2" t="s">
-        <v>72</v>
+        <v>8.1</v>
+      </c>
+      <c r="BW2" t="s">
+        <v>69</v>
+      </c>
+      <c r="BX2">
+        <v>87</v>
       </c>
       <c r="BY2">
-        <v>0</v>
-      </c>
-      <c r="BZ2" t="s">
-        <v>165</v>
+        <v>83.8</v>
+      </c>
+      <c r="BZ2">
+        <v>10</v>
       </c>
       <c r="CA2">
-        <v>87</v>
-      </c>
-      <c r="CB2">
-        <v>84</v>
-      </c>
-      <c r="CC2">
-        <v>10</v>
-      </c>
-      <c r="CD2">
         <v>9.199999999999999</v>
       </c>
-      <c r="CE2" t="s">
-        <v>64</v>
-      </c>
-      <c r="CF2" t="s">
-        <v>66</v>
-      </c>
-      <c r="CG2" t="s">
-        <v>67</v>
-      </c>
     </row>
-    <row r="3" spans="1:85">
+    <row r="3" spans="1:79">
       <c r="A3" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="B3" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="C3" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="D3" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="E3" t="s">
+        <v>142</v>
+      </c>
+      <c r="F3" t="s">
+        <v>145</v>
+      </c>
+      <c r="G3" t="s">
+        <v>148</v>
+      </c>
+      <c r="H3" t="s">
+        <v>70</v>
+      </c>
+      <c r="I3" t="s">
         <v>149</v>
       </c>
-      <c r="F3" t="s">
-        <v>152</v>
-      </c>
-      <c r="G3" t="s">
-        <v>155</v>
-      </c>
-      <c r="H3" t="s">
-        <v>73</v>
-      </c>
-      <c r="I3" t="s">
-        <v>156</v>
-      </c>
       <c r="J3">
-        <v>183</v>
+        <v>188.3</v>
       </c>
       <c r="K3">
         <v>0</v>
@@ -2003,19 +1920,19 @@
         <v>5</v>
       </c>
       <c r="M3">
-        <v>1.72</v>
+        <v>1.43</v>
       </c>
       <c r="N3">
-        <v>1.07</v>
+        <v>0.99</v>
       </c>
       <c r="O3">
         <v>0</v>
       </c>
       <c r="P3">
-        <v>4.4</v>
+        <v>5.2</v>
       </c>
       <c r="Q3">
-        <v>0.7</v>
+        <v>0.6</v>
       </c>
       <c r="R3">
         <v>100</v>
@@ -2024,246 +1941,237 @@
         <v>0</v>
       </c>
       <c r="T3" t="s">
-        <v>157</v>
+        <v>150</v>
       </c>
       <c r="U3" t="s">
-        <v>159</v>
+        <v>152</v>
       </c>
       <c r="V3" t="s">
-        <v>160</v>
+        <v>153</v>
       </c>
       <c r="W3">
         <v>1</v>
       </c>
       <c r="X3">
+        <v>8.699999999999999</v>
+      </c>
+      <c r="Y3">
+        <v>87.8</v>
+      </c>
+      <c r="Z3">
+        <v>77.8</v>
+      </c>
+      <c r="AA3">
+        <v>0.98</v>
+      </c>
+      <c r="AB3">
+        <v>0.7</v>
+      </c>
+      <c r="AC3">
+        <v>1.6</v>
+      </c>
+      <c r="AD3">
+        <v>1.6</v>
+      </c>
+      <c r="AE3" t="s">
+        <v>61</v>
+      </c>
+      <c r="AF3">
+        <v>84.2</v>
+      </c>
+      <c r="AG3">
+        <v>86</v>
+      </c>
+      <c r="AH3">
+        <v>70.59999999999999</v>
+      </c>
+      <c r="AI3">
+        <v>65.09999999999999</v>
+      </c>
+      <c r="AJ3">
+        <v>1011.9</v>
+      </c>
+      <c r="AK3">
+        <v>1014.2</v>
+      </c>
+      <c r="AL3">
         <v>0</v>
       </c>
-      <c r="Y3">
+      <c r="AM3">
         <v>0</v>
       </c>
-      <c r="Z3">
+      <c r="AN3">
         <v>0</v>
       </c>
-      <c r="AA3">
-        <v>10.1</v>
-      </c>
-      <c r="AB3">
-        <v>87.5</v>
-      </c>
-      <c r="AC3">
-        <v>77.90000000000001</v>
-      </c>
-      <c r="AD3">
+      <c r="AO3">
+        <v>37.7</v>
+      </c>
+      <c r="AP3">
+        <v>1677</v>
+      </c>
+      <c r="AQ3">
+        <v>8.9</v>
+      </c>
+      <c r="AR3">
+        <v>17.3</v>
+      </c>
+      <c r="AS3" t="s">
+        <v>63</v>
+      </c>
+      <c r="AT3">
+        <v>225.2</v>
+      </c>
+      <c r="AU3">
+        <v>7.3</v>
+      </c>
+      <c r="AV3">
+        <v>3</v>
+      </c>
+      <c r="AW3">
+        <v>8.9</v>
+      </c>
+      <c r="AX3">
+        <v>7.1</v>
+      </c>
+      <c r="AY3">
+        <v>2.7</v>
+      </c>
+      <c r="AZ3">
+        <v>8.300000000000001</v>
+      </c>
+      <c r="BA3">
+        <v>5</v>
+      </c>
+      <c r="BB3">
+        <v>6.4</v>
+      </c>
+      <c r="BC3">
+        <v>0.8</v>
+      </c>
+      <c r="BD3">
+        <v>0.9399999999999999</v>
+      </c>
+      <c r="BE3">
+        <v>1.03</v>
+      </c>
+      <c r="BF3">
         <v>0.98</v>
       </c>
-      <c r="AE3">
-        <v>0.7</v>
-      </c>
-      <c r="AF3">
-        <v>1.6</v>
-      </c>
-      <c r="AG3">
-        <v>1.6</v>
-      </c>
-      <c r="AH3" t="s">
-        <v>63</v>
-      </c>
-      <c r="AI3">
-        <v>84.40000000000001</v>
-      </c>
-      <c r="AJ3">
-        <v>86</v>
-      </c>
-      <c r="AK3">
-        <v>70.40000000000001</v>
-      </c>
-      <c r="AL3">
-        <v>64.3</v>
-      </c>
-      <c r="AM3">
-        <v>1012</v>
-      </c>
-      <c r="AN3">
-        <v>1014.2</v>
-      </c>
-      <c r="AO3">
-        <v>0</v>
-      </c>
-      <c r="AP3">
-        <v>0</v>
-      </c>
-      <c r="AQ3">
-        <v>0</v>
-      </c>
-      <c r="AR3">
-        <v>37.7</v>
-      </c>
-      <c r="AS3">
-        <v>1614</v>
-      </c>
-      <c r="AT3">
-        <v>9</v>
-      </c>
-      <c r="AU3">
-        <v>17.7</v>
-      </c>
-      <c r="AV3" t="s">
-        <v>65</v>
-      </c>
-      <c r="AW3">
-        <v>224.9</v>
-      </c>
-      <c r="AX3">
-        <v>7.3</v>
-      </c>
-      <c r="AY3">
-        <v>3.1</v>
-      </c>
-      <c r="AZ3">
-        <v>9</v>
-      </c>
-      <c r="BA3">
-        <v>7.2</v>
-      </c>
-      <c r="BB3">
-        <v>2.8</v>
-      </c>
-      <c r="BC3">
-        <v>8.300000000000001</v>
-      </c>
-      <c r="BD3">
-        <v>5</v>
-      </c>
-      <c r="BE3">
-        <v>6.5</v>
-      </c>
-      <c r="BF3">
-        <v>0.8</v>
-      </c>
       <c r="BG3">
-        <v>0.9399999999999999</v>
+        <v>0.09</v>
       </c>
       <c r="BH3">
-        <v>1.03</v>
-      </c>
-      <c r="BI3">
-        <v>0.98</v>
+        <v>1.1555</v>
+      </c>
+      <c r="BI3" t="s">
+        <v>156</v>
       </c>
       <c r="BJ3">
-        <v>0.09</v>
-      </c>
-      <c r="BK3">
-        <v>1.1553</v>
+        <v>1711</v>
+      </c>
+      <c r="BK3" t="s">
+        <v>59</v>
       </c>
       <c r="BL3" t="s">
-        <v>163</v>
+        <v>60</v>
       </c>
       <c r="BM3">
-        <v>1720</v>
-      </c>
-      <c r="BN3" t="s">
-        <v>61</v>
-      </c>
-      <c r="BO3" t="s">
-        <v>62</v>
+        <v>81.7</v>
+      </c>
+      <c r="BN3">
+        <v>1.076</v>
+      </c>
+      <c r="BO3">
+        <v>83.40000000000001</v>
       </c>
       <c r="BP3">
-        <v>81.90000000000001</v>
+        <v>78.3</v>
       </c>
       <c r="BQ3">
-        <v>1.077</v>
+        <v>59.4</v>
       </c>
       <c r="BR3">
-        <v>83.59999999999999</v>
+        <v>57.8</v>
       </c>
       <c r="BS3">
-        <v>78.59999999999999</v>
+        <v>52.4</v>
       </c>
       <c r="BT3">
-        <v>59.4</v>
-      </c>
-      <c r="BU3">
-        <v>57.8</v>
+        <v>12</v>
+      </c>
+      <c r="BU3" t="s">
+        <v>69</v>
       </c>
       <c r="BV3">
-        <v>52.2</v>
-      </c>
-      <c r="BW3">
-        <v>12</v>
-      </c>
-      <c r="BX3" t="s">
-        <v>72</v>
+        <v>15.1</v>
+      </c>
+      <c r="BW3" t="s">
+        <v>69</v>
+      </c>
+      <c r="BX3">
+        <v>87</v>
       </c>
       <c r="BY3">
-        <v>14.6</v>
-      </c>
-      <c r="BZ3" t="s">
-        <v>72</v>
+        <v>81.09999999999999</v>
+      </c>
+      <c r="BZ3">
+        <v>10</v>
       </c>
       <c r="CA3">
-        <v>87</v>
-      </c>
-      <c r="CB3">
-        <v>81.3</v>
-      </c>
-      <c r="CC3">
-        <v>10</v>
-      </c>
-      <c r="CD3">
         <v>8.4</v>
       </c>
     </row>
-    <row r="4" spans="1:85">
+    <row r="4" spans="1:79">
       <c r="A4" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="B4" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="C4" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="D4" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="E4" t="s">
-        <v>150</v>
+        <v>143</v>
       </c>
       <c r="F4" t="s">
-        <v>153</v>
+        <v>146</v>
       </c>
       <c r="G4" t="s">
-        <v>155</v>
+        <v>148</v>
       </c>
       <c r="H4" t="s">
-        <v>73</v>
+        <v>70</v>
       </c>
       <c r="I4" t="s">
-        <v>156</v>
+        <v>149</v>
       </c>
       <c r="J4">
-        <v>183</v>
+        <v>188.3</v>
       </c>
       <c r="K4">
-        <v>1</v>
+        <v>0.9</v>
       </c>
       <c r="L4">
         <v>5</v>
       </c>
       <c r="M4">
-        <v>1.37</v>
+        <v>1.09</v>
       </c>
       <c r="N4">
-        <v>1.3</v>
+        <v>0.92</v>
       </c>
       <c r="O4">
         <v>0</v>
       </c>
       <c r="P4">
-        <v>3.3</v>
+        <v>4.3</v>
       </c>
       <c r="Q4">
-        <v>0.6</v>
+        <v>0.2</v>
       </c>
       <c r="R4">
         <v>100</v>
@@ -2272,246 +2180,237 @@
         <v>0</v>
       </c>
       <c r="T4" t="s">
-        <v>157</v>
+        <v>150</v>
       </c>
       <c r="U4" t="s">
-        <v>160</v>
+        <v>153</v>
       </c>
       <c r="V4" t="s">
-        <v>161</v>
+        <v>154</v>
       </c>
       <c r="W4">
         <v>1</v>
       </c>
       <c r="X4">
-        <v>0.8506</v>
+        <v>7.1</v>
       </c>
       <c r="Y4">
-        <v>0.02</v>
+        <v>89.09999999999999</v>
       </c>
       <c r="Z4">
-        <v>0.01</v>
+        <v>76.5</v>
       </c>
       <c r="AA4">
-        <v>9.4</v>
+        <v>0.98</v>
       </c>
       <c r="AB4">
-        <v>88.5</v>
+        <v>0.7</v>
       </c>
       <c r="AC4">
-        <v>76.5</v>
+        <v>1.6</v>
       </c>
       <c r="AD4">
+        <v>1.6</v>
+      </c>
+      <c r="AE4" t="s">
+        <v>61</v>
+      </c>
+      <c r="AF4">
+        <v>82.7</v>
+      </c>
+      <c r="AG4">
+        <v>84.8</v>
+      </c>
+      <c r="AH4">
+        <v>70</v>
+      </c>
+      <c r="AI4">
+        <v>66.7</v>
+      </c>
+      <c r="AJ4">
+        <v>1012</v>
+      </c>
+      <c r="AK4">
+        <v>1014.3</v>
+      </c>
+      <c r="AL4">
+        <v>0</v>
+      </c>
+      <c r="AM4">
+        <v>0</v>
+      </c>
+      <c r="AN4">
+        <v>0</v>
+      </c>
+      <c r="AO4">
+        <v>37.1</v>
+      </c>
+      <c r="AP4">
+        <v>1469</v>
+      </c>
+      <c r="AQ4">
+        <v>8.800000000000001</v>
+      </c>
+      <c r="AR4">
+        <v>16.6</v>
+      </c>
+      <c r="AS4" t="s">
+        <v>63</v>
+      </c>
+      <c r="AT4">
+        <v>228.8</v>
+      </c>
+      <c r="AU4">
+        <v>6.9</v>
+      </c>
+      <c r="AV4">
+        <v>2.5</v>
+      </c>
+      <c r="AW4">
+        <v>8.800000000000001</v>
+      </c>
+      <c r="AX4">
+        <v>6.7</v>
+      </c>
+      <c r="AY4">
+        <v>2.2</v>
+      </c>
+      <c r="AZ4">
+        <v>8.199999999999999</v>
+      </c>
+      <c r="BA4">
+        <v>5.4</v>
+      </c>
+      <c r="BB4">
+        <v>6</v>
+      </c>
+      <c r="BC4">
+        <v>0.8</v>
+      </c>
+      <c r="BD4">
+        <v>0.9399999999999999</v>
+      </c>
+      <c r="BE4">
+        <v>1.03</v>
+      </c>
+      <c r="BF4">
         <v>0.98</v>
       </c>
-      <c r="AE4">
-        <v>0.7</v>
-      </c>
-      <c r="AF4">
-        <v>1.6</v>
-      </c>
-      <c r="AG4">
-        <v>1.6</v>
-      </c>
-      <c r="AH4" t="s">
-        <v>63</v>
-      </c>
-      <c r="AI4">
-        <v>82.8</v>
-      </c>
-      <c r="AJ4">
-        <v>84.8</v>
-      </c>
-      <c r="AK4">
-        <v>69.7</v>
-      </c>
-      <c r="AL4">
-        <v>66</v>
-      </c>
-      <c r="AM4">
-        <v>1012</v>
-      </c>
-      <c r="AN4">
-        <v>1014.3</v>
-      </c>
-      <c r="AO4">
-        <v>0</v>
-      </c>
-      <c r="AP4">
-        <v>0</v>
-      </c>
-      <c r="AQ4">
-        <v>0</v>
-      </c>
-      <c r="AR4">
-        <v>37.1</v>
-      </c>
-      <c r="AS4">
-        <v>1407</v>
-      </c>
-      <c r="AT4">
-        <v>8.9</v>
-      </c>
-      <c r="AU4">
-        <v>17.1</v>
-      </c>
-      <c r="AV4" t="s">
-        <v>65</v>
-      </c>
-      <c r="AW4">
-        <v>229.9</v>
-      </c>
-      <c r="AX4">
-        <v>6.9</v>
-      </c>
-      <c r="AY4">
-        <v>2.3</v>
-      </c>
-      <c r="AZ4">
-        <v>8.9</v>
-      </c>
-      <c r="BA4">
-        <v>6.7</v>
-      </c>
-      <c r="BB4">
-        <v>2.1</v>
-      </c>
-      <c r="BC4">
-        <v>8.300000000000001</v>
-      </c>
-      <c r="BD4">
-        <v>5.6</v>
-      </c>
-      <c r="BE4">
-        <v>6</v>
-      </c>
-      <c r="BF4">
-        <v>0.8</v>
-      </c>
       <c r="BG4">
-        <v>0.9399999999999999</v>
+        <v>0.09</v>
       </c>
       <c r="BH4">
-        <v>1.03</v>
-      </c>
-      <c r="BI4">
-        <v>0.98</v>
+        <v>1.1591</v>
+      </c>
+      <c r="BI4" t="s">
+        <v>156</v>
       </c>
       <c r="BJ4">
-        <v>0.09</v>
-      </c>
-      <c r="BK4">
-        <v>1.159</v>
+        <v>1607</v>
+      </c>
+      <c r="BK4" t="s">
+        <v>59</v>
       </c>
       <c r="BL4" t="s">
-        <v>163</v>
+        <v>60</v>
       </c>
       <c r="BM4">
-        <v>1613</v>
-      </c>
-      <c r="BN4" t="s">
-        <v>61</v>
-      </c>
-      <c r="BO4" t="s">
-        <v>62</v>
+        <v>79.7</v>
+      </c>
+      <c r="BN4">
+        <v>1.071</v>
+      </c>
+      <c r="BO4">
+        <v>81.7</v>
       </c>
       <c r="BP4">
-        <v>79.90000000000001</v>
+        <v>76.3</v>
       </c>
       <c r="BQ4">
-        <v>1.072</v>
+        <v>59</v>
       </c>
       <c r="BR4">
-        <v>81.90000000000001</v>
+        <v>57.2</v>
       </c>
       <c r="BS4">
-        <v>76.3</v>
+        <v>55.2</v>
       </c>
       <c r="BT4">
-        <v>59.1</v>
-      </c>
-      <c r="BU4">
-        <v>57.2</v>
+        <v>12</v>
+      </c>
+      <c r="BU4" t="s">
+        <v>69</v>
       </c>
       <c r="BV4">
+        <v>14</v>
+      </c>
+      <c r="BW4" t="s">
+        <v>69</v>
+      </c>
+      <c r="BX4">
+        <v>85</v>
+      </c>
+      <c r="BY4">
+        <v>79.8</v>
+      </c>
+      <c r="BZ4">
+        <v>10</v>
+      </c>
+      <c r="CA4">
+        <v>8.199999999999999</v>
+      </c>
+    </row>
+    <row r="5" spans="1:79">
+      <c r="A5" t="s">
         <v>55</v>
       </c>
-      <c r="BW4">
-        <v>12</v>
-      </c>
-      <c r="BX4" t="s">
-        <v>72</v>
-      </c>
-      <c r="BY4">
-        <v>13.2</v>
-      </c>
-      <c r="BZ4" t="s">
-        <v>72</v>
-      </c>
-      <c r="CA4">
-        <v>85</v>
-      </c>
-      <c r="CB4">
-        <v>80</v>
-      </c>
-      <c r="CC4">
-        <v>10</v>
-      </c>
-      <c r="CD4">
-        <v>8.4</v>
-      </c>
-    </row>
-    <row r="5" spans="1:85">
-      <c r="A5" t="s">
-        <v>57</v>
-      </c>
       <c r="B5" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="C5" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="D5" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="E5" t="s">
-        <v>151</v>
+        <v>144</v>
       </c>
       <c r="F5" t="s">
-        <v>154</v>
+        <v>147</v>
       </c>
       <c r="G5" t="s">
-        <v>155</v>
+        <v>148</v>
       </c>
       <c r="H5" t="s">
-        <v>73</v>
+        <v>70</v>
       </c>
       <c r="I5" t="s">
-        <v>156</v>
+        <v>149</v>
       </c>
       <c r="J5">
-        <v>183</v>
+        <v>188.3</v>
       </c>
       <c r="K5">
-        <v>2</v>
+        <v>1.9</v>
       </c>
       <c r="L5">
         <v>5</v>
       </c>
       <c r="M5">
-        <v>1.1</v>
+        <v>0.78</v>
       </c>
       <c r="N5">
-        <v>1.39</v>
+        <v>0.96</v>
       </c>
       <c r="O5">
         <v>0</v>
       </c>
       <c r="P5">
-        <v>5</v>
+        <v>5.8</v>
       </c>
       <c r="Q5">
-        <v>0.4</v>
+        <v>0.1</v>
       </c>
       <c r="R5">
         <v>100</v>
@@ -2520,197 +2419,188 @@
         <v>0</v>
       </c>
       <c r="T5" t="s">
-        <v>157</v>
+        <v>150</v>
       </c>
       <c r="U5" t="s">
-        <v>161</v>
+        <v>154</v>
       </c>
       <c r="V5" t="s">
-        <v>162</v>
+        <v>155</v>
       </c>
       <c r="W5">
         <v>1</v>
       </c>
       <c r="X5">
-        <v>0.72</v>
+        <v>6</v>
       </c>
       <c r="Y5">
-        <v>0.02</v>
+        <v>91.7</v>
       </c>
       <c r="Z5">
-        <v>0.01</v>
+        <v>76</v>
       </c>
       <c r="AA5">
-        <v>8.5</v>
+        <v>0.98</v>
       </c>
       <c r="AB5">
-        <v>91</v>
+        <v>0.7</v>
       </c>
       <c r="AC5">
-        <v>75.90000000000001</v>
+        <v>1.6</v>
       </c>
       <c r="AD5">
+        <v>1.6</v>
+      </c>
+      <c r="AE5" t="s">
+        <v>61</v>
+      </c>
+      <c r="AF5">
+        <v>80.90000000000001</v>
+      </c>
+      <c r="AG5">
+        <v>84.5</v>
+      </c>
+      <c r="AH5">
+        <v>70</v>
+      </c>
+      <c r="AI5">
+        <v>70.59999999999999</v>
+      </c>
+      <c r="AJ5">
+        <v>1012.3</v>
+      </c>
+      <c r="AK5">
+        <v>1014.6</v>
+      </c>
+      <c r="AL5">
+        <v>0</v>
+      </c>
+      <c r="AM5">
+        <v>0</v>
+      </c>
+      <c r="AN5">
+        <v>0</v>
+      </c>
+      <c r="AO5">
+        <v>35.1</v>
+      </c>
+      <c r="AP5">
+        <v>1399</v>
+      </c>
+      <c r="AQ5">
+        <v>8.699999999999999</v>
+      </c>
+      <c r="AR5">
+        <v>16.2</v>
+      </c>
+      <c r="AS5" t="s">
+        <v>63</v>
+      </c>
+      <c r="AT5">
+        <v>229.2</v>
+      </c>
+      <c r="AU5">
+        <v>6.8</v>
+      </c>
+      <c r="AV5">
+        <v>2.4</v>
+      </c>
+      <c r="AW5">
+        <v>8.699999999999999</v>
+      </c>
+      <c r="AX5">
+        <v>6.6</v>
+      </c>
+      <c r="AY5">
+        <v>2.1</v>
+      </c>
+      <c r="AZ5">
+        <v>8.1</v>
+      </c>
+      <c r="BA5">
+        <v>5.4</v>
+      </c>
+      <c r="BB5">
+        <v>5.9</v>
+      </c>
+      <c r="BC5">
+        <v>0.8</v>
+      </c>
+      <c r="BD5">
+        <v>0.9399999999999999</v>
+      </c>
+      <c r="BE5">
+        <v>1.03</v>
+      </c>
+      <c r="BF5">
         <v>0.98</v>
       </c>
-      <c r="AE5">
-        <v>0.7</v>
-      </c>
-      <c r="AF5">
-        <v>1.6</v>
-      </c>
-      <c r="AG5">
-        <v>1.6</v>
-      </c>
-      <c r="AH5" t="s">
-        <v>63</v>
-      </c>
-      <c r="AI5">
-        <v>81</v>
-      </c>
-      <c r="AJ5">
-        <v>84.5</v>
-      </c>
-      <c r="AK5">
-        <v>69.7</v>
-      </c>
-      <c r="AL5">
-        <v>69.90000000000001</v>
-      </c>
-      <c r="AM5">
-        <v>1012.3</v>
-      </c>
-      <c r="AN5">
-        <v>1014.6</v>
-      </c>
-      <c r="AO5">
-        <v>0</v>
-      </c>
-      <c r="AP5">
-        <v>0</v>
-      </c>
-      <c r="AQ5">
-        <v>0</v>
-      </c>
-      <c r="AR5">
-        <v>35.1</v>
-      </c>
-      <c r="AS5">
-        <v>1344</v>
-      </c>
-      <c r="AT5">
-        <v>8.9</v>
-      </c>
-      <c r="AU5">
-        <v>16.7</v>
-      </c>
-      <c r="AV5" t="s">
-        <v>65</v>
-      </c>
-      <c r="AW5">
-        <v>230.3</v>
-      </c>
-      <c r="AX5">
-        <v>6.8</v>
-      </c>
-      <c r="AY5">
-        <v>2.3</v>
-      </c>
-      <c r="AZ5">
-        <v>8.800000000000001</v>
-      </c>
-      <c r="BA5">
-        <v>6.6</v>
-      </c>
-      <c r="BB5">
-        <v>2</v>
-      </c>
-      <c r="BC5">
-        <v>8.199999999999999</v>
-      </c>
-      <c r="BD5">
-        <v>5.6</v>
-      </c>
-      <c r="BE5">
-        <v>5.9</v>
-      </c>
-      <c r="BF5">
-        <v>0.8</v>
-      </c>
       <c r="BG5">
-        <v>0.9399999999999999</v>
+        <v>0.09</v>
       </c>
       <c r="BH5">
-        <v>1.03</v>
-      </c>
-      <c r="BI5">
-        <v>0.98</v>
+        <v>1.1632</v>
+      </c>
+      <c r="BI5" t="s">
+        <v>157</v>
       </c>
       <c r="BJ5">
-        <v>0.09</v>
-      </c>
-      <c r="BK5">
-        <v>1.1631</v>
+        <v>1480</v>
+      </c>
+      <c r="BK5" t="s">
+        <v>59</v>
       </c>
       <c r="BL5" t="s">
-        <v>164</v>
+        <v>60</v>
       </c>
       <c r="BM5">
-        <v>1488</v>
-      </c>
-      <c r="BN5" t="s">
-        <v>61</v>
-      </c>
-      <c r="BO5" t="s">
-        <v>62</v>
+        <v>78.3</v>
+      </c>
+      <c r="BN5">
+        <v>1.068</v>
+      </c>
+      <c r="BO5">
+        <v>80.3</v>
       </c>
       <c r="BP5">
-        <v>78.5</v>
+        <v>74.90000000000001</v>
       </c>
       <c r="BQ5">
-        <v>1.068</v>
+        <v>58.6</v>
       </c>
       <c r="BR5">
-        <v>80.59999999999999</v>
+        <v>56.7</v>
       </c>
       <c r="BS5">
-        <v>75</v>
+        <v>57.6</v>
       </c>
       <c r="BT5">
-        <v>58.7</v>
-      </c>
-      <c r="BU5">
-        <v>56.7</v>
+        <v>12</v>
+      </c>
+      <c r="BU5" t="s">
+        <v>69</v>
       </c>
       <c r="BV5">
-        <v>57.2</v>
-      </c>
-      <c r="BW5">
-        <v>12</v>
-      </c>
-      <c r="BX5" t="s">
-        <v>72</v>
+        <v>10.3</v>
+      </c>
+      <c r="BW5" t="s">
+        <v>69</v>
+      </c>
+      <c r="BX5">
+        <v>82</v>
       </c>
       <c r="BY5">
-        <v>9.4</v>
-      </c>
-      <c r="BZ5" t="s">
-        <v>72</v>
+        <v>78.90000000000001</v>
+      </c>
+      <c r="BZ5">
+        <v>10</v>
       </c>
       <c r="CA5">
-        <v>82</v>
-      </c>
-      <c r="CB5">
-        <v>79.09999999999999</v>
-      </c>
-      <c r="CC5">
-        <v>10</v>
-      </c>
-      <c r="CD5">
-        <v>8.300000000000001</v>
+        <v>8</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:CG5"/>
+  <autoFilter ref="A1:CA5"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
@@ -2787,60 +2677,60 @@
         <v>7</v>
       </c>
       <c r="P1" s="1" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="Q1" s="1" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
     </row>
     <row r="2" spans="1:17">
       <c r="A2" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="B2" t="s">
+        <v>54</v>
+      </c>
+      <c r="C2" t="s">
         <v>56</v>
       </c>
-      <c r="C2" t="s">
+      <c r="D2" t="s">
         <v>58</v>
       </c>
-      <c r="D2" t="s">
-        <v>60</v>
-      </c>
       <c r="E2">
-        <v>61.7</v>
+        <v>62.7</v>
       </c>
       <c r="F2" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="G2">
-        <v>93.09999999999999</v>
+        <v>90.5</v>
       </c>
       <c r="H2">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="I2">
+        <v>6</v>
+      </c>
+      <c r="J2">
+        <v>3.8</v>
+      </c>
+      <c r="K2">
         <v>5</v>
       </c>
-      <c r="J2">
-        <v>3.5</v>
-      </c>
-      <c r="K2">
-        <v>4</v>
-      </c>
       <c r="L2" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="M2">
-        <v>85.2</v>
+        <v>84.2</v>
       </c>
       <c r="N2">
-        <v>1771</v>
+        <v>1710</v>
       </c>
       <c r="O2" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="P2" t="s">
-        <v>72</v>
+        <v>69</v>
       </c>
       <c r="Q2">
         <v>5</v>

</xml_diff>

<commit_message>
Update MLB weather 2026-07-14 07:50 PM PT
</commit_message>
<xml_diff>
--- a/mlb_weather_professional_v4_2026_07_14.xlsx
+++ b/mlb_weather_professional_v4_2026_07_14.xlsx
@@ -209,7 +209,7 @@
     <t>Clear</t>
   </si>
   <si>
-    <t>🟢 8.7 mph Out to RF</t>
+    <t>🟢 8.8 mph Out to RF</t>
   </si>
   <si>
     <t>SW</t>
@@ -221,7 +221,7 @@
     <t>B+</t>
   </si>
   <si>
-    <t>Density 79 | Wind 64 | Temp 63 | Altitude 62 | Confidence 90%</t>
+    <t>Density 79 | Wind 65 | Temp 62 | Altitude 62 | Confidence 93%</t>
   </si>
   <si>
     <t>🟢 Good</t>
@@ -233,7 +233,7 @@
     <t>LOW</t>
   </si>
   <si>
-    <t>2026-07-14 06:07:02 PM PDT</t>
+    <t>2026-07-14 07:50:23 PM PDT</t>
   </si>
   <si>
     <t>Period</t>
@@ -467,7 +467,7 @@
     <t>11:00 PM EDT</t>
   </si>
   <si>
-    <t>2026-07-15 01:07:02 UTC</t>
+    <t>2026-07-15 02:50:23 UTC</t>
   </si>
   <si>
     <t>2026-07-14T21:58:43+00:00</t>
@@ -1179,10 +1179,10 @@
         <v>61</v>
       </c>
       <c r="K2">
-        <v>85.8</v>
+        <v>85.5</v>
       </c>
       <c r="L2">
-        <v>60.4</v>
+        <v>60.3</v>
       </c>
       <c r="M2" t="s">
         <v>62</v>
@@ -1194,13 +1194,13 @@
         <v>63</v>
       </c>
       <c r="P2">
-        <v>2.8</v>
+        <v>2.9</v>
       </c>
       <c r="Q2">
-        <v>7.5</v>
+        <v>7.6</v>
       </c>
       <c r="R2">
-        <v>8.699999999999999</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="T2" t="s">
         <v>64</v>
@@ -1227,13 +1227,13 @@
         <v>3.8</v>
       </c>
       <c r="AB2">
-        <v>90.5</v>
+        <v>93.40000000000001</v>
       </c>
       <c r="AC2" t="s">
         <v>67</v>
       </c>
       <c r="AD2">
-        <v>6.4</v>
+        <v>6.5</v>
       </c>
       <c r="AE2">
         <v>5</v>
@@ -1245,34 +1245,34 @@
         <v>0</v>
       </c>
       <c r="AH2">
-        <v>4.8</v>
+        <v>4.7</v>
       </c>
       <c r="AI2">
-        <v>0.4</v>
+        <v>0.5</v>
       </c>
       <c r="AJ2">
-        <v>1.1557</v>
+        <v>1.1569</v>
       </c>
       <c r="AK2">
-        <v>1710</v>
+        <v>1684</v>
       </c>
       <c r="AL2">
-        <v>1012</v>
+        <v>1012.2</v>
       </c>
       <c r="AM2">
-        <v>70.2</v>
+        <v>69.3</v>
       </c>
       <c r="AN2">
-        <v>84.2</v>
+        <v>83.90000000000001</v>
       </c>
       <c r="AO2">
-        <v>64.09999999999999</v>
+        <v>62.5</v>
       </c>
       <c r="AP2" t="s">
         <v>68</v>
       </c>
       <c r="AQ2">
-        <v>17.2</v>
+        <v>17.3</v>
       </c>
       <c r="AR2">
         <v>0</v>
@@ -1290,13 +1290,13 @@
         <v>69</v>
       </c>
       <c r="AW2">
-        <v>15.1</v>
+        <v>13.3</v>
       </c>
       <c r="AX2" t="s">
         <v>70</v>
       </c>
       <c r="AY2">
-        <v>188.3</v>
+        <v>291.7</v>
       </c>
       <c r="AZ2">
         <v>5</v>
@@ -1672,7 +1672,7 @@
         <v>149</v>
       </c>
       <c r="J2">
-        <v>188.3</v>
+        <v>291.7</v>
       </c>
       <c r="K2">
         <v>0</v>
@@ -1681,19 +1681,19 @@
         <v>5</v>
       </c>
       <c r="M2">
-        <v>0.99</v>
+        <v>0.44</v>
       </c>
       <c r="N2">
-        <v>0.5600000000000001</v>
+        <v>0.58</v>
       </c>
       <c r="O2">
         <v>0</v>
       </c>
       <c r="P2">
-        <v>4.4</v>
+        <v>5.4</v>
       </c>
       <c r="Q2">
-        <v>0.5</v>
+        <v>0.6</v>
       </c>
       <c r="R2">
         <v>100</v>
@@ -1714,13 +1714,13 @@
         <v>1</v>
       </c>
       <c r="X2">
-        <v>5.7</v>
+        <v>3.5</v>
       </c>
       <c r="Y2">
-        <v>93</v>
+        <v>97.2</v>
       </c>
       <c r="Z2">
-        <v>81.7</v>
+        <v>82.90000000000001</v>
       </c>
       <c r="AA2">
         <v>0.98</v>
@@ -1738,22 +1738,22 @@
         <v>61</v>
       </c>
       <c r="AF2">
-        <v>85.8</v>
+        <v>85.5</v>
       </c>
       <c r="AG2">
-        <v>88.09999999999999</v>
+        <v>89.7</v>
       </c>
       <c r="AH2">
-        <v>70.09999999999999</v>
+        <v>69.90000000000001</v>
       </c>
       <c r="AI2">
-        <v>60.4</v>
+        <v>60.3</v>
       </c>
       <c r="AJ2">
-        <v>1011.9</v>
+        <v>1012.4</v>
       </c>
       <c r="AK2">
-        <v>1014.1</v>
+        <v>1014.7</v>
       </c>
       <c r="AL2">
         <v>0</v>
@@ -1765,46 +1765,46 @@
         <v>0</v>
       </c>
       <c r="AO2">
-        <v>49.3</v>
+        <v>54.6</v>
       </c>
       <c r="AP2">
-        <v>1542</v>
+        <v>1688</v>
       </c>
       <c r="AQ2">
         <v>9.4</v>
       </c>
       <c r="AR2">
-        <v>21.4</v>
+        <v>20.8</v>
       </c>
       <c r="AS2" t="s">
         <v>63</v>
       </c>
       <c r="AT2">
-        <v>225.5</v>
+        <v>224.8</v>
       </c>
       <c r="AU2">
-        <v>7.6</v>
+        <v>7.7</v>
       </c>
       <c r="AV2">
-        <v>3.1</v>
+        <v>3.3</v>
       </c>
       <c r="AW2">
         <v>9.4</v>
       </c>
       <c r="AX2">
-        <v>7.5</v>
+        <v>7.6</v>
       </c>
       <c r="AY2">
-        <v>2.8</v>
+        <v>2.9</v>
       </c>
       <c r="AZ2">
-        <v>8.699999999999999</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="BA2">
-        <v>5.3</v>
+        <v>5.2</v>
       </c>
       <c r="BB2">
-        <v>6.7</v>
+        <v>6.8</v>
       </c>
       <c r="BC2">
         <v>0.8</v>
@@ -1822,13 +1822,13 @@
         <v>0.09</v>
       </c>
       <c r="BH2">
-        <v>1.1523</v>
+        <v>1.1536</v>
       </c>
       <c r="BI2" t="s">
         <v>156</v>
       </c>
       <c r="BJ2">
-        <v>1817</v>
+        <v>1779</v>
       </c>
       <c r="BK2" t="s">
         <v>59</v>
@@ -1837,25 +1837,25 @@
         <v>60</v>
       </c>
       <c r="BM2">
-        <v>84.09999999999999</v>
+        <v>83.90000000000001</v>
       </c>
       <c r="BN2">
-        <v>1.082</v>
+        <v>1.081</v>
       </c>
       <c r="BO2">
-        <v>85.90000000000001</v>
+        <v>85.7</v>
       </c>
       <c r="BP2">
-        <v>80.59999999999999</v>
+        <v>80.40000000000001</v>
       </c>
       <c r="BQ2">
         <v>60</v>
       </c>
       <c r="BR2">
-        <v>58.2</v>
+        <v>58.1</v>
       </c>
       <c r="BS2">
-        <v>47.9</v>
+        <v>48.9</v>
       </c>
       <c r="BT2">
         <v>12</v>
@@ -1864,16 +1864,16 @@
         <v>69</v>
       </c>
       <c r="BV2">
-        <v>8.1</v>
+        <v>2.2</v>
       </c>
       <c r="BW2" t="s">
         <v>69</v>
       </c>
       <c r="BX2">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="BY2">
-        <v>83.8</v>
+        <v>84.7</v>
       </c>
       <c r="BZ2">
         <v>10</v>
@@ -1911,7 +1911,7 @@
         <v>149</v>
       </c>
       <c r="J3">
-        <v>188.3</v>
+        <v>291.7</v>
       </c>
       <c r="K3">
         <v>0</v>
@@ -1920,19 +1920,19 @@
         <v>5</v>
       </c>
       <c r="M3">
-        <v>1.43</v>
+        <v>0.68</v>
       </c>
       <c r="N3">
-        <v>0.99</v>
+        <v>1.02</v>
       </c>
       <c r="O3">
         <v>0</v>
       </c>
       <c r="P3">
-        <v>5.2</v>
+        <v>3.3</v>
       </c>
       <c r="Q3">
-        <v>0.6</v>
+        <v>0.5</v>
       </c>
       <c r="R3">
         <v>100</v>
@@ -1953,13 +1953,13 @@
         <v>1</v>
       </c>
       <c r="X3">
-        <v>8.699999999999999</v>
+        <v>5.8</v>
       </c>
       <c r="Y3">
-        <v>87.8</v>
+        <v>92</v>
       </c>
       <c r="Z3">
-        <v>77.8</v>
+        <v>79.3</v>
       </c>
       <c r="AA3">
         <v>0.98</v>
@@ -1977,22 +1977,22 @@
         <v>61</v>
       </c>
       <c r="AF3">
-        <v>84.2</v>
+        <v>83.90000000000001</v>
       </c>
       <c r="AG3">
-        <v>86</v>
+        <v>86.09999999999999</v>
       </c>
       <c r="AH3">
-        <v>70.59999999999999</v>
+        <v>69.2</v>
       </c>
       <c r="AI3">
-        <v>65.09999999999999</v>
+        <v>62.3</v>
       </c>
       <c r="AJ3">
-        <v>1011.9</v>
+        <v>1012.4</v>
       </c>
       <c r="AK3">
-        <v>1014.2</v>
+        <v>1014.7</v>
       </c>
       <c r="AL3">
         <v>0</v>
@@ -2004,46 +2004,46 @@
         <v>0</v>
       </c>
       <c r="AO3">
-        <v>37.7</v>
+        <v>52</v>
       </c>
       <c r="AP3">
-        <v>1677</v>
+        <v>1300</v>
       </c>
       <c r="AQ3">
-        <v>8.9</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="AR3">
-        <v>17.3</v>
+        <v>21.7</v>
       </c>
       <c r="AS3" t="s">
         <v>63</v>
       </c>
       <c r="AT3">
-        <v>225.2</v>
+        <v>226.5</v>
       </c>
       <c r="AU3">
-        <v>7.3</v>
+        <v>7.1</v>
       </c>
       <c r="AV3">
-        <v>3</v>
+        <v>2.8</v>
       </c>
       <c r="AW3">
-        <v>8.9</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="AX3">
-        <v>7.1</v>
+        <v>7</v>
       </c>
       <c r="AY3">
-        <v>2.7</v>
+        <v>2.5</v>
       </c>
       <c r="AZ3">
-        <v>8.300000000000001</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="BA3">
-        <v>5</v>
+        <v>5.1</v>
       </c>
       <c r="BB3">
-        <v>6.4</v>
+        <v>6.2</v>
       </c>
       <c r="BC3">
         <v>0.8</v>
@@ -2061,13 +2061,13 @@
         <v>0.09</v>
       </c>
       <c r="BH3">
-        <v>1.1555</v>
+        <v>1.1573</v>
       </c>
       <c r="BI3" t="s">
         <v>156</v>
       </c>
       <c r="BJ3">
-        <v>1711</v>
+        <v>1673</v>
       </c>
       <c r="BK3" t="s">
         <v>59</v>
@@ -2076,25 +2076,25 @@
         <v>60</v>
       </c>
       <c r="BM3">
-        <v>81.7</v>
+        <v>81.90000000000001</v>
       </c>
       <c r="BN3">
-        <v>1.076</v>
+        <v>1.077</v>
       </c>
       <c r="BO3">
-        <v>83.40000000000001</v>
+        <v>83.7</v>
       </c>
       <c r="BP3">
-        <v>78.3</v>
+        <v>78.5</v>
       </c>
       <c r="BQ3">
-        <v>59.4</v>
+        <v>59.2</v>
       </c>
       <c r="BR3">
-        <v>57.8</v>
+        <v>57.4</v>
       </c>
       <c r="BS3">
-        <v>52.4</v>
+        <v>50.6</v>
       </c>
       <c r="BT3">
         <v>12</v>
@@ -2103,22 +2103,22 @@
         <v>69</v>
       </c>
       <c r="BV3">
-        <v>15.1</v>
+        <v>9.800000000000001</v>
       </c>
       <c r="BW3" t="s">
         <v>69</v>
       </c>
       <c r="BX3">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="BY3">
-        <v>81.09999999999999</v>
+        <v>81.90000000000001</v>
       </c>
       <c r="BZ3">
         <v>10</v>
       </c>
       <c r="CA3">
-        <v>8.4</v>
+        <v>8.199999999999999</v>
       </c>
     </row>
     <row r="4" spans="1:79">
@@ -2150,28 +2150,28 @@
         <v>149</v>
       </c>
       <c r="J4">
-        <v>188.3</v>
+        <v>291.7</v>
       </c>
       <c r="K4">
-        <v>0.9</v>
+        <v>0</v>
       </c>
       <c r="L4">
         <v>5</v>
       </c>
       <c r="M4">
-        <v>1.09</v>
+        <v>1.33</v>
       </c>
       <c r="N4">
-        <v>0.92</v>
+        <v>0.87</v>
       </c>
       <c r="O4">
         <v>0</v>
       </c>
       <c r="P4">
-        <v>4.3</v>
+        <v>4.6</v>
       </c>
       <c r="Q4">
-        <v>0.2</v>
+        <v>0.3</v>
       </c>
       <c r="R4">
         <v>100</v>
@@ -2192,13 +2192,13 @@
         <v>1</v>
       </c>
       <c r="X4">
-        <v>7.1</v>
+        <v>7.9</v>
       </c>
       <c r="Y4">
         <v>89.09999999999999</v>
       </c>
       <c r="Z4">
-        <v>76.5</v>
+        <v>77.2</v>
       </c>
       <c r="AA4">
         <v>0.98</v>
@@ -2216,22 +2216,22 @@
         <v>61</v>
       </c>
       <c r="AF4">
-        <v>82.7</v>
+        <v>82.5</v>
       </c>
       <c r="AG4">
-        <v>84.8</v>
+        <v>82</v>
       </c>
       <c r="AH4">
-        <v>70</v>
+        <v>68.7</v>
       </c>
       <c r="AI4">
-        <v>66.7</v>
+        <v>64.5</v>
       </c>
       <c r="AJ4">
-        <v>1012</v>
+        <v>1011.7</v>
       </c>
       <c r="AK4">
-        <v>1014.3</v>
+        <v>1014</v>
       </c>
       <c r="AL4">
         <v>0</v>
@@ -2243,46 +2243,46 @@
         <v>0</v>
       </c>
       <c r="AO4">
-        <v>37.1</v>
+        <v>45.3</v>
       </c>
       <c r="AP4">
-        <v>1469</v>
+        <v>997</v>
       </c>
       <c r="AQ4">
-        <v>8.800000000000001</v>
+        <v>9.199999999999999</v>
       </c>
       <c r="AR4">
-        <v>16.6</v>
+        <v>17.8</v>
       </c>
       <c r="AS4" t="s">
         <v>63</v>
       </c>
       <c r="AT4">
-        <v>228.8</v>
+        <v>228.2</v>
       </c>
       <c r="AU4">
-        <v>6.9</v>
+        <v>7.2</v>
       </c>
       <c r="AV4">
-        <v>2.5</v>
+        <v>2.7</v>
       </c>
       <c r="AW4">
-        <v>8.800000000000001</v>
+        <v>9.1</v>
       </c>
       <c r="AX4">
-        <v>6.7</v>
+        <v>7.1</v>
       </c>
       <c r="AY4">
-        <v>2.2</v>
+        <v>2.4</v>
       </c>
       <c r="AZ4">
-        <v>8.199999999999999</v>
+        <v>8.5</v>
       </c>
       <c r="BA4">
-        <v>5.4</v>
+        <v>5.5</v>
       </c>
       <c r="BB4">
-        <v>6</v>
+        <v>6.3</v>
       </c>
       <c r="BC4">
         <v>0.8</v>
@@ -2300,7 +2300,7 @@
         <v>0.09</v>
       </c>
       <c r="BH4">
-        <v>1.1591</v>
+        <v>1.1595</v>
       </c>
       <c r="BI4" t="s">
         <v>156</v>
@@ -2315,34 +2315,34 @@
         <v>60</v>
       </c>
       <c r="BM4">
-        <v>79.7</v>
+        <v>80.5</v>
       </c>
       <c r="BN4">
-        <v>1.071</v>
+        <v>1.073</v>
       </c>
       <c r="BO4">
-        <v>81.7</v>
+        <v>82.5</v>
       </c>
       <c r="BP4">
-        <v>76.3</v>
+        <v>77</v>
       </c>
       <c r="BQ4">
-        <v>59</v>
+        <v>59.2</v>
       </c>
       <c r="BR4">
-        <v>57.2</v>
+        <v>57.1</v>
       </c>
       <c r="BS4">
-        <v>55.2</v>
+        <v>55.7</v>
       </c>
       <c r="BT4">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="BU4" t="s">
         <v>69</v>
       </c>
       <c r="BV4">
-        <v>14</v>
+        <v>13.3</v>
       </c>
       <c r="BW4" t="s">
         <v>69</v>
@@ -2351,13 +2351,13 @@
         <v>85</v>
       </c>
       <c r="BY4">
-        <v>79.8</v>
+        <v>79.59999999999999</v>
       </c>
       <c r="BZ4">
         <v>10</v>
       </c>
       <c r="CA4">
-        <v>8.199999999999999</v>
+        <v>8.800000000000001</v>
       </c>
     </row>
     <row r="5" spans="1:79">
@@ -2389,28 +2389,28 @@
         <v>149</v>
       </c>
       <c r="J5">
-        <v>188.3</v>
+        <v>291.7</v>
       </c>
       <c r="K5">
-        <v>1.9</v>
+        <v>0.2</v>
       </c>
       <c r="L5">
         <v>5</v>
       </c>
       <c r="M5">
-        <v>0.78</v>
+        <v>1.16</v>
       </c>
       <c r="N5">
-        <v>0.96</v>
+        <v>0.89</v>
       </c>
       <c r="O5">
         <v>0</v>
       </c>
       <c r="P5">
-        <v>5.8</v>
+        <v>6.6</v>
       </c>
       <c r="Q5">
-        <v>0.1</v>
+        <v>0.3</v>
       </c>
       <c r="R5">
         <v>100</v>
@@ -2431,13 +2431,13 @@
         <v>1</v>
       </c>
       <c r="X5">
-        <v>6</v>
+        <v>7.3</v>
       </c>
       <c r="Y5">
-        <v>91.7</v>
+        <v>91</v>
       </c>
       <c r="Z5">
-        <v>76</v>
+        <v>76.3</v>
       </c>
       <c r="AA5">
         <v>0.98</v>
@@ -2455,22 +2455,22 @@
         <v>61</v>
       </c>
       <c r="AF5">
-        <v>80.90000000000001</v>
+        <v>80.7</v>
       </c>
       <c r="AG5">
-        <v>84.5</v>
+        <v>81.59999999999999</v>
       </c>
       <c r="AH5">
-        <v>70</v>
+        <v>68.59999999999999</v>
       </c>
       <c r="AI5">
-        <v>70.59999999999999</v>
+        <v>68.3</v>
       </c>
       <c r="AJ5">
-        <v>1012.3</v>
+        <v>1011.4</v>
       </c>
       <c r="AK5">
-        <v>1014.6</v>
+        <v>1013.7</v>
       </c>
       <c r="AL5">
         <v>0</v>
@@ -2482,46 +2482,46 @@
         <v>0</v>
       </c>
       <c r="AO5">
-        <v>35.1</v>
+        <v>41.6</v>
       </c>
       <c r="AP5">
-        <v>1399</v>
+        <v>933</v>
       </c>
       <c r="AQ5">
-        <v>8.699999999999999</v>
+        <v>8.9</v>
       </c>
       <c r="AR5">
-        <v>16.2</v>
+        <v>16.7</v>
       </c>
       <c r="AS5" t="s">
         <v>63</v>
       </c>
       <c r="AT5">
-        <v>229.2</v>
+        <v>228.2</v>
       </c>
       <c r="AU5">
-        <v>6.8</v>
+        <v>7</v>
       </c>
       <c r="AV5">
-        <v>2.4</v>
+        <v>2.6</v>
       </c>
       <c r="AW5">
-        <v>8.699999999999999</v>
+        <v>8.9</v>
       </c>
       <c r="AX5">
-        <v>6.6</v>
+        <v>6.9</v>
       </c>
       <c r="AY5">
-        <v>2.1</v>
+        <v>2.3</v>
       </c>
       <c r="AZ5">
-        <v>8.1</v>
+        <v>8.300000000000001</v>
       </c>
       <c r="BA5">
         <v>5.4</v>
       </c>
       <c r="BB5">
-        <v>5.9</v>
+        <v>6.2</v>
       </c>
       <c r="BC5">
         <v>0.8</v>
@@ -2539,13 +2539,13 @@
         <v>0.09</v>
       </c>
       <c r="BH5">
-        <v>1.1632</v>
+        <v>1.1633</v>
       </c>
       <c r="BI5" t="s">
         <v>157</v>
       </c>
       <c r="BJ5">
-        <v>1480</v>
+        <v>1491</v>
       </c>
       <c r="BK5" t="s">
         <v>59</v>
@@ -2554,28 +2554,28 @@
         <v>60</v>
       </c>
       <c r="BM5">
-        <v>78.3</v>
+        <v>78.8</v>
       </c>
       <c r="BN5">
-        <v>1.068</v>
+        <v>1.069</v>
       </c>
       <c r="BO5">
-        <v>80.3</v>
+        <v>80.8</v>
       </c>
       <c r="BP5">
-        <v>74.90000000000001</v>
+        <v>75.40000000000001</v>
       </c>
       <c r="BQ5">
+        <v>58.7</v>
+      </c>
+      <c r="BR5">
+        <v>56.6</v>
+      </c>
+      <c r="BS5">
         <v>58.6</v>
       </c>
-      <c r="BR5">
-        <v>56.7</v>
-      </c>
-      <c r="BS5">
-        <v>57.6</v>
-      </c>
       <c r="BT5">
-        <v>12</v>
+        <v>9.300000000000001</v>
       </c>
       <c r="BU5" t="s">
         <v>69</v>
@@ -2590,13 +2590,13 @@
         <v>82</v>
       </c>
       <c r="BY5">
-        <v>78.90000000000001</v>
+        <v>78.5</v>
       </c>
       <c r="BZ5">
         <v>10</v>
       </c>
       <c r="CA5">
-        <v>8</v>
+        <v>8.300000000000001</v>
       </c>
     </row>
   </sheetData>
@@ -2703,7 +2703,7 @@
         <v>65</v>
       </c>
       <c r="G2">
-        <v>90.5</v>
+        <v>93.40000000000001</v>
       </c>
       <c r="H2">
         <v>8</v>
@@ -2721,10 +2721,10 @@
         <v>67</v>
       </c>
       <c r="M2">
-        <v>84.2</v>
+        <v>83.90000000000001</v>
       </c>
       <c r="N2">
-        <v>1710</v>
+        <v>1684</v>
       </c>
       <c r="O2" t="s">
         <v>59</v>

</xml_diff>

<commit_message>
Update MLB weather 2026-07-14 10:44 PM PT
</commit_message>
<xml_diff>
--- a/mlb_weather_professional_v4_2026_07_14.xlsx
+++ b/mlb_weather_professional_v4_2026_07_14.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="400" uniqueCount="158">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="400" uniqueCount="153">
   <si>
     <t>Date</t>
   </si>
@@ -209,7 +209,7 @@
     <t>Clear</t>
   </si>
   <si>
-    <t>🟢 8.8 mph Out to RF</t>
+    <t>🟢 8.0 mph Out to RF</t>
   </si>
   <si>
     <t>SW</t>
@@ -221,7 +221,7 @@
     <t>B+</t>
   </si>
   <si>
-    <t>Density 79 | Wind 65 | Temp 62 | Altitude 62 | Confidence 93%</t>
+    <t>Density 74 | Wind 63 | Temp 58 | Altitude 60 | Confidence 92%</t>
   </si>
   <si>
     <t>🟢 Good</t>
@@ -233,7 +233,7 @@
     <t>LOW</t>
   </si>
   <si>
-    <t>2026-07-14 07:50:23 PM PDT</t>
+    <t>2026-07-14 10:44:03 PM PDT</t>
   </si>
   <si>
     <t>Period</t>
@@ -467,7 +467,7 @@
     <t>11:00 PM EDT</t>
   </si>
   <si>
-    <t>2026-07-15 02:50:23 UTC</t>
+    <t>2026-07-15 05:44:03 UTC</t>
   </si>
   <si>
     <t>2026-07-14T21:58:43+00:00</t>
@@ -476,22 +476,7 @@
     <t>YES</t>
   </si>
   <si>
-    <t>2026-07-14T19:00</t>
-  </si>
-  <si>
-    <t>2026-07-14T20:00</t>
-  </si>
-  <si>
-    <t>2026-07-14T21:00</t>
-  </si>
-  <si>
-    <t>2026-07-14T22:00</t>
-  </si>
-  <si>
-    <t>2026-07-14T23:00</t>
-  </si>
-  <si>
-    <t>LIGHT</t>
+    <t>2026-07-15T00:00</t>
   </si>
   <si>
     <t>NEUTRAL</t>
@@ -1179,28 +1164,28 @@
         <v>61</v>
       </c>
       <c r="K2">
-        <v>85.5</v>
+        <v>79.3</v>
       </c>
       <c r="L2">
-        <v>60.3</v>
+        <v>70.40000000000001</v>
       </c>
       <c r="M2" t="s">
         <v>62</v>
       </c>
       <c r="N2">
-        <v>9.4</v>
+        <v>8.6</v>
       </c>
       <c r="O2" t="s">
         <v>63</v>
       </c>
       <c r="P2">
-        <v>2.9</v>
+        <v>2.1</v>
       </c>
       <c r="Q2">
-        <v>7.6</v>
+        <v>6.6</v>
       </c>
       <c r="R2">
-        <v>8.800000000000001</v>
+        <v>8</v>
       </c>
       <c r="T2" t="s">
         <v>64</v>
@@ -1209,7 +1194,7 @@
         <v>0</v>
       </c>
       <c r="V2">
-        <v>62.7</v>
+        <v>60.9</v>
       </c>
       <c r="W2" t="s">
         <v>65</v>
@@ -1218,25 +1203,25 @@
         <v>66</v>
       </c>
       <c r="Y2">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="Z2">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="AA2">
-        <v>3.8</v>
+        <v>3.3</v>
       </c>
       <c r="AB2">
-        <v>93.40000000000001</v>
+        <v>91.59999999999999</v>
       </c>
       <c r="AC2" t="s">
         <v>67</v>
       </c>
       <c r="AD2">
-        <v>6.5</v>
+        <v>5.9</v>
       </c>
       <c r="AE2">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="AF2">
         <v>100</v>
@@ -1245,34 +1230,34 @@
         <v>0</v>
       </c>
       <c r="AH2">
-        <v>4.7</v>
+        <v>9.199999999999999</v>
       </c>
       <c r="AI2">
-        <v>0.5</v>
+        <v>0.6</v>
       </c>
       <c r="AJ2">
-        <v>1.1569</v>
+        <v>1.167</v>
       </c>
       <c r="AK2">
-        <v>1684</v>
+        <v>1384</v>
       </c>
       <c r="AL2">
-        <v>1012.2</v>
+        <v>1012</v>
       </c>
       <c r="AM2">
-        <v>69.3</v>
+        <v>68.2</v>
       </c>
       <c r="AN2">
-        <v>83.90000000000001</v>
+        <v>79.3</v>
       </c>
       <c r="AO2">
-        <v>62.5</v>
+        <v>70.40000000000001</v>
       </c>
       <c r="AP2" t="s">
         <v>68</v>
       </c>
       <c r="AQ2">
-        <v>17.3</v>
+        <v>12.3</v>
       </c>
       <c r="AR2">
         <v>0</v>
@@ -1284,19 +1269,19 @@
         <v>69</v>
       </c>
       <c r="AU2">
-        <v>12</v>
+        <v>8.4</v>
       </c>
       <c r="AV2" t="s">
         <v>69</v>
       </c>
       <c r="AW2">
-        <v>13.3</v>
+        <v>9.1</v>
       </c>
       <c r="AX2" t="s">
         <v>70</v>
       </c>
       <c r="AY2">
-        <v>291.7</v>
+        <v>465.3</v>
       </c>
       <c r="AZ2">
         <v>5</v>
@@ -1672,7 +1657,7 @@
         <v>149</v>
       </c>
       <c r="J2">
-        <v>291.7</v>
+        <v>465.3</v>
       </c>
       <c r="K2">
         <v>0</v>
@@ -1681,16 +1666,16 @@
         <v>5</v>
       </c>
       <c r="M2">
-        <v>0.44</v>
+        <v>1.16</v>
       </c>
       <c r="N2">
-        <v>0.58</v>
+        <v>0.95</v>
       </c>
       <c r="O2">
         <v>0</v>
       </c>
       <c r="P2">
-        <v>5.4</v>
+        <v>9.199999999999999</v>
       </c>
       <c r="Q2">
         <v>0.6</v>
@@ -1708,19 +1693,19 @@
         <v>151</v>
       </c>
       <c r="V2" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="W2">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="X2">
-        <v>3.5</v>
+        <v>7.5</v>
       </c>
       <c r="Y2">
-        <v>97.2</v>
+        <v>91.59999999999999</v>
       </c>
       <c r="Z2">
-        <v>82.90000000000001</v>
+        <v>75</v>
       </c>
       <c r="AA2">
         <v>0.98</v>
@@ -1738,25 +1723,25 @@
         <v>61</v>
       </c>
       <c r="AF2">
-        <v>85.5</v>
+        <v>79.3</v>
       </c>
       <c r="AG2">
-        <v>89.7</v>
+        <v>80.59999999999999</v>
       </c>
       <c r="AH2">
-        <v>69.90000000000001</v>
+        <v>68.2</v>
       </c>
       <c r="AI2">
-        <v>60.3</v>
+        <v>70.40000000000001</v>
       </c>
       <c r="AJ2">
-        <v>1012.4</v>
+        <v>1012</v>
       </c>
       <c r="AK2">
-        <v>1014.7</v>
+        <v>1014.2</v>
       </c>
       <c r="AL2">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="AM2">
         <v>0</v>
@@ -1765,46 +1750,46 @@
         <v>0</v>
       </c>
       <c r="AO2">
-        <v>54.6</v>
+        <v>42.4</v>
       </c>
       <c r="AP2">
-        <v>1688</v>
+        <v>835</v>
       </c>
       <c r="AQ2">
-        <v>9.4</v>
+        <v>8.6</v>
       </c>
       <c r="AR2">
-        <v>20.8</v>
+        <v>16.4</v>
       </c>
       <c r="AS2" t="s">
         <v>63</v>
       </c>
       <c r="AT2">
-        <v>224.8</v>
+        <v>229.3</v>
       </c>
       <c r="AU2">
-        <v>7.7</v>
+        <v>6.7</v>
       </c>
       <c r="AV2">
-        <v>3.3</v>
+        <v>2.4</v>
       </c>
       <c r="AW2">
-        <v>9.4</v>
+        <v>8.6</v>
       </c>
       <c r="AX2">
-        <v>7.6</v>
+        <v>6.6</v>
       </c>
       <c r="AY2">
-        <v>2.9</v>
+        <v>2.1</v>
       </c>
       <c r="AZ2">
-        <v>8.800000000000001</v>
+        <v>8</v>
       </c>
       <c r="BA2">
-        <v>5.2</v>
+        <v>5.3</v>
       </c>
       <c r="BB2">
-        <v>6.8</v>
+        <v>5.9</v>
       </c>
       <c r="BC2">
         <v>0.8</v>
@@ -1822,13 +1807,13 @@
         <v>0.09</v>
       </c>
       <c r="BH2">
-        <v>1.1536</v>
+        <v>1.167</v>
       </c>
       <c r="BI2" t="s">
-        <v>156</v>
+        <v>152</v>
       </c>
       <c r="BJ2">
-        <v>1779</v>
+        <v>1384</v>
       </c>
       <c r="BK2" t="s">
         <v>59</v>
@@ -1837,49 +1822,49 @@
         <v>60</v>
       </c>
       <c r="BM2">
-        <v>83.90000000000001</v>
+        <v>77.2</v>
       </c>
       <c r="BN2">
-        <v>1.081</v>
+        <v>1.065</v>
       </c>
       <c r="BO2">
-        <v>85.7</v>
+        <v>79.2</v>
       </c>
       <c r="BP2">
-        <v>80.40000000000001</v>
+        <v>73.8</v>
       </c>
       <c r="BQ2">
-        <v>60</v>
+        <v>58.2</v>
       </c>
       <c r="BR2">
-        <v>58.1</v>
+        <v>56.1</v>
       </c>
       <c r="BS2">
-        <v>48.9</v>
+        <v>60.8</v>
       </c>
       <c r="BT2">
-        <v>12</v>
+        <v>8.4</v>
       </c>
       <c r="BU2" t="s">
         <v>69</v>
       </c>
       <c r="BV2">
-        <v>2.2</v>
+        <v>9.1</v>
       </c>
       <c r="BW2" t="s">
         <v>69</v>
       </c>
       <c r="BX2">
-        <v>85</v>
+        <v>80</v>
       </c>
       <c r="BY2">
-        <v>84.7</v>
+        <v>77.59999999999999</v>
       </c>
       <c r="BZ2">
         <v>10</v>
       </c>
       <c r="CA2">
-        <v>9.199999999999999</v>
+        <v>7.9</v>
       </c>
     </row>
     <row r="3" spans="1:79">
@@ -1911,7 +1896,7 @@
         <v>149</v>
       </c>
       <c r="J3">
-        <v>291.7</v>
+        <v>465.3</v>
       </c>
       <c r="K3">
         <v>0</v>
@@ -1920,19 +1905,19 @@
         <v>5</v>
       </c>
       <c r="M3">
-        <v>0.68</v>
+        <v>1.16</v>
       </c>
       <c r="N3">
-        <v>1.02</v>
+        <v>0.95</v>
       </c>
       <c r="O3">
         <v>0</v>
       </c>
       <c r="P3">
-        <v>3.3</v>
+        <v>9.199999999999999</v>
       </c>
       <c r="Q3">
-        <v>0.5</v>
+        <v>0.6</v>
       </c>
       <c r="R3">
         <v>100</v>
@@ -1944,22 +1929,22 @@
         <v>150</v>
       </c>
       <c r="U3" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="V3" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
       <c r="W3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="X3">
-        <v>5.8</v>
+        <v>7.5</v>
       </c>
       <c r="Y3">
-        <v>92</v>
+        <v>91.59999999999999</v>
       </c>
       <c r="Z3">
-        <v>79.3</v>
+        <v>75</v>
       </c>
       <c r="AA3">
         <v>0.98</v>
@@ -1977,25 +1962,25 @@
         <v>61</v>
       </c>
       <c r="AF3">
-        <v>83.90000000000001</v>
+        <v>79.3</v>
       </c>
       <c r="AG3">
-        <v>86.09999999999999</v>
+        <v>80.59999999999999</v>
       </c>
       <c r="AH3">
-        <v>69.2</v>
+        <v>68.2</v>
       </c>
       <c r="AI3">
-        <v>62.3</v>
+        <v>70.40000000000001</v>
       </c>
       <c r="AJ3">
-        <v>1012.4</v>
+        <v>1012</v>
       </c>
       <c r="AK3">
-        <v>1014.7</v>
+        <v>1014.2</v>
       </c>
       <c r="AL3">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="AM3">
         <v>0</v>
@@ -2004,46 +1989,46 @@
         <v>0</v>
       </c>
       <c r="AO3">
-        <v>52</v>
+        <v>42.4</v>
       </c>
       <c r="AP3">
-        <v>1300</v>
+        <v>835</v>
       </c>
       <c r="AQ3">
-        <v>8.800000000000001</v>
+        <v>8.6</v>
       </c>
       <c r="AR3">
-        <v>21.7</v>
+        <v>16.4</v>
       </c>
       <c r="AS3" t="s">
         <v>63</v>
       </c>
       <c r="AT3">
-        <v>226.5</v>
+        <v>229.3</v>
       </c>
       <c r="AU3">
-        <v>7.1</v>
+        <v>6.7</v>
       </c>
       <c r="AV3">
-        <v>2.8</v>
+        <v>2.4</v>
       </c>
       <c r="AW3">
-        <v>8.800000000000001</v>
+        <v>8.6</v>
       </c>
       <c r="AX3">
-        <v>7</v>
+        <v>6.6</v>
       </c>
       <c r="AY3">
-        <v>2.5</v>
+        <v>2.1</v>
       </c>
       <c r="AZ3">
-        <v>8.199999999999999</v>
+        <v>8</v>
       </c>
       <c r="BA3">
-        <v>5.1</v>
+        <v>5.3</v>
       </c>
       <c r="BB3">
-        <v>6.2</v>
+        <v>5.9</v>
       </c>
       <c r="BC3">
         <v>0.8</v>
@@ -2061,13 +2046,13 @@
         <v>0.09</v>
       </c>
       <c r="BH3">
-        <v>1.1573</v>
+        <v>1.167</v>
       </c>
       <c r="BI3" t="s">
-        <v>156</v>
+        <v>152</v>
       </c>
       <c r="BJ3">
-        <v>1673</v>
+        <v>1384</v>
       </c>
       <c r="BK3" t="s">
         <v>59</v>
@@ -2076,49 +2061,49 @@
         <v>60</v>
       </c>
       <c r="BM3">
-        <v>81.90000000000001</v>
+        <v>77.2</v>
       </c>
       <c r="BN3">
-        <v>1.077</v>
+        <v>1.065</v>
       </c>
       <c r="BO3">
-        <v>83.7</v>
+        <v>79.2</v>
       </c>
       <c r="BP3">
-        <v>78.5</v>
+        <v>73.8</v>
       </c>
       <c r="BQ3">
-        <v>59.2</v>
+        <v>58.2</v>
       </c>
       <c r="BR3">
-        <v>57.4</v>
+        <v>56.1</v>
       </c>
       <c r="BS3">
-        <v>50.6</v>
+        <v>60.8</v>
       </c>
       <c r="BT3">
-        <v>12</v>
+        <v>8.4</v>
       </c>
       <c r="BU3" t="s">
         <v>69</v>
       </c>
       <c r="BV3">
-        <v>9.800000000000001</v>
+        <v>9.1</v>
       </c>
       <c r="BW3" t="s">
         <v>69</v>
       </c>
       <c r="BX3">
-        <v>85</v>
+        <v>80</v>
       </c>
       <c r="BY3">
-        <v>81.90000000000001</v>
+        <v>77.59999999999999</v>
       </c>
       <c r="BZ3">
         <v>10</v>
       </c>
       <c r="CA3">
-        <v>8.199999999999999</v>
+        <v>7.9</v>
       </c>
     </row>
     <row r="4" spans="1:79">
@@ -2150,7 +2135,7 @@
         <v>149</v>
       </c>
       <c r="J4">
-        <v>291.7</v>
+        <v>465.3</v>
       </c>
       <c r="K4">
         <v>0</v>
@@ -2159,19 +2144,19 @@
         <v>5</v>
       </c>
       <c r="M4">
-        <v>1.33</v>
+        <v>1.16</v>
       </c>
       <c r="N4">
-        <v>0.87</v>
+        <v>0.95</v>
       </c>
       <c r="O4">
         <v>0</v>
       </c>
       <c r="P4">
-        <v>4.6</v>
+        <v>9.199999999999999</v>
       </c>
       <c r="Q4">
-        <v>0.3</v>
+        <v>0.6</v>
       </c>
       <c r="R4">
         <v>100</v>
@@ -2183,22 +2168,22 @@
         <v>150</v>
       </c>
       <c r="U4" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
       <c r="V4" t="s">
-        <v>154</v>
+        <v>151</v>
       </c>
       <c r="W4">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="X4">
-        <v>7.9</v>
+        <v>7.5</v>
       </c>
       <c r="Y4">
-        <v>89.09999999999999</v>
+        <v>91.59999999999999</v>
       </c>
       <c r="Z4">
-        <v>77.2</v>
+        <v>75</v>
       </c>
       <c r="AA4">
         <v>0.98</v>
@@ -2216,25 +2201,25 @@
         <v>61</v>
       </c>
       <c r="AF4">
-        <v>82.5</v>
+        <v>79.3</v>
       </c>
       <c r="AG4">
-        <v>82</v>
+        <v>80.59999999999999</v>
       </c>
       <c r="AH4">
-        <v>68.7</v>
+        <v>68.2</v>
       </c>
       <c r="AI4">
-        <v>64.5</v>
+        <v>70.40000000000001</v>
       </c>
       <c r="AJ4">
-        <v>1011.7</v>
+        <v>1012</v>
       </c>
       <c r="AK4">
-        <v>1014</v>
+        <v>1014.2</v>
       </c>
       <c r="AL4">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="AM4">
         <v>0</v>
@@ -2243,46 +2228,46 @@
         <v>0</v>
       </c>
       <c r="AO4">
-        <v>45.3</v>
+        <v>42.4</v>
       </c>
       <c r="AP4">
-        <v>997</v>
+        <v>835</v>
       </c>
       <c r="AQ4">
-        <v>9.199999999999999</v>
+        <v>8.6</v>
       </c>
       <c r="AR4">
-        <v>17.8</v>
+        <v>16.4</v>
       </c>
       <c r="AS4" t="s">
         <v>63</v>
       </c>
       <c r="AT4">
-        <v>228.2</v>
+        <v>229.3</v>
       </c>
       <c r="AU4">
-        <v>7.2</v>
+        <v>6.7</v>
       </c>
       <c r="AV4">
-        <v>2.7</v>
+        <v>2.4</v>
       </c>
       <c r="AW4">
-        <v>9.1</v>
+        <v>8.6</v>
       </c>
       <c r="AX4">
-        <v>7.1</v>
+        <v>6.6</v>
       </c>
       <c r="AY4">
-        <v>2.4</v>
+        <v>2.1</v>
       </c>
       <c r="AZ4">
-        <v>8.5</v>
+        <v>8</v>
       </c>
       <c r="BA4">
-        <v>5.5</v>
+        <v>5.3</v>
       </c>
       <c r="BB4">
-        <v>6.3</v>
+        <v>5.9</v>
       </c>
       <c r="BC4">
         <v>0.8</v>
@@ -2300,13 +2285,13 @@
         <v>0.09</v>
       </c>
       <c r="BH4">
-        <v>1.1595</v>
+        <v>1.167</v>
       </c>
       <c r="BI4" t="s">
-        <v>156</v>
+        <v>152</v>
       </c>
       <c r="BJ4">
-        <v>1607</v>
+        <v>1384</v>
       </c>
       <c r="BK4" t="s">
         <v>59</v>
@@ -2315,49 +2300,49 @@
         <v>60</v>
       </c>
       <c r="BM4">
-        <v>80.5</v>
+        <v>77.2</v>
       </c>
       <c r="BN4">
-        <v>1.073</v>
+        <v>1.065</v>
       </c>
       <c r="BO4">
-        <v>82.5</v>
+        <v>79.2</v>
       </c>
       <c r="BP4">
-        <v>77</v>
+        <v>73.8</v>
       </c>
       <c r="BQ4">
-        <v>59.2</v>
+        <v>58.2</v>
       </c>
       <c r="BR4">
-        <v>57.1</v>
+        <v>56.1</v>
       </c>
       <c r="BS4">
-        <v>55.7</v>
+        <v>60.8</v>
       </c>
       <c r="BT4">
-        <v>10</v>
+        <v>8.4</v>
       </c>
       <c r="BU4" t="s">
         <v>69</v>
       </c>
       <c r="BV4">
-        <v>13.3</v>
+        <v>9.1</v>
       </c>
       <c r="BW4" t="s">
         <v>69</v>
       </c>
       <c r="BX4">
-        <v>85</v>
+        <v>80</v>
       </c>
       <c r="BY4">
-        <v>79.59999999999999</v>
+        <v>77.59999999999999</v>
       </c>
       <c r="BZ4">
         <v>10</v>
       </c>
       <c r="CA4">
-        <v>8.800000000000001</v>
+        <v>7.9</v>
       </c>
     </row>
     <row r="5" spans="1:79">
@@ -2389,10 +2374,10 @@
         <v>149</v>
       </c>
       <c r="J5">
-        <v>291.7</v>
+        <v>465.3</v>
       </c>
       <c r="K5">
-        <v>0.2</v>
+        <v>0</v>
       </c>
       <c r="L5">
         <v>5</v>
@@ -2401,16 +2386,16 @@
         <v>1.16</v>
       </c>
       <c r="N5">
-        <v>0.89</v>
+        <v>0.95</v>
       </c>
       <c r="O5">
         <v>0</v>
       </c>
       <c r="P5">
-        <v>6.6</v>
+        <v>9.199999999999999</v>
       </c>
       <c r="Q5">
-        <v>0.3</v>
+        <v>0.6</v>
       </c>
       <c r="R5">
         <v>100</v>
@@ -2422,22 +2407,22 @@
         <v>150</v>
       </c>
       <c r="U5" t="s">
-        <v>154</v>
+        <v>151</v>
       </c>
       <c r="V5" t="s">
-        <v>155</v>
+        <v>151</v>
       </c>
       <c r="W5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="X5">
-        <v>7.3</v>
+        <v>7.5</v>
       </c>
       <c r="Y5">
-        <v>91</v>
+        <v>91.59999999999999</v>
       </c>
       <c r="Z5">
-        <v>76.3</v>
+        <v>75</v>
       </c>
       <c r="AA5">
         <v>0.98</v>
@@ -2455,25 +2440,25 @@
         <v>61</v>
       </c>
       <c r="AF5">
-        <v>80.7</v>
+        <v>79.3</v>
       </c>
       <c r="AG5">
-        <v>81.59999999999999</v>
+        <v>80.59999999999999</v>
       </c>
       <c r="AH5">
-        <v>68.59999999999999</v>
+        <v>68.2</v>
       </c>
       <c r="AI5">
-        <v>68.3</v>
+        <v>70.40000000000001</v>
       </c>
       <c r="AJ5">
-        <v>1011.4</v>
+        <v>1012</v>
       </c>
       <c r="AK5">
-        <v>1013.7</v>
+        <v>1014.2</v>
       </c>
       <c r="AL5">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="AM5">
         <v>0</v>
@@ -2482,46 +2467,46 @@
         <v>0</v>
       </c>
       <c r="AO5">
-        <v>41.6</v>
+        <v>42.4</v>
       </c>
       <c r="AP5">
-        <v>933</v>
+        <v>835</v>
       </c>
       <c r="AQ5">
-        <v>8.9</v>
+        <v>8.6</v>
       </c>
       <c r="AR5">
-        <v>16.7</v>
+        <v>16.4</v>
       </c>
       <c r="AS5" t="s">
         <v>63</v>
       </c>
       <c r="AT5">
-        <v>228.2</v>
+        <v>229.3</v>
       </c>
       <c r="AU5">
-        <v>7</v>
+        <v>6.7</v>
       </c>
       <c r="AV5">
-        <v>2.6</v>
+        <v>2.4</v>
       </c>
       <c r="AW5">
-        <v>8.9</v>
+        <v>8.6</v>
       </c>
       <c r="AX5">
-        <v>6.9</v>
+        <v>6.6</v>
       </c>
       <c r="AY5">
-        <v>2.3</v>
+        <v>2.1</v>
       </c>
       <c r="AZ5">
-        <v>8.300000000000001</v>
+        <v>8</v>
       </c>
       <c r="BA5">
-        <v>5.4</v>
+        <v>5.3</v>
       </c>
       <c r="BB5">
-        <v>6.2</v>
+        <v>5.9</v>
       </c>
       <c r="BC5">
         <v>0.8</v>
@@ -2539,13 +2524,13 @@
         <v>0.09</v>
       </c>
       <c r="BH5">
-        <v>1.1633</v>
+        <v>1.167</v>
       </c>
       <c r="BI5" t="s">
-        <v>157</v>
+        <v>152</v>
       </c>
       <c r="BJ5">
-        <v>1491</v>
+        <v>1384</v>
       </c>
       <c r="BK5" t="s">
         <v>59</v>
@@ -2554,49 +2539,49 @@
         <v>60</v>
       </c>
       <c r="BM5">
-        <v>78.8</v>
+        <v>77.2</v>
       </c>
       <c r="BN5">
-        <v>1.069</v>
+        <v>1.065</v>
       </c>
       <c r="BO5">
-        <v>80.8</v>
+        <v>79.2</v>
       </c>
       <c r="BP5">
-        <v>75.40000000000001</v>
+        <v>73.8</v>
       </c>
       <c r="BQ5">
-        <v>58.7</v>
+        <v>58.2</v>
       </c>
       <c r="BR5">
-        <v>56.6</v>
+        <v>56.1</v>
       </c>
       <c r="BS5">
-        <v>58.6</v>
+        <v>60.8</v>
       </c>
       <c r="BT5">
-        <v>9.300000000000001</v>
+        <v>8.4</v>
       </c>
       <c r="BU5" t="s">
         <v>69</v>
       </c>
       <c r="BV5">
-        <v>10.3</v>
+        <v>9.1</v>
       </c>
       <c r="BW5" t="s">
         <v>69</v>
       </c>
       <c r="BX5">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="BY5">
-        <v>78.5</v>
+        <v>77.59999999999999</v>
       </c>
       <c r="BZ5">
         <v>10</v>
       </c>
       <c r="CA5">
-        <v>8.300000000000001</v>
+        <v>7.9</v>
       </c>
     </row>
   </sheetData>
@@ -2697,34 +2682,34 @@
         <v>58</v>
       </c>
       <c r="E2">
-        <v>62.7</v>
+        <v>60.9</v>
       </c>
       <c r="F2" t="s">
         <v>65</v>
       </c>
       <c r="G2">
-        <v>93.40000000000001</v>
+        <v>91.59999999999999</v>
       </c>
       <c r="H2">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="I2">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="J2">
-        <v>3.8</v>
+        <v>3.3</v>
       </c>
       <c r="K2">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="L2" t="s">
         <v>67</v>
       </c>
       <c r="M2">
-        <v>83.90000000000001</v>
+        <v>79.3</v>
       </c>
       <c r="N2">
-        <v>1684</v>
+        <v>1384</v>
       </c>
       <c r="O2" t="s">
         <v>59</v>

</xml_diff>